<commit_message>
fix: Pairing issue and Alignment losses issue in 764 clover v2
</commit_message>
<xml_diff>
--- a/metrix_calculation.xlsx
+++ b/metrix_calculation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course\CS_764\project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course\CS_764\project\NeurIPS2025-LEAR-main\csi764_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEFC3197-B7B1-4048-94E5-B93D67380420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933B75E9-1A7A-4969-822C-7D3C3F4D825A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="28">
   <si>
     <t>After Task</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -137,6 +138,10 @@
   </si>
   <si>
     <t>t = 33 task aware</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 33 t_Agnostic Claude version</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -311,6 +316,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -328,15 +342,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -618,7 +623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:J254"/>
+  <dimension ref="C3:T254"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="18.625" customWidth="1"/>
@@ -631,16 +636,16 @@
   <sheetData>
     <row r="3" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="11"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C5" s="2" t="s">
@@ -837,16 +842,16 @@
     </row>
     <row r="22" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="11"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="5"/>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C24" s="2" t="s">
@@ -1043,16 +1048,16 @@
     </row>
     <row r="38" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
-      <c r="I39" s="10"/>
-      <c r="J39" s="11"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="5"/>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C40" s="2" t="s">
@@ -1249,16 +1254,16 @@
     </row>
     <row r="54" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="10"/>
-      <c r="H55" s="10"/>
-      <c r="I55" s="10"/>
-      <c r="J55" s="11"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+      <c r="H55" s="4"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="5"/>
     </row>
     <row r="56" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C56" s="2" t="s">
@@ -1455,16 +1460,16 @@
     </row>
     <row r="69" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="70" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="9" t="s">
+      <c r="C70" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D70" s="10"/>
-      <c r="E70" s="10"/>
-      <c r="F70" s="10"/>
-      <c r="G70" s="10"/>
-      <c r="H70" s="10"/>
-      <c r="I70" s="10"/>
-      <c r="J70" s="11"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+      <c r="H70" s="4"/>
+      <c r="I70" s="4"/>
+      <c r="J70" s="5"/>
     </row>
     <row r="71" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C71" s="2" t="s">
@@ -1661,16 +1666,16 @@
     </row>
     <row r="85" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="86" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="9" t="s">
+      <c r="C86" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D86" s="10"/>
-      <c r="E86" s="10"/>
-      <c r="F86" s="10"/>
-      <c r="G86" s="10"/>
-      <c r="H86" s="10"/>
-      <c r="I86" s="10"/>
-      <c r="J86" s="11"/>
+      <c r="D86" s="4"/>
+      <c r="E86" s="4"/>
+      <c r="F86" s="4"/>
+      <c r="G86" s="4"/>
+      <c r="H86" s="4"/>
+      <c r="I86" s="4"/>
+      <c r="J86" s="5"/>
     </row>
     <row r="87" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C87" s="2" t="s">
@@ -1867,16 +1872,16 @@
     </row>
     <row r="106" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="107" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C107" s="9" t="s">
+      <c r="C107" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D107" s="10"/>
-      <c r="E107" s="10"/>
-      <c r="F107" s="10"/>
-      <c r="G107" s="10"/>
-      <c r="H107" s="10"/>
-      <c r="I107" s="10"/>
-      <c r="J107" s="11"/>
+      <c r="D107" s="4"/>
+      <c r="E107" s="4"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="4"/>
+      <c r="H107" s="4"/>
+      <c r="I107" s="4"/>
+      <c r="J107" s="5"/>
     </row>
     <row r="108" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C108" s="2" t="s">
@@ -2073,16 +2078,16 @@
     </row>
     <row r="122" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="123" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C123" s="9" t="s">
+      <c r="C123" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D123" s="10"/>
-      <c r="E123" s="10"/>
-      <c r="F123" s="10"/>
-      <c r="G123" s="10"/>
-      <c r="H123" s="10"/>
-      <c r="I123" s="10"/>
-      <c r="J123" s="11"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
+      <c r="G123" s="4"/>
+      <c r="H123" s="4"/>
+      <c r="I123" s="4"/>
+      <c r="J123" s="5"/>
     </row>
     <row r="124" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C124" s="2" t="s">
@@ -2279,16 +2284,16 @@
     </row>
     <row r="138" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="139" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C139" s="9" t="s">
+      <c r="C139" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D139" s="10"/>
-      <c r="E139" s="10"/>
-      <c r="F139" s="10"/>
-      <c r="G139" s="10"/>
-      <c r="H139" s="10"/>
-      <c r="I139" s="10"/>
-      <c r="J139" s="11"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="4"/>
+      <c r="F139" s="4"/>
+      <c r="G139" s="4"/>
+      <c r="H139" s="4"/>
+      <c r="I139" s="4"/>
+      <c r="J139" s="5"/>
     </row>
     <row r="140" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C140" s="2" t="s">
@@ -2485,16 +2490,16 @@
     </row>
     <row r="153" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="154" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C154" s="9" t="s">
+      <c r="C154" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D154" s="10"/>
-      <c r="E154" s="10"/>
-      <c r="F154" s="10"/>
-      <c r="G154" s="10"/>
-      <c r="H154" s="10"/>
-      <c r="I154" s="10"/>
-      <c r="J154" s="11"/>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4"/>
+      <c r="F154" s="4"/>
+      <c r="G154" s="4"/>
+      <c r="H154" s="4"/>
+      <c r="I154" s="4"/>
+      <c r="J154" s="5"/>
     </row>
     <row r="155" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C155" s="2" t="s">
@@ -2691,16 +2696,16 @@
     </row>
     <row r="168" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="169" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C169" s="9" t="s">
+      <c r="C169" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D169" s="10"/>
-      <c r="E169" s="10"/>
-      <c r="F169" s="10"/>
-      <c r="G169" s="10"/>
-      <c r="H169" s="10"/>
-      <c r="I169" s="10"/>
-      <c r="J169" s="11"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="4"/>
+      <c r="H169" s="4"/>
+      <c r="I169" s="4"/>
+      <c r="J169" s="5"/>
     </row>
     <row r="170" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C170" s="2" t="s">
@@ -2897,16 +2902,16 @@
     </row>
     <row r="183" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="184" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C184" s="9" t="s">
+      <c r="C184" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D184" s="10"/>
-      <c r="E184" s="10"/>
-      <c r="F184" s="10"/>
-      <c r="G184" s="10"/>
-      <c r="H184" s="10"/>
-      <c r="I184" s="10"/>
-      <c r="J184" s="11"/>
+      <c r="D184" s="4"/>
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
+      <c r="G184" s="4"/>
+      <c r="H184" s="4"/>
+      <c r="I184" s="4"/>
+      <c r="J184" s="5"/>
     </row>
     <row r="185" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C185" s="2" t="s">
@@ -3102,41 +3107,51 @@
     </row>
     <row r="202" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="203" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C203" s="3" t="s">
+      <c r="C203" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D203" s="4"/>
-      <c r="E203" s="4"/>
-      <c r="F203" s="4"/>
-      <c r="G203" s="4"/>
-      <c r="H203" s="4"/>
-      <c r="I203" s="4"/>
-      <c r="J203" s="5"/>
+      <c r="D203" s="7"/>
+      <c r="E203" s="7"/>
+      <c r="F203" s="7"/>
+      <c r="G203" s="7"/>
+      <c r="H203" s="7"/>
+      <c r="I203" s="7"/>
+      <c r="J203" s="8"/>
     </row>
     <row r="204" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C204" s="6"/>
-      <c r="D204" s="7"/>
-      <c r="E204" s="7"/>
-      <c r="F204" s="7"/>
-      <c r="G204" s="7"/>
-      <c r="H204" s="7"/>
-      <c r="I204" s="7"/>
-      <c r="J204" s="8"/>
+      <c r="C204" s="9"/>
+      <c r="D204" s="10"/>
+      <c r="E204" s="10"/>
+      <c r="F204" s="10"/>
+      <c r="G204" s="10"/>
+      <c r="H204" s="10"/>
+      <c r="I204" s="10"/>
+      <c r="J204" s="11"/>
     </row>
     <row r="208" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C209" s="9" t="s">
+    <row r="209" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C209" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D209" s="10"/>
-      <c r="E209" s="10"/>
-      <c r="F209" s="10"/>
-      <c r="G209" s="10"/>
-      <c r="H209" s="10"/>
-      <c r="I209" s="10"/>
-      <c r="J209" s="11"/>
-    </row>
-    <row r="210" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="D209" s="4"/>
+      <c r="E209" s="4"/>
+      <c r="F209" s="4"/>
+      <c r="G209" s="4"/>
+      <c r="H209" s="4"/>
+      <c r="I209" s="4"/>
+      <c r="J209" s="5"/>
+      <c r="M209" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="N209" s="4"/>
+      <c r="O209" s="4"/>
+      <c r="P209" s="4"/>
+      <c r="Q209" s="4"/>
+      <c r="R209" s="4"/>
+      <c r="S209" s="4"/>
+      <c r="T209" s="5"/>
+    </row>
+    <row r="210" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C210" s="2" t="s">
         <v>0</v>
       </c>
@@ -3161,8 +3176,32 @@
       <c r="J210" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="211" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M210" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="N210" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="O210" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="P210" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q210" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="R210" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="S210" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="T210" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="211" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C211" s="1" t="s">
         <v>1</v>
       </c>
@@ -3175,8 +3214,20 @@
       <c r="H211" s="1"/>
       <c r="I211" s="1"/>
       <c r="J211" s="1"/>
-    </row>
-    <row r="212" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M211" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N211" s="1">
+        <v>96.794871794871796</v>
+      </c>
+      <c r="O211" s="1"/>
+      <c r="P211" s="1"/>
+      <c r="Q211" s="1"/>
+      <c r="R211" s="1"/>
+      <c r="S211" s="1"/>
+      <c r="T211" s="1"/>
+    </row>
+    <row r="212" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C212" s="1" t="s">
         <v>2</v>
       </c>
@@ -3191,8 +3242,22 @@
       <c r="H212" s="1"/>
       <c r="I212" s="1"/>
       <c r="J212" s="1"/>
-    </row>
-    <row r="213" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M212" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N212" s="1">
+        <v>95.883413461538396</v>
+      </c>
+      <c r="O212" s="1">
+        <v>85.917467948717899</v>
+      </c>
+      <c r="P212" s="1"/>
+      <c r="Q212" s="1"/>
+      <c r="R212" s="1"/>
+      <c r="S212" s="1"/>
+      <c r="T212" s="1"/>
+    </row>
+    <row r="213" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C213" s="1" t="s">
         <v>3</v>
       </c>
@@ -3208,8 +3273,23 @@
       <c r="H213" s="1"/>
       <c r="I213" s="1"/>
       <c r="J213" s="1"/>
-    </row>
-    <row r="214" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M213" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N213" s="1">
+        <v>95.252403846153797</v>
+      </c>
+      <c r="O213" s="1">
+        <v>85.637019230769198</v>
+      </c>
+      <c r="P213" s="1">
+        <v>96.689723320158095</v>
+      </c>
+      <c r="R213" s="1"/>
+      <c r="S213" s="1"/>
+      <c r="T213" s="1"/>
+    </row>
+    <row r="214" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C214" s="1" t="s">
         <v>4</v>
       </c>
@@ -3228,8 +3308,26 @@
       <c r="H214" s="1"/>
       <c r="I214" s="1"/>
       <c r="J214" s="1"/>
-    </row>
-    <row r="215" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M214" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N214" s="1">
+        <v>94.340945512820497</v>
+      </c>
+      <c r="O214" s="1">
+        <v>83.954326923076906</v>
+      </c>
+      <c r="P214" s="1">
+        <v>95.615118577075094</v>
+      </c>
+      <c r="Q214" s="1">
+        <v>79.328208556149704</v>
+      </c>
+      <c r="R214" s="1"/>
+      <c r="S214" s="1"/>
+      <c r="T214" s="1"/>
+    </row>
+    <row r="215" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C215" s="1" t="s">
         <v>5</v>
       </c>
@@ -3250,8 +3348,28 @@
       </c>
       <c r="I215" s="1"/>
       <c r="J215" s="1"/>
-    </row>
-    <row r="216" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M215" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N215" s="1">
+        <v>94.491185897435898</v>
+      </c>
+      <c r="O215" s="1">
+        <v>83.092948717948701</v>
+      </c>
+      <c r="P215">
+        <v>94.503458498023704</v>
+      </c>
+      <c r="Q215" s="1">
+        <v>76.353609625668398</v>
+      </c>
+      <c r="R215" s="1">
+        <v>85.226362179487097</v>
+      </c>
+      <c r="S215" s="1"/>
+      <c r="T215" s="1"/>
+    </row>
+    <row r="216" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C216" s="1" t="s">
         <v>6</v>
       </c>
@@ -3274,8 +3392,30 @@
         <v>92.346938775510196</v>
       </c>
       <c r="J216" s="1"/>
-    </row>
-    <row r="217" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M216" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N216" s="1">
+        <v>93.459535256410206</v>
+      </c>
+      <c r="O216" s="1">
+        <v>81.951121794871796</v>
+      </c>
+      <c r="P216" s="1">
+        <v>92.243083003952506</v>
+      </c>
+      <c r="Q216" s="1">
+        <v>75.150401069518693</v>
+      </c>
+      <c r="R216" s="1">
+        <v>84.685496794871796</v>
+      </c>
+      <c r="S216" s="1">
+        <v>90.784438775510196</v>
+      </c>
+      <c r="T216" s="1"/>
+    </row>
+    <row r="217" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C217" s="1" t="s">
         <v>7</v>
       </c>
@@ -3300,8 +3440,32 @@
       <c r="J217" s="1">
         <v>49.4791666666666</v>
       </c>
-    </row>
-    <row r="219" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M217" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N217" s="1">
+        <v>94.080528846153797</v>
+      </c>
+      <c r="O217" s="1">
+        <v>82.171474358974294</v>
+      </c>
+      <c r="P217" s="1">
+        <v>91.983695652173907</v>
+      </c>
+      <c r="Q217" s="1">
+        <v>75.250668449197804</v>
+      </c>
+      <c r="R217" s="1">
+        <v>84.715544871794805</v>
+      </c>
+      <c r="S217" s="1">
+        <v>90.832270408163197</v>
+      </c>
+      <c r="T217" s="1">
+        <v>58.6805555555555</v>
+      </c>
+    </row>
+    <row r="219" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C219" t="s">
         <v>8</v>
       </c>
@@ -3309,8 +3473,15 @@
         <f>AVERAGE(D217:J217)</f>
         <v>80.72086876165568</v>
       </c>
-    </row>
-    <row r="220" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M219" t="s">
+        <v>8</v>
+      </c>
+      <c r="N219">
+        <f>AVERAGE(N217:T217)</f>
+        <v>82.530676877430466</v>
+      </c>
+    </row>
+    <row r="220" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C220" t="s">
         <v>9</v>
       </c>
@@ -3318,8 +3489,15 @@
         <f>(SUM((D217-D211)+(E217-E212)+(F217-F213)+(G217-G214)+(H217-H215)+(I217-I216)))/6</f>
         <v>-2.5438816609293013</v>
       </c>
-    </row>
-    <row r="221" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M220" t="s">
+        <v>9</v>
+      </c>
+      <c r="N220">
+        <f>(SUM((N217-N211)+(O217-O212)+(P217-P213)+(Q217-Q214)+(R217-R215)+(S217-S216)))/6</f>
+        <v>-2.6178149980728307</v>
+      </c>
+    </row>
+    <row r="221" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C221" t="s">
         <v>10</v>
       </c>
@@ -3327,19 +3505,26 @@
         <f>SUM((MAX(D211:D217)-D217)+(MAX(E212:E217)-E217)+(MAX(F213:F217)-F217)+(MAX(G214:G217)-G217)+(MAX(H215:H217)-H217)+(MAX(I216:I217)-I217))/6</f>
         <v>2.5438816609293013</v>
       </c>
+      <c r="M221" t="s">
+        <v>10</v>
+      </c>
+      <c r="N221">
+        <f>SUM((MAX(N211:N217)-N217)+(MAX(O212:O217)-O217)+(MAX(P213:P217)-P217)+(MAX(Q214:Q217)-Q217)+(MAX(R215:R217)-R217)+(MAX(S216:S217)-S217))/6</f>
+        <v>2.6257869368483306</v>
+      </c>
     </row>
     <row r="225" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="226" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C226" s="9" t="s">
+      <c r="C226" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D226" s="10"/>
-      <c r="E226" s="10"/>
-      <c r="F226" s="10"/>
-      <c r="G226" s="10"/>
-      <c r="H226" s="10"/>
-      <c r="I226" s="10"/>
-      <c r="J226" s="11"/>
+      <c r="D226" s="4"/>
+      <c r="E226" s="4"/>
+      <c r="F226" s="4"/>
+      <c r="G226" s="4"/>
+      <c r="H226" s="4"/>
+      <c r="I226" s="4"/>
+      <c r="J226" s="5"/>
     </row>
     <row r="227" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C227" s="2" t="s">
@@ -3535,16 +3720,16 @@
     </row>
     <row r="241" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="242" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C242" s="9" t="s">
+      <c r="C242" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D242" s="10"/>
-      <c r="E242" s="10"/>
-      <c r="F242" s="10"/>
-      <c r="G242" s="10"/>
-      <c r="H242" s="10"/>
-      <c r="I242" s="10"/>
-      <c r="J242" s="11"/>
+      <c r="D242" s="4"/>
+      <c r="E242" s="4"/>
+      <c r="F242" s="4"/>
+      <c r="G242" s="4"/>
+      <c r="H242" s="4"/>
+      <c r="I242" s="4"/>
+      <c r="J242" s="5"/>
     </row>
     <row r="243" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C243" s="2" t="s">
@@ -3739,23 +3924,24 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
+    <mergeCell ref="M209:T209"/>
+    <mergeCell ref="C203:J204"/>
+    <mergeCell ref="C209:J209"/>
+    <mergeCell ref="C226:J226"/>
+    <mergeCell ref="C242:J242"/>
+    <mergeCell ref="C184:J184"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="C39:J39"/>
+    <mergeCell ref="C55:J55"/>
+    <mergeCell ref="C70:J70"/>
     <mergeCell ref="C169:J169"/>
     <mergeCell ref="C86:J86"/>
     <mergeCell ref="C107:J107"/>
     <mergeCell ref="C123:J123"/>
     <mergeCell ref="C139:J139"/>
     <mergeCell ref="C154:J154"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="C23:J23"/>
-    <mergeCell ref="C39:J39"/>
-    <mergeCell ref="C55:J55"/>
-    <mergeCell ref="C70:J70"/>
-    <mergeCell ref="C203:J204"/>
-    <mergeCell ref="C209:J209"/>
-    <mergeCell ref="C226:J226"/>
-    <mergeCell ref="C242:J242"/>
-    <mergeCell ref="C184:J184"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update: new data record
</commit_message>
<xml_diff>
--- a/metrix_calculation.xlsx
+++ b/metrix_calculation.xlsx
@@ -5,18 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course\CS_764\project\NeurIPS2025-LEAR-main\csi764_project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course\CS_764\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933B75E9-1A7A-4969-822C-7D3C3F4D825A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49CECC17-9C04-49EB-9417-7B59243D3325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="41">
   <si>
     <t>After Task</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -142,6 +141,65 @@
   </si>
   <si>
     <t>t = 33 t_Agnostic Claude version</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>original Claude Version comparsion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 33 task aware Claude</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 20 t_aware claude</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 25 t_aware claude</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 30 t_aware claude</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 35 t_aware claude</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 40 t_aware claude</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 45 t_aware claude</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[DEBUG] Task 7 -&gt; Expert 7
+[DEBUG] Task-expert mapping: [1, 2, 3, 4, 5, 6, 7]
+[DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>42.70833333333333]</t>
+  </si>
+  <si>
+    <t>[DEBUG] Task 7 -&gt; Expert 2
+[DEBUG] Task-expert mapping: [1, 1, 1, 2, 1, 2, 2]
+[DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[DEBUG] Task 7 -&gt; Expert 1
+[DEBUG] Task-expert mapping: [1, 1, 1, 1, 1, 1, 1]
+[DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[DEBUG] Task 7 -&gt; Expert 2
+[DEBUG] Task-expert mapping: [1, 1, 1, 2, 3, 4, 2]
+[DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -312,10 +370,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -623,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:T254"/>
+  <dimension ref="C3:T362"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="18.625" customWidth="1"/>
@@ -636,16 +700,16 @@
   <sheetData>
     <row r="3" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="5"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="7"/>
     </row>
     <row r="5" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C5" s="2" t="s">
@@ -842,16 +906,16 @@
     </row>
     <row r="22" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="5"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="7"/>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C24" s="2" t="s">
@@ -1048,16 +1112,16 @@
     </row>
     <row r="38" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="5"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="7"/>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C40" s="2" t="s">
@@ -1254,16 +1318,16 @@
     </row>
     <row r="54" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="5"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="7"/>
     </row>
     <row r="56" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C56" s="2" t="s">
@@ -1460,16 +1524,16 @@
     </row>
     <row r="69" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="70" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
-      <c r="J70" s="5"/>
+      <c r="D70" s="6"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6"/>
+      <c r="H70" s="6"/>
+      <c r="I70" s="6"/>
+      <c r="J70" s="7"/>
     </row>
     <row r="71" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C71" s="2" t="s">
@@ -1666,16 +1730,16 @@
     </row>
     <row r="85" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="86" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="3" t="s">
+      <c r="C86" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D86" s="4"/>
-      <c r="E86" s="4"/>
-      <c r="F86" s="4"/>
-      <c r="G86" s="4"/>
-      <c r="H86" s="4"/>
-      <c r="I86" s="4"/>
-      <c r="J86" s="5"/>
+      <c r="D86" s="6"/>
+      <c r="E86" s="6"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="6"/>
+      <c r="H86" s="6"/>
+      <c r="I86" s="6"/>
+      <c r="J86" s="7"/>
     </row>
     <row r="87" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C87" s="2" t="s">
@@ -1872,16 +1936,16 @@
     </row>
     <row r="106" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="107" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C107" s="3" t="s">
+      <c r="C107" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D107" s="4"/>
-      <c r="E107" s="4"/>
-      <c r="F107" s="4"/>
-      <c r="G107" s="4"/>
-      <c r="H107" s="4"/>
-      <c r="I107" s="4"/>
-      <c r="J107" s="5"/>
+      <c r="D107" s="6"/>
+      <c r="E107" s="6"/>
+      <c r="F107" s="6"/>
+      <c r="G107" s="6"/>
+      <c r="H107" s="6"/>
+      <c r="I107" s="6"/>
+      <c r="J107" s="7"/>
     </row>
     <row r="108" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C108" s="2" t="s">
@@ -2078,16 +2142,16 @@
     </row>
     <row r="122" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="123" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C123" s="3" t="s">
+      <c r="C123" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D123" s="4"/>
-      <c r="E123" s="4"/>
-      <c r="F123" s="4"/>
-      <c r="G123" s="4"/>
-      <c r="H123" s="4"/>
-      <c r="I123" s="4"/>
-      <c r="J123" s="5"/>
+      <c r="D123" s="6"/>
+      <c r="E123" s="6"/>
+      <c r="F123" s="6"/>
+      <c r="G123" s="6"/>
+      <c r="H123" s="6"/>
+      <c r="I123" s="6"/>
+      <c r="J123" s="7"/>
     </row>
     <row r="124" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C124" s="2" t="s">
@@ -2284,16 +2348,16 @@
     </row>
     <row r="138" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="139" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C139" s="3" t="s">
+      <c r="C139" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D139" s="4"/>
-      <c r="E139" s="4"/>
-      <c r="F139" s="4"/>
-      <c r="G139" s="4"/>
-      <c r="H139" s="4"/>
-      <c r="I139" s="4"/>
-      <c r="J139" s="5"/>
+      <c r="D139" s="6"/>
+      <c r="E139" s="6"/>
+      <c r="F139" s="6"/>
+      <c r="G139" s="6"/>
+      <c r="H139" s="6"/>
+      <c r="I139" s="6"/>
+      <c r="J139" s="7"/>
     </row>
     <row r="140" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C140" s="2" t="s">
@@ -2490,16 +2554,16 @@
     </row>
     <row r="153" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="154" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C154" s="3" t="s">
+      <c r="C154" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D154" s="4"/>
-      <c r="E154" s="4"/>
-      <c r="F154" s="4"/>
-      <c r="G154" s="4"/>
-      <c r="H154" s="4"/>
-      <c r="I154" s="4"/>
-      <c r="J154" s="5"/>
+      <c r="D154" s="6"/>
+      <c r="E154" s="6"/>
+      <c r="F154" s="6"/>
+      <c r="G154" s="6"/>
+      <c r="H154" s="6"/>
+      <c r="I154" s="6"/>
+      <c r="J154" s="7"/>
     </row>
     <row r="155" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C155" s="2" t="s">
@@ -2696,16 +2760,16 @@
     </row>
     <row r="168" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="169" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C169" s="3" t="s">
+      <c r="C169" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D169" s="4"/>
-      <c r="E169" s="4"/>
-      <c r="F169" s="4"/>
-      <c r="G169" s="4"/>
-      <c r="H169" s="4"/>
-      <c r="I169" s="4"/>
-      <c r="J169" s="5"/>
+      <c r="D169" s="6"/>
+      <c r="E169" s="6"/>
+      <c r="F169" s="6"/>
+      <c r="G169" s="6"/>
+      <c r="H169" s="6"/>
+      <c r="I169" s="6"/>
+      <c r="J169" s="7"/>
     </row>
     <row r="170" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C170" s="2" t="s">
@@ -2902,16 +2966,16 @@
     </row>
     <row r="183" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="184" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C184" s="3" t="s">
+      <c r="C184" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D184" s="4"/>
-      <c r="E184" s="4"/>
-      <c r="F184" s="4"/>
-      <c r="G184" s="4"/>
-      <c r="H184" s="4"/>
-      <c r="I184" s="4"/>
-      <c r="J184" s="5"/>
+      <c r="D184" s="6"/>
+      <c r="E184" s="6"/>
+      <c r="F184" s="6"/>
+      <c r="G184" s="6"/>
+      <c r="H184" s="6"/>
+      <c r="I184" s="6"/>
+      <c r="J184" s="7"/>
     </row>
     <row r="185" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C185" s="2" t="s">
@@ -3107,49 +3171,49 @@
     </row>
     <row r="202" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="203" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C203" s="6" t="s">
+      <c r="C203" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D203" s="7"/>
-      <c r="E203" s="7"/>
-      <c r="F203" s="7"/>
-      <c r="G203" s="7"/>
-      <c r="H203" s="7"/>
-      <c r="I203" s="7"/>
-      <c r="J203" s="8"/>
+      <c r="D203" s="9"/>
+      <c r="E203" s="9"/>
+      <c r="F203" s="9"/>
+      <c r="G203" s="9"/>
+      <c r="H203" s="9"/>
+      <c r="I203" s="9"/>
+      <c r="J203" s="10"/>
     </row>
     <row r="204" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C204" s="9"/>
-      <c r="D204" s="10"/>
-      <c r="E204" s="10"/>
-      <c r="F204" s="10"/>
-      <c r="G204" s="10"/>
-      <c r="H204" s="10"/>
-      <c r="I204" s="10"/>
-      <c r="J204" s="11"/>
+      <c r="C204" s="11"/>
+      <c r="D204" s="12"/>
+      <c r="E204" s="12"/>
+      <c r="F204" s="12"/>
+      <c r="G204" s="12"/>
+      <c r="H204" s="12"/>
+      <c r="I204" s="12"/>
+      <c r="J204" s="13"/>
     </row>
     <row r="208" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="209" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C209" s="3" t="s">
+      <c r="C209" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D209" s="4"/>
-      <c r="E209" s="4"/>
-      <c r="F209" s="4"/>
-      <c r="G209" s="4"/>
-      <c r="H209" s="4"/>
-      <c r="I209" s="4"/>
-      <c r="J209" s="5"/>
-      <c r="M209" s="3" t="s">
+      <c r="D209" s="6"/>
+      <c r="E209" s="6"/>
+      <c r="F209" s="6"/>
+      <c r="G209" s="6"/>
+      <c r="H209" s="6"/>
+      <c r="I209" s="6"/>
+      <c r="J209" s="7"/>
+      <c r="M209" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="N209" s="4"/>
-      <c r="O209" s="4"/>
-      <c r="P209" s="4"/>
-      <c r="Q209" s="4"/>
-      <c r="R209" s="4"/>
-      <c r="S209" s="4"/>
-      <c r="T209" s="5"/>
+      <c r="N209" s="6"/>
+      <c r="O209" s="6"/>
+      <c r="P209" s="6"/>
+      <c r="Q209" s="6"/>
+      <c r="R209" s="6"/>
+      <c r="S209" s="6"/>
+      <c r="T209" s="7"/>
     </row>
     <row r="210" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C210" s="2" t="s">
@@ -3513,20 +3577,30 @@
         <v>2.6257869368483306</v>
       </c>
     </row>
-    <row r="225" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C226" s="3" t="s">
+    <row r="225" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C226" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D226" s="4"/>
-      <c r="E226" s="4"/>
-      <c r="F226" s="4"/>
-      <c r="G226" s="4"/>
-      <c r="H226" s="4"/>
-      <c r="I226" s="4"/>
-      <c r="J226" s="5"/>
-    </row>
-    <row r="227" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="D226" s="6"/>
+      <c r="E226" s="6"/>
+      <c r="F226" s="6"/>
+      <c r="G226" s="6"/>
+      <c r="H226" s="6"/>
+      <c r="I226" s="6"/>
+      <c r="J226" s="7"/>
+      <c r="M226" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N226" s="6"/>
+      <c r="O226" s="6"/>
+      <c r="P226" s="6"/>
+      <c r="Q226" s="6"/>
+      <c r="R226" s="6"/>
+      <c r="S226" s="6"/>
+      <c r="T226" s="7"/>
+    </row>
+    <row r="227" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C227" s="2" t="s">
         <v>0</v>
       </c>
@@ -3551,8 +3625,32 @@
       <c r="J227" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="228" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M227" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="N227" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="O227" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="P227" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q227" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="R227" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="S227" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="T227" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="228" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C228" s="1" t="s">
         <v>1</v>
       </c>
@@ -3565,8 +3663,20 @@
       <c r="H228" s="1"/>
       <c r="I228" s="1"/>
       <c r="J228" s="1"/>
-    </row>
-    <row r="229" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M228" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N228" s="1">
+        <v>97.115384615384599</v>
+      </c>
+      <c r="O228" s="1"/>
+      <c r="P228" s="1"/>
+      <c r="Q228" s="1"/>
+      <c r="R228" s="1"/>
+      <c r="S228" s="1"/>
+      <c r="T228" s="1"/>
+    </row>
+    <row r="229" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C229" s="1" t="s">
         <v>2</v>
       </c>
@@ -3581,8 +3691,22 @@
       <c r="H229" s="1"/>
       <c r="I229" s="1"/>
       <c r="J229" s="1"/>
-    </row>
-    <row r="230" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M229" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N229" s="1">
+        <v>96.394230769230703</v>
+      </c>
+      <c r="O229" s="1">
+        <v>85.917467948717899</v>
+      </c>
+      <c r="P229" s="1"/>
+      <c r="Q229" s="1"/>
+      <c r="R229" s="1"/>
+      <c r="S229" s="1"/>
+      <c r="T229" s="1"/>
+    </row>
+    <row r="230" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C230" s="1" t="s">
         <v>3</v>
       </c>
@@ -3598,8 +3722,23 @@
       <c r="H230" s="1"/>
       <c r="I230" s="1"/>
       <c r="J230" s="1"/>
-    </row>
-    <row r="231" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M230" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N230" s="1">
+        <v>95.633012820512803</v>
+      </c>
+      <c r="O230" s="1">
+        <v>85.506810897435898</v>
+      </c>
+      <c r="P230" s="1">
+        <v>95.825098814229193</v>
+      </c>
+      <c r="R230" s="1"/>
+      <c r="S230" s="1"/>
+      <c r="T230" s="1"/>
+    </row>
+    <row r="231" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C231" s="1" t="s">
         <v>4</v>
       </c>
@@ -3618,8 +3757,26 @@
       <c r="H231" s="1"/>
       <c r="I231" s="1"/>
       <c r="J231" s="1"/>
-    </row>
-    <row r="232" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M231" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N231" s="1">
+        <v>94.991987179487097</v>
+      </c>
+      <c r="O231" s="1">
+        <v>83.173076923076906</v>
+      </c>
+      <c r="P231" s="1">
+        <v>94.503458498023704</v>
+      </c>
+      <c r="Q231" s="1">
+        <v>79.261363636363598</v>
+      </c>
+      <c r="R231" s="1"/>
+      <c r="S231" s="1"/>
+      <c r="T231" s="1"/>
+    </row>
+    <row r="232" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C232" s="1" t="s">
         <v>5</v>
       </c>
@@ -3640,8 +3797,28 @@
       </c>
       <c r="I232" s="1"/>
       <c r="J232" s="1"/>
-    </row>
-    <row r="233" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M232" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N232" s="1">
+        <v>95.172275641025607</v>
+      </c>
+      <c r="O232" s="1">
+        <v>83.143028846153797</v>
+      </c>
+      <c r="P232">
+        <v>94.330533596837896</v>
+      </c>
+      <c r="Q232" s="1">
+        <v>75.768716577540104</v>
+      </c>
+      <c r="R232" s="1">
+        <v>84.985977564102498</v>
+      </c>
+      <c r="S232" s="1"/>
+      <c r="T232" s="1"/>
+    </row>
+    <row r="233" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C233" s="1" t="s">
         <v>6</v>
       </c>
@@ -3664,8 +3841,30 @@
         <v>91.390306122448905</v>
       </c>
       <c r="J233" s="1"/>
-    </row>
-    <row r="234" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M233" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N233" s="1">
+        <v>94.370993589743506</v>
+      </c>
+      <c r="O233" s="1">
+        <v>82.231570512820497</v>
+      </c>
+      <c r="P233" s="1">
+        <v>94.071146245059296</v>
+      </c>
+      <c r="Q233" s="1">
+        <v>74.899732620320805</v>
+      </c>
+      <c r="R233" s="1">
+        <v>84.495192307692307</v>
+      </c>
+      <c r="S233" s="1">
+        <v>92.346938775510196</v>
+      </c>
+      <c r="T233" s="1"/>
+    </row>
+    <row r="234" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C234" s="1" t="s">
         <v>7</v>
       </c>
@@ -3690,8 +3889,32 @@
       <c r="J234" s="1">
         <v>42.7083333333333</v>
       </c>
-    </row>
-    <row r="236" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M234" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N234" s="1">
+        <v>94.521233974358907</v>
+      </c>
+      <c r="O234" s="1">
+        <v>82.321714743589695</v>
+      </c>
+      <c r="P234" s="1">
+        <v>94.429347826086897</v>
+      </c>
+      <c r="Q234" s="1">
+        <v>74.933155080213893</v>
+      </c>
+      <c r="R234" s="1">
+        <v>84.354967948717899</v>
+      </c>
+      <c r="S234" s="1">
+        <v>92.362882653061206</v>
+      </c>
+      <c r="T234" s="1">
+        <v>48.0902777777777</v>
+      </c>
+    </row>
+    <row r="236" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C236" t="s">
         <v>8</v>
       </c>
@@ -3699,8 +3922,15 @@
         <f>AVERAGE(D234:J234)</f>
         <v>79.842739588179839</v>
       </c>
-    </row>
-    <row r="237" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M236" t="s">
+        <v>8</v>
+      </c>
+      <c r="N236">
+        <f>AVERAGE(N234:T234)</f>
+        <v>81.57336857197231</v>
+      </c>
+    </row>
+    <row r="237" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C237" t="s">
         <v>9</v>
       </c>
@@ -3708,8 +3938,15 @@
         <f>(SUM((D234-D228)+(E234-E229)+(F234-F230)+(G234-G231)+(H234-H232)+(I234-I233)))/6</f>
         <v>-2.4709734326359531</v>
       </c>
-    </row>
-    <row r="238" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M237" t="s">
+        <v>9</v>
+      </c>
+      <c r="N237">
+        <f>(SUM((N234-N228)+(O234-O229)+(P234-P230)+(Q234-Q231)+(R234-R232)+(S234-S233)))/6</f>
+        <v>-2.0881548547132476</v>
+      </c>
+    </row>
+    <row r="238" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C238" t="s">
         <v>10</v>
       </c>
@@ -3717,21 +3954,38 @@
         <f>SUM((MAX(D228:D234)-D234)+(MAX(E229:E234)-E234)+(MAX(F230:F234)-F234)+(MAX(G231:G234)-G234)+(MAX(H232:H234)-H234)+(MAX(I233:I234)-I234))/6</f>
         <v>2.4709734326359531</v>
       </c>
-    </row>
-    <row r="241" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C242" s="3" t="s">
+      <c r="M238" t="s">
+        <v>10</v>
+      </c>
+      <c r="N238">
+        <f>SUM((MAX(N228:N234)-N234)+(MAX(O229:O234)-O234)+(MAX(P230:P234)-P234)+(MAX(Q231:Q234)-Q234)+(MAX(R232:R234)-R234)+(MAX(S233:S234)-S234))/6</f>
+        <v>2.0908121676384162</v>
+      </c>
+    </row>
+    <row r="241" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C242" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D242" s="4"/>
-      <c r="E242" s="4"/>
-      <c r="F242" s="4"/>
-      <c r="G242" s="4"/>
-      <c r="H242" s="4"/>
-      <c r="I242" s="4"/>
-      <c r="J242" s="5"/>
-    </row>
-    <row r="243" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="D242" s="6"/>
+      <c r="E242" s="6"/>
+      <c r="F242" s="6"/>
+      <c r="G242" s="6"/>
+      <c r="H242" s="6"/>
+      <c r="I242" s="6"/>
+      <c r="J242" s="7"/>
+      <c r="M242" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N242" s="6"/>
+      <c r="O242" s="6"/>
+      <c r="P242" s="6"/>
+      <c r="Q242" s="6"/>
+      <c r="R242" s="6"/>
+      <c r="S242" s="6"/>
+      <c r="T242" s="7"/>
+    </row>
+    <row r="243" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C243" s="2" t="s">
         <v>0</v>
       </c>
@@ -3756,8 +4010,32 @@
       <c r="J243" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="244" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M243" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="N243" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="O243" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="P243" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q243" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="R243" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="S243" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="T243" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="244" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C244" s="1" t="s">
         <v>1</v>
       </c>
@@ -3770,8 +4048,20 @@
       <c r="H244" s="1"/>
       <c r="I244" s="1"/>
       <c r="J244" s="1"/>
-    </row>
-    <row r="245" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M244" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N244" s="1">
+        <v>97.095352564102498</v>
+      </c>
+      <c r="O244" s="1"/>
+      <c r="P244" s="1"/>
+      <c r="Q244" s="1"/>
+      <c r="R244" s="1"/>
+      <c r="S244" s="1"/>
+      <c r="T244" s="1"/>
+    </row>
+    <row r="245" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C245" s="1" t="s">
         <v>2</v>
       </c>
@@ -3786,8 +4076,22 @@
       <c r="H245" s="1"/>
       <c r="I245" s="1"/>
       <c r="J245" s="1"/>
-    </row>
-    <row r="246" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M245" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N245" s="1">
+        <v>96.664663461538396</v>
+      </c>
+      <c r="O245" s="1">
+        <v>85.707131410256395</v>
+      </c>
+      <c r="P245" s="1"/>
+      <c r="Q245" s="1"/>
+      <c r="R245" s="1"/>
+      <c r="S245" s="1"/>
+      <c r="T245" s="1"/>
+    </row>
+    <row r="246" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C246" s="1" t="s">
         <v>3</v>
       </c>
@@ -3803,8 +4107,23 @@
       <c r="H246" s="1"/>
       <c r="I246" s="1"/>
       <c r="J246" s="1"/>
-    </row>
-    <row r="247" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M246" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N246" s="1">
+        <v>96.264022435897402</v>
+      </c>
+      <c r="O246" s="1">
+        <v>85.216346153846104</v>
+      </c>
+      <c r="P246" s="1">
+        <v>96.245059288537504</v>
+      </c>
+      <c r="R246" s="1"/>
+      <c r="S246" s="1"/>
+      <c r="T246" s="1"/>
+    </row>
+    <row r="247" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C247" s="1" t="s">
         <v>4</v>
       </c>
@@ -3823,8 +4142,26 @@
       <c r="H247" s="1"/>
       <c r="I247" s="1"/>
       <c r="J247" s="1"/>
-    </row>
-    <row r="248" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M247" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N247" s="1">
+        <v>95.092147435897402</v>
+      </c>
+      <c r="O247">
+        <v>83.183092948717899</v>
+      </c>
+      <c r="P247" s="1">
+        <v>96.208003952569101</v>
+      </c>
+      <c r="Q247" s="1">
+        <v>78.542780748663105</v>
+      </c>
+      <c r="R247" s="1"/>
+      <c r="S247" s="1"/>
+      <c r="T247" s="1"/>
+    </row>
+    <row r="248" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C248" s="1" t="s">
         <v>5</v>
       </c>
@@ -3845,8 +4182,28 @@
       </c>
       <c r="I248" s="1"/>
       <c r="J248" s="1"/>
-    </row>
-    <row r="249" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M248" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N248" s="1">
+        <v>95.092147435897402</v>
+      </c>
+      <c r="O248" s="1">
+        <v>83.193108974358907</v>
+      </c>
+      <c r="P248">
+        <v>95.281620553359602</v>
+      </c>
+      <c r="Q248" s="1">
+        <v>75.300802139037401</v>
+      </c>
+      <c r="R248" s="1">
+        <v>85.476762820512803</v>
+      </c>
+      <c r="S248" s="1"/>
+      <c r="T248" s="1"/>
+    </row>
+    <row r="249" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C249" s="1" t="s">
         <v>6</v>
       </c>
@@ -3869,8 +4226,30 @@
         <v>92.267219387755105</v>
       </c>
       <c r="J249" s="1"/>
-    </row>
-    <row r="250" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M249" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N249" s="1">
+        <v>94.561298076922995</v>
+      </c>
+      <c r="O249" s="1">
+        <v>82.281650641025607</v>
+      </c>
+      <c r="P249" s="1">
+        <v>94.157608695652101</v>
+      </c>
+      <c r="Q249" s="1">
+        <v>74.030748663101605</v>
+      </c>
+      <c r="R249" s="1">
+        <v>84.765625</v>
+      </c>
+      <c r="S249" s="1">
+        <v>92.171556122448905</v>
+      </c>
+      <c r="T249" s="1"/>
+    </row>
+    <row r="250" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C250" s="1" t="s">
         <v>7</v>
       </c>
@@ -3895,8 +4274,32 @@
       <c r="J250" s="1">
         <v>50.3472222222222</v>
       </c>
-    </row>
-    <row r="252" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M250" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N250" s="1">
+        <v>94.641426282051199</v>
+      </c>
+      <c r="O250" s="1">
+        <v>82.421875</v>
+      </c>
+      <c r="P250" s="1">
+        <v>94.034090909090907</v>
+      </c>
+      <c r="Q250" s="1">
+        <v>74.916443850267299</v>
+      </c>
+      <c r="R250" s="1">
+        <v>84.985977564102498</v>
+      </c>
+      <c r="S250" s="1">
+        <v>91.868622448979593</v>
+      </c>
+      <c r="T250" s="1">
+        <v>60.9375</v>
+      </c>
+    </row>
+    <row r="252" spans="3:20" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C252" t="s">
         <v>8</v>
       </c>
@@ -3904,8 +4307,22 @@
         <f>AVERAGE(D250:J250)</f>
         <v>81.121108752847562</v>
       </c>
-    </row>
-    <row r="253" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M252" t="s">
+        <v>8</v>
+      </c>
+      <c r="N252">
+        <f>AVERAGE(N250:T250)</f>
+        <v>83.400848007784504</v>
+      </c>
+      <c r="P252" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q252" s="3"/>
+      <c r="R252" s="3"/>
+      <c r="S252" s="3"/>
+      <c r="T252" s="3"/>
+    </row>
+    <row r="253" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C253" t="s">
         <v>9</v>
       </c>
@@ -3913,8 +4330,20 @@
         <f>(SUM((D250-D244)+(E250-E245)+(F250-F246)+(G250-G247)+(H250-H248)+(I250-I249)))/6</f>
         <v>-2.0039063879834038</v>
       </c>
-    </row>
-    <row r="254" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="M253" t="s">
+        <v>9</v>
+      </c>
+      <c r="N253">
+        <f>(SUM((N250-N244)+(O250-O245)+(P250-P246)+(Q250-Q247)+(R250-R248)+(S250-S249)))/6</f>
+        <v>-2.0617011500049522</v>
+      </c>
+      <c r="P253" s="3"/>
+      <c r="Q253" s="3"/>
+      <c r="R253" s="3"/>
+      <c r="S253" s="3"/>
+      <c r="T253" s="3"/>
+    </row>
+    <row r="254" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C254" t="s">
         <v>10</v>
       </c>
@@ -3922,26 +4351,1376 @@
         <f>SUM((MAX(D244:D250)-D250)+(MAX(E245:E250)-E250)+(MAX(F246:F250)-F250)+(MAX(G247:G250)-G250)+(MAX(H248:H250)-H250)+(MAX(I249:I250)-I250))/6</f>
         <v>2.0039063879834038</v>
       </c>
+      <c r="M254" t="s">
+        <v>10</v>
+      </c>
+      <c r="N254">
+        <f>SUM((MAX(N244:N250)-N250)+(MAX(O245:O250)-O250)+(MAX(P246:P250)-P250)+(MAX(Q247:Q250)-Q250)+(MAX(R248:R250)-R250)+(MAX(S249:S250)-S250))/6</f>
+        <v>2.0617011500049522</v>
+      </c>
+      <c r="P254" s="3"/>
+      <c r="Q254" s="3"/>
+      <c r="R254" s="3"/>
+      <c r="S254" s="3"/>
+      <c r="T254" s="3"/>
+    </row>
+    <row r="255" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="P255" s="3"/>
+      <c r="Q255" s="3"/>
+      <c r="R255" s="3"/>
+      <c r="S255" s="3"/>
+      <c r="T255" s="3"/>
+    </row>
+    <row r="267" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="268" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C268" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D268" s="6"/>
+      <c r="E268" s="6"/>
+      <c r="F268" s="6"/>
+      <c r="G268" s="6"/>
+      <c r="H268" s="6"/>
+      <c r="I268" s="6"/>
+      <c r="J268" s="7"/>
+    </row>
+    <row r="269" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C269" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D269" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E269" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F269" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G269" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H269" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I269" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J269" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="270" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C270" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D270" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="E270" s="1"/>
+      <c r="F270" s="1"/>
+      <c r="G270" s="1"/>
+      <c r="H270" s="1"/>
+      <c r="I270" s="1"/>
+      <c r="J270" s="1"/>
+    </row>
+    <row r="271" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C271" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D271" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="E271" s="1">
+        <v>77.0833333333333</v>
+      </c>
+      <c r="F271" s="1"/>
+      <c r="G271" s="1"/>
+      <c r="H271" s="1"/>
+      <c r="I271" s="1"/>
+      <c r="J271" s="1"/>
+    </row>
+    <row r="272" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C272" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D272" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E272" s="1">
+        <v>78.125</v>
+      </c>
+      <c r="F272" s="1">
+        <v>96.875</v>
+      </c>
+      <c r="G272" s="1"/>
+      <c r="H272" s="1"/>
+      <c r="I272" s="1"/>
+      <c r="J272" s="1"/>
+    </row>
+    <row r="273" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C273" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D273" s="1">
+        <v>88.5416666666666</v>
+      </c>
+      <c r="E273" s="1">
+        <v>78.125</v>
+      </c>
+      <c r="F273" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="G273" s="1">
+        <v>51.0416666666666</v>
+      </c>
+      <c r="H273" s="1"/>
+      <c r="I273" s="1"/>
+      <c r="J273" s="1"/>
+    </row>
+    <row r="274" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C274" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D274" s="1">
+        <v>90.625</v>
+      </c>
+      <c r="E274" s="1">
+        <v>77.0833333333333</v>
+      </c>
+      <c r="F274" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="G274" s="1">
+        <v>53.125</v>
+      </c>
+      <c r="H274" s="1">
+        <v>65.625</v>
+      </c>
+      <c r="I274" s="1"/>
+      <c r="J274" s="1"/>
+    </row>
+    <row r="275" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C275" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D275" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E275" s="1">
+        <v>76.0416666666666</v>
+      </c>
+      <c r="F275" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="G275" s="1">
+        <v>53.125</v>
+      </c>
+      <c r="H275" s="1">
+        <v>63.5416666666666</v>
+      </c>
+      <c r="I275" s="1">
+        <v>76.0416666666666</v>
+      </c>
+      <c r="J275" s="1"/>
+    </row>
+    <row r="276" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C276" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D276" s="1">
+        <v>88.5416666666666</v>
+      </c>
+      <c r="E276" s="1">
+        <v>80.2083333333333</v>
+      </c>
+      <c r="F276" s="1">
+        <v>94.7916666666666</v>
+      </c>
+      <c r="G276" s="1">
+        <v>48.9583333333333</v>
+      </c>
+      <c r="H276" s="1">
+        <v>68.75</v>
+      </c>
+      <c r="I276" s="1">
+        <v>78.125</v>
+      </c>
+      <c r="J276" s="1">
+        <v>58.3333333333333</v>
+      </c>
+    </row>
+    <row r="278" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C278" t="s">
+        <v>8</v>
+      </c>
+      <c r="D278">
+        <f>AVERAGE(D276:J276)</f>
+        <v>73.9583333333333</v>
+      </c>
+      <c r="F278" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G278" s="4"/>
+      <c r="H278" s="4"/>
+      <c r="I278" s="4"/>
+    </row>
+    <row r="279" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C279" t="s">
+        <v>9</v>
+      </c>
+      <c r="D279">
+        <f>(SUM((D276-D270)+(E276-E271)+(F276-F272)+(G276-G273)+(H276-H274)+(I276-I275)))/6</f>
+        <v>-0.17361111111111663</v>
+      </c>
+      <c r="F279" s="4"/>
+      <c r="G279" s="4"/>
+      <c r="H279" s="4"/>
+      <c r="I279" s="4"/>
+    </row>
+    <row r="280" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C280" t="s">
+        <v>10</v>
+      </c>
+      <c r="D280">
+        <f>SUM((MAX(D270:D276)-D276)+(MAX(E271:E276)-E276)+(MAX(F272:F276)-F276)+(MAX(G273:G276)-G276)+(MAX(H274:H276)-H276)+(MAX(I275:I276)-I276))/6</f>
+        <v>1.9097222222222499</v>
+      </c>
+      <c r="F280" s="4"/>
+      <c r="G280" s="4"/>
+      <c r="H280" s="4"/>
+      <c r="I280" s="4"/>
+    </row>
+    <row r="286" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="287" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C287" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D287" s="6"/>
+      <c r="E287" s="6"/>
+      <c r="F287" s="6"/>
+      <c r="G287" s="6"/>
+      <c r="H287" s="6"/>
+      <c r="I287" s="6"/>
+      <c r="J287" s="7"/>
+    </row>
+    <row r="288" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C288" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D288" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E288" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F288" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G288" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H288" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I288" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J288" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="289" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C289" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D289" s="1">
+        <v>94.7916666666666</v>
+      </c>
+      <c r="E289" s="1"/>
+      <c r="F289" s="1"/>
+      <c r="G289" s="1"/>
+      <c r="H289" s="1"/>
+      <c r="I289" s="1"/>
+      <c r="J289" s="1"/>
+    </row>
+    <row r="290" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C290" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D290" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E290" s="1">
+        <v>83.3333333333333</v>
+      </c>
+      <c r="F290" s="1"/>
+      <c r="G290" s="1"/>
+      <c r="H290" s="1"/>
+      <c r="I290" s="1"/>
+      <c r="J290" s="1"/>
+    </row>
+    <row r="291" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C291" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D291" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E291" s="1">
+        <v>82.2916666666666</v>
+      </c>
+      <c r="F291" s="1">
+        <v>56.25</v>
+      </c>
+      <c r="G291" s="1"/>
+      <c r="H291" s="1"/>
+      <c r="I291" s="1"/>
+      <c r="J291" s="1"/>
+    </row>
+    <row r="292" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C292" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D292" s="1">
+        <v>88.5416666666666</v>
+      </c>
+      <c r="E292" s="1">
+        <v>83.3333333333333</v>
+      </c>
+      <c r="F292" s="1">
+        <v>54.1666666666666</v>
+      </c>
+      <c r="G292" s="1">
+        <v>48.9583333333333</v>
+      </c>
+      <c r="H292" s="1"/>
+      <c r="I292" s="1"/>
+      <c r="J292" s="1"/>
+    </row>
+    <row r="293" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C293" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D293" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="E293" s="1">
+        <v>86.4583333333333</v>
+      </c>
+      <c r="F293" s="1">
+        <v>58.3333333333333</v>
+      </c>
+      <c r="G293" s="1">
+        <v>48.9583333333333</v>
+      </c>
+      <c r="H293" s="1">
+        <v>62.5</v>
+      </c>
+      <c r="I293" s="1"/>
+      <c r="J293" s="1"/>
+    </row>
+    <row r="294" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C294" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D294" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E294" s="1">
+        <v>84.375</v>
+      </c>
+      <c r="F294" s="1">
+        <v>64.5833333333333</v>
+      </c>
+      <c r="G294" s="1">
+        <v>50</v>
+      </c>
+      <c r="H294" s="1">
+        <v>64.5833333333333</v>
+      </c>
+      <c r="I294" s="1">
+        <v>79.1666666666666</v>
+      </c>
+      <c r="J294" s="1"/>
+    </row>
+    <row r="295" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C295" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D295" s="1">
+        <v>90.625</v>
+      </c>
+      <c r="E295" s="1">
+        <v>82.2916666666666</v>
+      </c>
+      <c r="F295" s="1">
+        <v>62.5</v>
+      </c>
+      <c r="G295" s="1">
+        <v>44.7916666666666</v>
+      </c>
+      <c r="H295" s="1">
+        <v>57.2916666666666</v>
+      </c>
+      <c r="I295" s="1">
+        <v>70.8333333333333</v>
+      </c>
+      <c r="J295" s="1">
+        <v>43.75</v>
+      </c>
+    </row>
+    <row r="297" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C297" t="s">
+        <v>8</v>
+      </c>
+      <c r="D297">
+        <f>AVERAGE(D295:J295)</f>
+        <v>64.5833333333333</v>
+      </c>
+      <c r="F297" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G297" s="4"/>
+      <c r="H297" s="4"/>
+      <c r="I297" s="4"/>
+    </row>
+    <row r="298" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C298" t="s">
+        <v>9</v>
+      </c>
+      <c r="D298">
+        <f>(SUM((D295-D289)+(E295-E290)+(F295-F291)+(G295-G292)+(H295-H293)+(I295-I294)))/6</f>
+        <v>-2.7777777777777835</v>
+      </c>
+      <c r="F298" s="4"/>
+      <c r="G298" s="4"/>
+      <c r="H298" s="4"/>
+      <c r="I298" s="4"/>
+    </row>
+    <row r="299" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C299" t="s">
+        <v>10</v>
+      </c>
+      <c r="D299">
+        <f>SUM((MAX(D289:D295)-D295)+(MAX(E290:E295)-E295)+(MAX(F291:F295)-F295)+(MAX(G292:G295)-G295)+(MAX(H293:H295)-H295)+(MAX(I294:I295)-I295))/6</f>
+        <v>5.208333333333333</v>
+      </c>
+      <c r="F299" s="4"/>
+      <c r="G299" s="4"/>
+      <c r="H299" s="4"/>
+      <c r="I299" s="4"/>
+    </row>
+    <row r="302" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="303" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C303" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D303" s="6"/>
+      <c r="E303" s="6"/>
+      <c r="F303" s="6"/>
+      <c r="G303" s="6"/>
+      <c r="H303" s="6"/>
+      <c r="I303" s="6"/>
+      <c r="J303" s="7"/>
+    </row>
+    <row r="304" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C304" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D304" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E304" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F304" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G304" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H304" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I304" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J304" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="305" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C305" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D305" s="1">
+        <v>88.5416666666666</v>
+      </c>
+      <c r="E305" s="1"/>
+      <c r="F305" s="1"/>
+      <c r="G305" s="1"/>
+      <c r="H305" s="1"/>
+      <c r="I305" s="1"/>
+      <c r="J305" s="1"/>
+    </row>
+    <row r="306" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C306" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D306" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="E306" s="1">
+        <v>75</v>
+      </c>
+      <c r="F306" s="1"/>
+      <c r="G306" s="1"/>
+      <c r="H306" s="1"/>
+      <c r="I306" s="1"/>
+      <c r="J306" s="1"/>
+    </row>
+    <row r="307" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C307" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D307" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="E307" s="1">
+        <v>75</v>
+      </c>
+      <c r="F307" s="1">
+        <v>90.625</v>
+      </c>
+      <c r="G307" s="1"/>
+      <c r="H307" s="1"/>
+      <c r="I307" s="1"/>
+      <c r="J307" s="1"/>
+    </row>
+    <row r="308" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C308" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D308" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="E308" s="1">
+        <v>79.1666666666666</v>
+      </c>
+      <c r="F308" s="1">
+        <v>90.625</v>
+      </c>
+      <c r="G308" s="1">
+        <v>48.9583333333333</v>
+      </c>
+      <c r="H308" s="1"/>
+      <c r="I308" s="1"/>
+      <c r="J308" s="1"/>
+    </row>
+    <row r="309" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C309" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D309" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="E309" s="1">
+        <v>80.2083333333333</v>
+      </c>
+      <c r="F309" s="1">
+        <v>86.4583333333333</v>
+      </c>
+      <c r="G309" s="1">
+        <v>52.0833333333333</v>
+      </c>
+      <c r="H309" s="1">
+        <v>87.5</v>
+      </c>
+      <c r="I309" s="1"/>
+      <c r="J309" s="1"/>
+    </row>
+    <row r="310" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C310" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D310" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="E310" s="1">
+        <v>78.125</v>
+      </c>
+      <c r="F310" s="1">
+        <v>83.3333333333333</v>
+      </c>
+      <c r="G310" s="1">
+        <v>48.9583333333333</v>
+      </c>
+      <c r="H310" s="1">
+        <v>85.4166666666666</v>
+      </c>
+      <c r="I310" s="1">
+        <v>77.0833333333333</v>
+      </c>
+      <c r="J310" s="1"/>
+    </row>
+    <row r="311" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C311" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D311" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="E311" s="1">
+        <v>77.0833333333333</v>
+      </c>
+      <c r="F311" s="1">
+        <v>94.7916666666666</v>
+      </c>
+      <c r="G311" s="1">
+        <v>44.7916666666666</v>
+      </c>
+      <c r="H311" s="1">
+        <v>90.625</v>
+      </c>
+      <c r="I311" s="1">
+        <v>72.9166666666666</v>
+      </c>
+      <c r="J311" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="313" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C313" t="s">
+        <v>8</v>
+      </c>
+      <c r="D313">
+        <f>AVERAGE(D311:J311)</f>
+        <v>78.298611111111072</v>
+      </c>
+      <c r="F313" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G313" s="4"/>
+      <c r="H313" s="4"/>
+      <c r="I313" s="4"/>
+    </row>
+    <row r="314" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C314" t="s">
+        <v>9</v>
+      </c>
+      <c r="D314">
+        <f>(SUM((D311-D305)+(E311-E306)+(F311-F307)+(G311-G308)+(H311-H309)+(I311-I310)))/6</f>
+        <v>0.34722222222220012</v>
+      </c>
+      <c r="F314" s="4"/>
+      <c r="G314" s="4"/>
+      <c r="H314" s="4"/>
+      <c r="I314" s="4"/>
+    </row>
+    <row r="315" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C315" t="s">
+        <v>10</v>
+      </c>
+      <c r="D315">
+        <f>SUM((MAX(D305:D311)-D311)+(MAX(E306:E311)-E311)+(MAX(F307:F311)-F311)+(MAX(G308:G311)-G311)+(MAX(H309:H311)-H311)+(MAX(I310:I311)-I311))/6</f>
+        <v>2.4305555555555665</v>
+      </c>
+      <c r="F315" s="4"/>
+      <c r="G315" s="4"/>
+      <c r="H315" s="4"/>
+      <c r="I315" s="4"/>
+    </row>
+    <row r="318" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="319" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C319" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D319" s="6"/>
+      <c r="E319" s="6"/>
+      <c r="F319" s="6"/>
+      <c r="G319" s="6"/>
+      <c r="H319" s="6"/>
+      <c r="I319" s="6"/>
+      <c r="J319" s="7"/>
+    </row>
+    <row r="320" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C320" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D320" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E320" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F320" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G320" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H320" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I320" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J320" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="321" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C321" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D321" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E321" s="1"/>
+      <c r="F321" s="1"/>
+      <c r="G321" s="1"/>
+      <c r="H321" s="1"/>
+      <c r="I321" s="1"/>
+      <c r="J321" s="1"/>
+    </row>
+    <row r="322" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C322" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D322" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E322" s="1">
+        <v>84.375</v>
+      </c>
+      <c r="F322" s="1"/>
+      <c r="G322" s="1"/>
+      <c r="H322" s="1"/>
+      <c r="I322" s="1"/>
+      <c r="J322" s="1"/>
+    </row>
+    <row r="323" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C323" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D323" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="E323" s="1">
+        <v>86.4583333333333</v>
+      </c>
+      <c r="F323" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="G323" s="1"/>
+      <c r="H323" s="1"/>
+      <c r="I323" s="1"/>
+      <c r="J323" s="1"/>
+    </row>
+    <row r="324" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C324" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D324" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E324" s="1">
+        <v>85.4166666666666</v>
+      </c>
+      <c r="F324" s="1">
+        <v>90.625</v>
+      </c>
+      <c r="G324" s="1">
+        <v>50</v>
+      </c>
+      <c r="H324" s="1"/>
+      <c r="I324" s="1"/>
+      <c r="J324" s="1"/>
+    </row>
+    <row r="325" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C325" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D325" s="1">
+        <v>92.7083333333333</v>
+      </c>
+      <c r="E325" s="1">
+        <v>86.4583333333333</v>
+      </c>
+      <c r="F325" s="1">
+        <v>86.4583333333333</v>
+      </c>
+      <c r="G325" s="1">
+        <v>51.0416666666666</v>
+      </c>
+      <c r="H325" s="1">
+        <v>83.3333333333333</v>
+      </c>
+      <c r="I325" s="1"/>
+      <c r="J325" s="1"/>
+    </row>
+    <row r="326" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C326" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D326" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="E326" s="1">
+        <v>84.375</v>
+      </c>
+      <c r="F326" s="1">
+        <v>89.5833333333333</v>
+      </c>
+      <c r="G326" s="1">
+        <v>50</v>
+      </c>
+      <c r="H326" s="1">
+        <v>83.3333333333333</v>
+      </c>
+      <c r="I326" s="1">
+        <v>80.2083333333333</v>
+      </c>
+      <c r="J326" s="1"/>
+    </row>
+    <row r="327" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C327" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D327" s="1">
+        <v>92.7083333333333</v>
+      </c>
+      <c r="E327" s="1">
+        <v>81.25</v>
+      </c>
+      <c r="F327" s="1">
+        <v>88.5416666666666</v>
+      </c>
+      <c r="G327" s="1">
+        <v>47.9166666666666</v>
+      </c>
+      <c r="H327" s="1">
+        <v>85.4166666666666</v>
+      </c>
+      <c r="I327" s="1">
+        <v>77.0833333333333</v>
+      </c>
+      <c r="J327" s="1">
+        <v>42.7083333333333</v>
+      </c>
+    </row>
+    <row r="329" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C329" t="s">
+        <v>8</v>
+      </c>
+      <c r="D329">
+        <f>AVERAGE(D327:J327)</f>
+        <v>73.660714285714249</v>
+      </c>
+      <c r="F329" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G329" s="4"/>
+      <c r="H329" s="4"/>
+      <c r="I329" s="4"/>
+    </row>
+    <row r="330" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C330" t="s">
+        <v>9</v>
+      </c>
+      <c r="D330">
+        <f>(SUM((D327-D321)+(E327-E322)+(F327-F323)+(G327-G324)+(H327-H325)+(I327-I326)))/6</f>
+        <v>-1.3888888888888999</v>
+      </c>
+      <c r="F330" s="4"/>
+      <c r="G330" s="4"/>
+      <c r="H330" s="4"/>
+      <c r="I330" s="4"/>
+    </row>
+    <row r="331" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C331" t="s">
+        <v>10</v>
+      </c>
+      <c r="D331">
+        <f>SUM((MAX(D321:D327)-D327)+(MAX(E322:E327)-E327)+(MAX(F323:F327)-F327)+(MAX(G324:G327)-G327)+(MAX(H325:H327)-H327)+(MAX(I326:I327)-I327))/6</f>
+        <v>2.6041666666666665</v>
+      </c>
+      <c r="F331" s="4"/>
+      <c r="G331" s="4"/>
+      <c r="H331" s="4"/>
+      <c r="I331" s="4"/>
+    </row>
+    <row r="333" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="334" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C334" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D334" s="6"/>
+      <c r="E334" s="6"/>
+      <c r="F334" s="6"/>
+      <c r="G334" s="6"/>
+      <c r="H334" s="6"/>
+      <c r="I334" s="6"/>
+      <c r="J334" s="7"/>
+    </row>
+    <row r="335" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C335" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D335" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E335" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F335" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G335" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H335" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I335" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J335" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="336" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C336" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D336" s="1">
+        <v>92.7083333333333</v>
+      </c>
+      <c r="E336" s="1"/>
+      <c r="F336" s="1"/>
+      <c r="G336" s="1"/>
+      <c r="H336" s="1"/>
+      <c r="I336" s="1"/>
+      <c r="J336" s="1"/>
+    </row>
+    <row r="337" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C337" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D337" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E337" s="1">
+        <v>76.0416666666666</v>
+      </c>
+      <c r="F337" s="1"/>
+      <c r="G337" s="1"/>
+      <c r="H337" s="1"/>
+      <c r="I337" s="1"/>
+      <c r="J337" s="1"/>
+    </row>
+    <row r="338" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C338" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D338" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E338" s="1">
+        <v>77.0833333333333</v>
+      </c>
+      <c r="F338" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="G338" s="1"/>
+      <c r="H338" s="1"/>
+      <c r="I338" s="1"/>
+      <c r="J338" s="1"/>
+    </row>
+    <row r="339" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C339" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D339" s="1">
+        <v>90.625</v>
+      </c>
+      <c r="E339" s="1">
+        <v>78.125</v>
+      </c>
+      <c r="F339" s="1">
+        <v>92.7083333333333</v>
+      </c>
+      <c r="G339" s="1">
+        <v>48.9583333333333</v>
+      </c>
+      <c r="H339" s="1"/>
+      <c r="I339" s="1"/>
+      <c r="J339" s="1"/>
+    </row>
+    <row r="340" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C340" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D340" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E340" s="1">
+        <v>81.25</v>
+      </c>
+      <c r="F340" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="G340" s="1">
+        <v>47.9166666666666</v>
+      </c>
+      <c r="H340" s="1">
+        <v>65.625</v>
+      </c>
+      <c r="I340" s="1"/>
+      <c r="J340" s="1"/>
+    </row>
+    <row r="341" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C341" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D341" s="1">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="E341" s="1">
+        <v>81.25</v>
+      </c>
+      <c r="F341" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="G341" s="1">
+        <v>46.875</v>
+      </c>
+      <c r="H341" s="1">
+        <v>65.625</v>
+      </c>
+      <c r="I341" s="1">
+        <v>77.0833333333333</v>
+      </c>
+      <c r="J341" s="1"/>
+    </row>
+    <row r="342" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C342" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D342" s="1">
+        <v>90.625</v>
+      </c>
+      <c r="E342" s="1">
+        <v>81.25</v>
+      </c>
+      <c r="F342" s="1">
+        <v>95.8333333333333</v>
+      </c>
+      <c r="G342" s="1">
+        <v>42.7083333333333</v>
+      </c>
+      <c r="H342" s="1">
+        <v>67.7083333333333</v>
+      </c>
+      <c r="I342" s="1">
+        <v>69.7916666666666</v>
+      </c>
+      <c r="J342" s="1">
+        <v>53.125</v>
+      </c>
+    </row>
+    <row r="344" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C344" t="s">
+        <v>8</v>
+      </c>
+      <c r="D344">
+        <f>AVERAGE(D342:J342)</f>
+        <v>71.577380952380935</v>
+      </c>
+      <c r="F344" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G344" s="4"/>
+      <c r="H344" s="4"/>
+      <c r="I344" s="4"/>
+    </row>
+    <row r="345" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C345" t="s">
+        <v>9</v>
+      </c>
+      <c r="D345">
+        <f>(SUM((D342-D336)+(E342-E337)+(F342-F338)+(G342-G339)+(H342-H340)+(I342-I341)))/6</f>
+        <v>-1.0416666666666667</v>
+      </c>
+      <c r="F345" s="4"/>
+      <c r="G345" s="4"/>
+      <c r="H345" s="4"/>
+      <c r="I345" s="4"/>
+    </row>
+    <row r="346" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C346" t="s">
+        <v>10</v>
+      </c>
+      <c r="D346">
+        <f>SUM((MAX(D336:D342)-D342)+(MAX(E337:E342)-E342)+(MAX(F338:F342)-F342)+(MAX(G339:G342)-G342)+(MAX(H340:H342)-H342)+(MAX(I341:I342)-I342))/6</f>
+        <v>2.6041666666666665</v>
+      </c>
+      <c r="F346" s="4"/>
+      <c r="G346" s="4"/>
+      <c r="H346" s="4"/>
+      <c r="I346" s="4"/>
+    </row>
+    <row r="349" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="350" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C350" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D350" s="6"/>
+      <c r="E350" s="6"/>
+      <c r="F350" s="6"/>
+      <c r="G350" s="6"/>
+      <c r="H350" s="6"/>
+      <c r="I350" s="6"/>
+      <c r="J350" s="7"/>
+    </row>
+    <row r="351" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C351" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D351" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E351" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F351" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G351" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H351" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I351" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J351" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="352" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C352" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D352" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="E352" s="1"/>
+      <c r="F352" s="1"/>
+      <c r="G352" s="1"/>
+      <c r="H352" s="1"/>
+      <c r="I352" s="1"/>
+      <c r="J352" s="1"/>
+    </row>
+    <row r="353" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C353" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D353" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="E353" s="1">
+        <v>83.3333333333333</v>
+      </c>
+      <c r="I353" s="1"/>
+      <c r="J353" s="1"/>
+    </row>
+    <row r="354" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C354" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D354" s="1">
+        <v>94.7916666666666</v>
+      </c>
+      <c r="E354" s="1">
+        <v>78.125</v>
+      </c>
+      <c r="F354" s="1">
+        <v>97.9166666666666</v>
+      </c>
+      <c r="H354" s="1"/>
+      <c r="I354" s="1"/>
+      <c r="J354" s="1"/>
+    </row>
+    <row r="355" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C355" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D355" s="1">
+        <v>92.7083333333333</v>
+      </c>
+      <c r="E355" s="1">
+        <v>80.2083333333333</v>
+      </c>
+      <c r="F355" s="1">
+        <v>96.875</v>
+      </c>
+      <c r="G355" s="1">
+        <v>47.9166666666666</v>
+      </c>
+      <c r="H355" s="1"/>
+      <c r="I355" s="1"/>
+      <c r="J355" s="1"/>
+    </row>
+    <row r="356" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C356" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D356" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="E356" s="1">
+        <v>83.3333333333333</v>
+      </c>
+      <c r="F356" s="1">
+        <v>97.9166666666666</v>
+      </c>
+      <c r="G356" s="1">
+        <v>46.875</v>
+      </c>
+      <c r="H356" s="1">
+        <v>51.0416666666666</v>
+      </c>
+      <c r="I356" s="1"/>
+      <c r="J356" s="1"/>
+    </row>
+    <row r="357" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C357" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D357" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="E357" s="1">
+        <v>81.25</v>
+      </c>
+      <c r="F357" s="1">
+        <v>97.9166666666666</v>
+      </c>
+      <c r="G357" s="1">
+        <v>46.875</v>
+      </c>
+      <c r="H357" s="1">
+        <v>50</v>
+      </c>
+      <c r="I357" s="1">
+        <v>75</v>
+      </c>
+      <c r="J357" s="1"/>
+    </row>
+    <row r="358" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C358" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D358" s="1">
+        <v>92.7083333333333</v>
+      </c>
+      <c r="E358" s="1">
+        <v>76.0416666666666</v>
+      </c>
+      <c r="F358" s="1">
+        <v>97.9166666666666</v>
+      </c>
+      <c r="G358" s="1">
+        <v>35.4166666666666</v>
+      </c>
+      <c r="H358" s="1">
+        <v>61.4583333333333</v>
+      </c>
+      <c r="I358" s="1">
+        <v>64.5833333333333</v>
+      </c>
+      <c r="J358" s="1">
+        <v>42.7083333333333</v>
+      </c>
+    </row>
+    <row r="360" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C360" t="s">
+        <v>8</v>
+      </c>
+      <c r="D360">
+        <f>AVERAGE(D358:J358)</f>
+        <v>67.261904761904731</v>
+      </c>
+      <c r="F360" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G360" s="4"/>
+      <c r="H360" s="4"/>
+      <c r="I360" s="4"/>
+    </row>
+    <row r="361" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C361" t="s">
+        <v>9</v>
+      </c>
+      <c r="D361">
+        <f>(SUM((D358-D352)+(E358-E353)+(F358-F354)+(G358-G355)+(H358-H356)+(I358-I357)))/6</f>
+        <v>-3.4722222222222334</v>
+      </c>
+      <c r="F361" s="4"/>
+      <c r="G361" s="4"/>
+      <c r="H361" s="4"/>
+      <c r="I361" s="4"/>
+    </row>
+    <row r="362" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C362" t="s">
+        <v>10</v>
+      </c>
+      <c r="D362">
+        <f>SUM((MAX(D352:D358)-D358)+(MAX(E353:E358)-E358)+(MAX(F355:F358)-F358)+(MAX(G355:G358)-G358)+(MAX(H356:H358)-H358)+(MAX(I357:I358)-I358))/6</f>
+        <v>5.38194444444445</v>
+      </c>
+      <c r="F362" s="4"/>
+      <c r="G362" s="4"/>
+      <c r="H362" s="4"/>
+      <c r="I362" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="M209:T209"/>
-    <mergeCell ref="C203:J204"/>
-    <mergeCell ref="C209:J209"/>
-    <mergeCell ref="C226:J226"/>
-    <mergeCell ref="C242:J242"/>
-    <mergeCell ref="C184:J184"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="C23:J23"/>
-    <mergeCell ref="C39:J39"/>
-    <mergeCell ref="C55:J55"/>
-    <mergeCell ref="C70:J70"/>
+  <mergeCells count="32">
     <mergeCell ref="C169:J169"/>
     <mergeCell ref="C86:J86"/>
     <mergeCell ref="C107:J107"/>
     <mergeCell ref="C123:J123"/>
     <mergeCell ref="C139:J139"/>
     <mergeCell ref="C154:J154"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="C39:J39"/>
+    <mergeCell ref="C55:J55"/>
+    <mergeCell ref="C70:J70"/>
+    <mergeCell ref="C203:J204"/>
+    <mergeCell ref="C209:J209"/>
+    <mergeCell ref="C226:J226"/>
+    <mergeCell ref="C242:J242"/>
+    <mergeCell ref="C184:J184"/>
+    <mergeCell ref="M209:T209"/>
+    <mergeCell ref="M226:T226"/>
+    <mergeCell ref="M242:T242"/>
+    <mergeCell ref="C268:J268"/>
+    <mergeCell ref="C287:J287"/>
+    <mergeCell ref="F360:I362"/>
+    <mergeCell ref="P252:T255"/>
+    <mergeCell ref="F344:I346"/>
+    <mergeCell ref="C303:J303"/>
+    <mergeCell ref="C319:J319"/>
+    <mergeCell ref="C334:J334"/>
+    <mergeCell ref="C350:J350"/>
+    <mergeCell ref="F278:I280"/>
+    <mergeCell ref="F297:I299"/>
+    <mergeCell ref="F313:I315"/>
+    <mergeCell ref="F329:I331"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update: README update, log update for task_aware. Put LEAR_task_aware backup file
</commit_message>
<xml_diff>
--- a/metrix_calculation.xlsx
+++ b/metrix_calculation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course\CS_764\project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course\CS_764\project\NeurIPS2025-LEAR-main\csi764_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49CECC17-9C04-49EB-9417-7B59243D3325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C115F016-8215-4692-85B9-20E2C4B7C120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="42">
   <si>
     <t>After Task</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -199,6 +199,12 @@
   <si>
     <t>[DEBUG] Task 7 -&gt; Expert 2
 [DEBUG] Task-expert mapping: [1, 1, 1, 2, 3, 4, 2]
+[DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[DEBUG] Task 7 -&gt; Expert 2
+[DEBUG] Task-expert mapping: [1, 1, 1, 2, 1, 3, 2]
 [DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -374,12 +380,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -405,6 +405,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -700,16 +706,16 @@
   <sheetData>
     <row r="3" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="7"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C5" s="2" t="s">
@@ -906,16 +912,16 @@
     </row>
     <row r="22" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="7"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="5"/>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C24" s="2" t="s">
@@ -1112,16 +1118,16 @@
     </row>
     <row r="38" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="7"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="5"/>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C40" s="2" t="s">
@@ -1318,16 +1324,16 @@
     </row>
     <row r="54" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6"/>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
-      <c r="I55" s="6"/>
-      <c r="J55" s="7"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+      <c r="H55" s="4"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="5"/>
     </row>
     <row r="56" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C56" s="2" t="s">
@@ -1524,16 +1530,16 @@
     </row>
     <row r="69" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="70" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="5" t="s">
+      <c r="C70" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D70" s="6"/>
-      <c r="E70" s="6"/>
-      <c r="F70" s="6"/>
-      <c r="G70" s="6"/>
-      <c r="H70" s="6"/>
-      <c r="I70" s="6"/>
-      <c r="J70" s="7"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+      <c r="H70" s="4"/>
+      <c r="I70" s="4"/>
+      <c r="J70" s="5"/>
     </row>
     <row r="71" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C71" s="2" t="s">
@@ -1730,16 +1736,16 @@
     </row>
     <row r="85" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="86" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="5" t="s">
+      <c r="C86" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D86" s="6"/>
-      <c r="E86" s="6"/>
-      <c r="F86" s="6"/>
-      <c r="G86" s="6"/>
-      <c r="H86" s="6"/>
-      <c r="I86" s="6"/>
-      <c r="J86" s="7"/>
+      <c r="D86" s="4"/>
+      <c r="E86" s="4"/>
+      <c r="F86" s="4"/>
+      <c r="G86" s="4"/>
+      <c r="H86" s="4"/>
+      <c r="I86" s="4"/>
+      <c r="J86" s="5"/>
     </row>
     <row r="87" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C87" s="2" t="s">
@@ -1936,16 +1942,16 @@
     </row>
     <row r="106" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="107" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C107" s="5" t="s">
+      <c r="C107" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D107" s="6"/>
-      <c r="E107" s="6"/>
-      <c r="F107" s="6"/>
-      <c r="G107" s="6"/>
-      <c r="H107" s="6"/>
-      <c r="I107" s="6"/>
-      <c r="J107" s="7"/>
+      <c r="D107" s="4"/>
+      <c r="E107" s="4"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="4"/>
+      <c r="H107" s="4"/>
+      <c r="I107" s="4"/>
+      <c r="J107" s="5"/>
     </row>
     <row r="108" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C108" s="2" t="s">
@@ -2142,16 +2148,16 @@
     </row>
     <row r="122" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="123" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C123" s="5" t="s">
+      <c r="C123" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D123" s="6"/>
-      <c r="E123" s="6"/>
-      <c r="F123" s="6"/>
-      <c r="G123" s="6"/>
-      <c r="H123" s="6"/>
-      <c r="I123" s="6"/>
-      <c r="J123" s="7"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
+      <c r="G123" s="4"/>
+      <c r="H123" s="4"/>
+      <c r="I123" s="4"/>
+      <c r="J123" s="5"/>
     </row>
     <row r="124" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C124" s="2" t="s">
@@ -2348,16 +2354,16 @@
     </row>
     <row r="138" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="139" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C139" s="5" t="s">
+      <c r="C139" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D139" s="6"/>
-      <c r="E139" s="6"/>
-      <c r="F139" s="6"/>
-      <c r="G139" s="6"/>
-      <c r="H139" s="6"/>
-      <c r="I139" s="6"/>
-      <c r="J139" s="7"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="4"/>
+      <c r="F139" s="4"/>
+      <c r="G139" s="4"/>
+      <c r="H139" s="4"/>
+      <c r="I139" s="4"/>
+      <c r="J139" s="5"/>
     </row>
     <row r="140" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C140" s="2" t="s">
@@ -2554,16 +2560,16 @@
     </row>
     <row r="153" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="154" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C154" s="5" t="s">
+      <c r="C154" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D154" s="6"/>
-      <c r="E154" s="6"/>
-      <c r="F154" s="6"/>
-      <c r="G154" s="6"/>
-      <c r="H154" s="6"/>
-      <c r="I154" s="6"/>
-      <c r="J154" s="7"/>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4"/>
+      <c r="F154" s="4"/>
+      <c r="G154" s="4"/>
+      <c r="H154" s="4"/>
+      <c r="I154" s="4"/>
+      <c r="J154" s="5"/>
     </row>
     <row r="155" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C155" s="2" t="s">
@@ -2760,16 +2766,16 @@
     </row>
     <row r="168" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="169" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C169" s="5" t="s">
+      <c r="C169" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D169" s="6"/>
-      <c r="E169" s="6"/>
-      <c r="F169" s="6"/>
-      <c r="G169" s="6"/>
-      <c r="H169" s="6"/>
-      <c r="I169" s="6"/>
-      <c r="J169" s="7"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="4"/>
+      <c r="H169" s="4"/>
+      <c r="I169" s="4"/>
+      <c r="J169" s="5"/>
     </row>
     <row r="170" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C170" s="2" t="s">
@@ -2966,16 +2972,16 @@
     </row>
     <row r="183" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="184" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C184" s="5" t="s">
+      <c r="C184" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D184" s="6"/>
-      <c r="E184" s="6"/>
-      <c r="F184" s="6"/>
-      <c r="G184" s="6"/>
-      <c r="H184" s="6"/>
-      <c r="I184" s="6"/>
-      <c r="J184" s="7"/>
+      <c r="D184" s="4"/>
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
+      <c r="G184" s="4"/>
+      <c r="H184" s="4"/>
+      <c r="I184" s="4"/>
+      <c r="J184" s="5"/>
     </row>
     <row r="185" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C185" s="2" t="s">
@@ -3171,49 +3177,49 @@
     </row>
     <row r="202" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="203" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C203" s="8" t="s">
+      <c r="C203" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D203" s="9"/>
-      <c r="E203" s="9"/>
-      <c r="F203" s="9"/>
-      <c r="G203" s="9"/>
-      <c r="H203" s="9"/>
-      <c r="I203" s="9"/>
-      <c r="J203" s="10"/>
+      <c r="D203" s="7"/>
+      <c r="E203" s="7"/>
+      <c r="F203" s="7"/>
+      <c r="G203" s="7"/>
+      <c r="H203" s="7"/>
+      <c r="I203" s="7"/>
+      <c r="J203" s="8"/>
     </row>
     <row r="204" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C204" s="11"/>
-      <c r="D204" s="12"/>
-      <c r="E204" s="12"/>
-      <c r="F204" s="12"/>
-      <c r="G204" s="12"/>
-      <c r="H204" s="12"/>
-      <c r="I204" s="12"/>
-      <c r="J204" s="13"/>
+      <c r="C204" s="9"/>
+      <c r="D204" s="10"/>
+      <c r="E204" s="10"/>
+      <c r="F204" s="10"/>
+      <c r="G204" s="10"/>
+      <c r="H204" s="10"/>
+      <c r="I204" s="10"/>
+      <c r="J204" s="11"/>
     </row>
     <row r="208" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="209" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C209" s="5" t="s">
+      <c r="C209" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D209" s="6"/>
-      <c r="E209" s="6"/>
-      <c r="F209" s="6"/>
-      <c r="G209" s="6"/>
-      <c r="H209" s="6"/>
-      <c r="I209" s="6"/>
-      <c r="J209" s="7"/>
-      <c r="M209" s="5" t="s">
+      <c r="D209" s="4"/>
+      <c r="E209" s="4"/>
+      <c r="F209" s="4"/>
+      <c r="G209" s="4"/>
+      <c r="H209" s="4"/>
+      <c r="I209" s="4"/>
+      <c r="J209" s="5"/>
+      <c r="M209" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="N209" s="6"/>
-      <c r="O209" s="6"/>
-      <c r="P209" s="6"/>
-      <c r="Q209" s="6"/>
-      <c r="R209" s="6"/>
-      <c r="S209" s="6"/>
-      <c r="T209" s="7"/>
+      <c r="N209" s="4"/>
+      <c r="O209" s="4"/>
+      <c r="P209" s="4"/>
+      <c r="Q209" s="4"/>
+      <c r="R209" s="4"/>
+      <c r="S209" s="4"/>
+      <c r="T209" s="5"/>
     </row>
     <row r="210" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C210" s="2" t="s">
@@ -3544,6 +3550,13 @@
         <f>AVERAGE(N217:T217)</f>
         <v>82.530676877430466</v>
       </c>
+      <c r="P219" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q219" s="12"/>
+      <c r="R219" s="12"/>
+      <c r="S219" s="12"/>
+      <c r="T219" s="12"/>
     </row>
     <row r="220" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C220" t="s">
@@ -3560,6 +3573,11 @@
         <f>(SUM((N217-N211)+(O217-O212)+(P217-P213)+(Q217-Q214)+(R217-R215)+(S217-S216)))/6</f>
         <v>-2.6178149980728307</v>
       </c>
+      <c r="P220" s="12"/>
+      <c r="Q220" s="12"/>
+      <c r="R220" s="12"/>
+      <c r="S220" s="12"/>
+      <c r="T220" s="12"/>
     </row>
     <row r="221" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C221" t="s">
@@ -3576,29 +3594,41 @@
         <f>SUM((MAX(N211:N217)-N217)+(MAX(O212:O217)-O217)+(MAX(P213:P217)-P217)+(MAX(Q214:Q217)-Q217)+(MAX(R215:R217)-R217)+(MAX(S216:S217)-S217))/6</f>
         <v>2.6257869368483306</v>
       </c>
+      <c r="P221" s="12"/>
+      <c r="Q221" s="12"/>
+      <c r="R221" s="12"/>
+      <c r="S221" s="12"/>
+      <c r="T221" s="12"/>
+    </row>
+    <row r="222" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="P222" s="12"/>
+      <c r="Q222" s="12"/>
+      <c r="R222" s="12"/>
+      <c r="S222" s="12"/>
+      <c r="T222" s="12"/>
     </row>
     <row r="225" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="226" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C226" s="5" t="s">
+      <c r="C226" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D226" s="6"/>
-      <c r="E226" s="6"/>
-      <c r="F226" s="6"/>
-      <c r="G226" s="6"/>
-      <c r="H226" s="6"/>
-      <c r="I226" s="6"/>
-      <c r="J226" s="7"/>
-      <c r="M226" s="5" t="s">
+      <c r="D226" s="4"/>
+      <c r="E226" s="4"/>
+      <c r="F226" s="4"/>
+      <c r="G226" s="4"/>
+      <c r="H226" s="4"/>
+      <c r="I226" s="4"/>
+      <c r="J226" s="5"/>
+      <c r="M226" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="N226" s="6"/>
-      <c r="O226" s="6"/>
-      <c r="P226" s="6"/>
-      <c r="Q226" s="6"/>
-      <c r="R226" s="6"/>
-      <c r="S226" s="6"/>
-      <c r="T226" s="7"/>
+      <c r="N226" s="4"/>
+      <c r="O226" s="4"/>
+      <c r="P226" s="4"/>
+      <c r="Q226" s="4"/>
+      <c r="R226" s="4"/>
+      <c r="S226" s="4"/>
+      <c r="T226" s="5"/>
     </row>
     <row r="227" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C227" s="2" t="s">
@@ -3964,26 +3994,26 @@
     </row>
     <row r="241" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="242" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C242" s="5" t="s">
+      <c r="C242" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D242" s="6"/>
-      <c r="E242" s="6"/>
-      <c r="F242" s="6"/>
-      <c r="G242" s="6"/>
-      <c r="H242" s="6"/>
-      <c r="I242" s="6"/>
-      <c r="J242" s="7"/>
-      <c r="M242" s="5" t="s">
+      <c r="D242" s="4"/>
+      <c r="E242" s="4"/>
+      <c r="F242" s="4"/>
+      <c r="G242" s="4"/>
+      <c r="H242" s="4"/>
+      <c r="I242" s="4"/>
+      <c r="J242" s="5"/>
+      <c r="M242" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="N242" s="6"/>
-      <c r="O242" s="6"/>
-      <c r="P242" s="6"/>
-      <c r="Q242" s="6"/>
-      <c r="R242" s="6"/>
-      <c r="S242" s="6"/>
-      <c r="T242" s="7"/>
+      <c r="N242" s="4"/>
+      <c r="O242" s="4"/>
+      <c r="P242" s="4"/>
+      <c r="Q242" s="4"/>
+      <c r="R242" s="4"/>
+      <c r="S242" s="4"/>
+      <c r="T242" s="5"/>
     </row>
     <row r="243" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C243" s="2" t="s">
@@ -4314,13 +4344,13 @@
         <f>AVERAGE(N250:T250)</f>
         <v>83.400848007784504</v>
       </c>
-      <c r="P252" s="3" t="s">
+      <c r="P252" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="Q252" s="3"/>
-      <c r="R252" s="3"/>
-      <c r="S252" s="3"/>
-      <c r="T252" s="3"/>
+      <c r="Q252" s="12"/>
+      <c r="R252" s="12"/>
+      <c r="S252" s="12"/>
+      <c r="T252" s="12"/>
     </row>
     <row r="253" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C253" t="s">
@@ -4337,11 +4367,11 @@
         <f>(SUM((N250-N244)+(O250-O245)+(P250-P246)+(Q250-Q247)+(R250-R248)+(S250-S249)))/6</f>
         <v>-2.0617011500049522</v>
       </c>
-      <c r="P253" s="3"/>
-      <c r="Q253" s="3"/>
-      <c r="R253" s="3"/>
-      <c r="S253" s="3"/>
-      <c r="T253" s="3"/>
+      <c r="P253" s="12"/>
+      <c r="Q253" s="12"/>
+      <c r="R253" s="12"/>
+      <c r="S253" s="12"/>
+      <c r="T253" s="12"/>
     </row>
     <row r="254" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C254" t="s">
@@ -4358,31 +4388,31 @@
         <f>SUM((MAX(N244:N250)-N250)+(MAX(O245:O250)-O250)+(MAX(P246:P250)-P250)+(MAX(Q247:Q250)-Q250)+(MAX(R248:R250)-R250)+(MAX(S249:S250)-S250))/6</f>
         <v>2.0617011500049522</v>
       </c>
-      <c r="P254" s="3"/>
-      <c r="Q254" s="3"/>
-      <c r="R254" s="3"/>
-      <c r="S254" s="3"/>
-      <c r="T254" s="3"/>
+      <c r="P254" s="12"/>
+      <c r="Q254" s="12"/>
+      <c r="R254" s="12"/>
+      <c r="S254" s="12"/>
+      <c r="T254" s="12"/>
     </row>
     <row r="255" spans="3:20" x14ac:dyDescent="0.2">
-      <c r="P255" s="3"/>
-      <c r="Q255" s="3"/>
-      <c r="R255" s="3"/>
-      <c r="S255" s="3"/>
-      <c r="T255" s="3"/>
+      <c r="P255" s="12"/>
+      <c r="Q255" s="12"/>
+      <c r="R255" s="12"/>
+      <c r="S255" s="12"/>
+      <c r="T255" s="12"/>
     </row>
     <row r="267" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="268" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C268" s="5" t="s">
+      <c r="C268" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D268" s="6"/>
-      <c r="E268" s="6"/>
-      <c r="F268" s="6"/>
-      <c r="G268" s="6"/>
-      <c r="H268" s="6"/>
-      <c r="I268" s="6"/>
-      <c r="J268" s="7"/>
+      <c r="D268" s="4"/>
+      <c r="E268" s="4"/>
+      <c r="F268" s="4"/>
+      <c r="G268" s="4"/>
+      <c r="H268" s="4"/>
+      <c r="I268" s="4"/>
+      <c r="J268" s="5"/>
     </row>
     <row r="269" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C269" s="2" t="s">
@@ -4558,12 +4588,12 @@
         <f>AVERAGE(D276:J276)</f>
         <v>73.9583333333333</v>
       </c>
-      <c r="F278" s="3" t="s">
+      <c r="F278" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="G278" s="4"/>
-      <c r="H278" s="4"/>
-      <c r="I278" s="4"/>
+      <c r="G278" s="13"/>
+      <c r="H278" s="13"/>
+      <c r="I278" s="13"/>
     </row>
     <row r="279" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C279" t="s">
@@ -4573,10 +4603,10 @@
         <f>(SUM((D276-D270)+(E276-E271)+(F276-F272)+(G276-G273)+(H276-H274)+(I276-I275)))/6</f>
         <v>-0.17361111111111663</v>
       </c>
-      <c r="F279" s="4"/>
-      <c r="G279" s="4"/>
-      <c r="H279" s="4"/>
-      <c r="I279" s="4"/>
+      <c r="F279" s="13"/>
+      <c r="G279" s="13"/>
+      <c r="H279" s="13"/>
+      <c r="I279" s="13"/>
     </row>
     <row r="280" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C280" t="s">
@@ -4586,23 +4616,23 @@
         <f>SUM((MAX(D270:D276)-D276)+(MAX(E271:E276)-E276)+(MAX(F272:F276)-F276)+(MAX(G273:G276)-G276)+(MAX(H274:H276)-H276)+(MAX(I275:I276)-I276))/6</f>
         <v>1.9097222222222499</v>
       </c>
-      <c r="F280" s="4"/>
-      <c r="G280" s="4"/>
-      <c r="H280" s="4"/>
-      <c r="I280" s="4"/>
+      <c r="F280" s="13"/>
+      <c r="G280" s="13"/>
+      <c r="H280" s="13"/>
+      <c r="I280" s="13"/>
     </row>
     <row r="286" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="287" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C287" s="5" t="s">
+      <c r="C287" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D287" s="6"/>
-      <c r="E287" s="6"/>
-      <c r="F287" s="6"/>
-      <c r="G287" s="6"/>
-      <c r="H287" s="6"/>
-      <c r="I287" s="6"/>
-      <c r="J287" s="7"/>
+      <c r="D287" s="4"/>
+      <c r="E287" s="4"/>
+      <c r="F287" s="4"/>
+      <c r="G287" s="4"/>
+      <c r="H287" s="4"/>
+      <c r="I287" s="4"/>
+      <c r="J287" s="5"/>
     </row>
     <row r="288" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C288" s="2" t="s">
@@ -4778,12 +4808,12 @@
         <f>AVERAGE(D295:J295)</f>
         <v>64.5833333333333</v>
       </c>
-      <c r="F297" s="3" t="s">
+      <c r="F297" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="G297" s="4"/>
-      <c r="H297" s="4"/>
-      <c r="I297" s="4"/>
+      <c r="G297" s="13"/>
+      <c r="H297" s="13"/>
+      <c r="I297" s="13"/>
     </row>
     <row r="298" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C298" t="s">
@@ -4793,10 +4823,10 @@
         <f>(SUM((D295-D289)+(E295-E290)+(F295-F291)+(G295-G292)+(H295-H293)+(I295-I294)))/6</f>
         <v>-2.7777777777777835</v>
       </c>
-      <c r="F298" s="4"/>
-      <c r="G298" s="4"/>
-      <c r="H298" s="4"/>
-      <c r="I298" s="4"/>
+      <c r="F298" s="13"/>
+      <c r="G298" s="13"/>
+      <c r="H298" s="13"/>
+      <c r="I298" s="13"/>
     </row>
     <row r="299" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C299" t="s">
@@ -4806,23 +4836,23 @@
         <f>SUM((MAX(D289:D295)-D295)+(MAX(E290:E295)-E295)+(MAX(F291:F295)-F295)+(MAX(G292:G295)-G295)+(MAX(H293:H295)-H295)+(MAX(I294:I295)-I295))/6</f>
         <v>5.208333333333333</v>
       </c>
-      <c r="F299" s="4"/>
-      <c r="G299" s="4"/>
-      <c r="H299" s="4"/>
-      <c r="I299" s="4"/>
+      <c r="F299" s="13"/>
+      <c r="G299" s="13"/>
+      <c r="H299" s="13"/>
+      <c r="I299" s="13"/>
     </row>
     <row r="302" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="303" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C303" s="5" t="s">
+      <c r="C303" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D303" s="6"/>
-      <c r="E303" s="6"/>
-      <c r="F303" s="6"/>
-      <c r="G303" s="6"/>
-      <c r="H303" s="6"/>
-      <c r="I303" s="6"/>
-      <c r="J303" s="7"/>
+      <c r="D303" s="4"/>
+      <c r="E303" s="4"/>
+      <c r="F303" s="4"/>
+      <c r="G303" s="4"/>
+      <c r="H303" s="4"/>
+      <c r="I303" s="4"/>
+      <c r="J303" s="5"/>
     </row>
     <row r="304" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C304" s="2" t="s">
@@ -4998,12 +5028,12 @@
         <f>AVERAGE(D311:J311)</f>
         <v>78.298611111111072</v>
       </c>
-      <c r="F313" s="3" t="s">
+      <c r="F313" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="G313" s="4"/>
-      <c r="H313" s="4"/>
-      <c r="I313" s="4"/>
+      <c r="G313" s="13"/>
+      <c r="H313" s="13"/>
+      <c r="I313" s="13"/>
     </row>
     <row r="314" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C314" t="s">
@@ -5013,10 +5043,10 @@
         <f>(SUM((D311-D305)+(E311-E306)+(F311-F307)+(G311-G308)+(H311-H309)+(I311-I310)))/6</f>
         <v>0.34722222222220012</v>
       </c>
-      <c r="F314" s="4"/>
-      <c r="G314" s="4"/>
-      <c r="H314" s="4"/>
-      <c r="I314" s="4"/>
+      <c r="F314" s="13"/>
+      <c r="G314" s="13"/>
+      <c r="H314" s="13"/>
+      <c r="I314" s="13"/>
     </row>
     <row r="315" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C315" t="s">
@@ -5026,23 +5056,23 @@
         <f>SUM((MAX(D305:D311)-D311)+(MAX(E306:E311)-E311)+(MAX(F307:F311)-F311)+(MAX(G308:G311)-G311)+(MAX(H309:H311)-H311)+(MAX(I310:I311)-I311))/6</f>
         <v>2.4305555555555665</v>
       </c>
-      <c r="F315" s="4"/>
-      <c r="G315" s="4"/>
-      <c r="H315" s="4"/>
-      <c r="I315" s="4"/>
+      <c r="F315" s="13"/>
+      <c r="G315" s="13"/>
+      <c r="H315" s="13"/>
+      <c r="I315" s="13"/>
     </row>
     <row r="318" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="319" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C319" s="5" t="s">
+      <c r="C319" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D319" s="6"/>
-      <c r="E319" s="6"/>
-      <c r="F319" s="6"/>
-      <c r="G319" s="6"/>
-      <c r="H319" s="6"/>
-      <c r="I319" s="6"/>
-      <c r="J319" s="7"/>
+      <c r="D319" s="4"/>
+      <c r="E319" s="4"/>
+      <c r="F319" s="4"/>
+      <c r="G319" s="4"/>
+      <c r="H319" s="4"/>
+      <c r="I319" s="4"/>
+      <c r="J319" s="5"/>
     </row>
     <row r="320" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C320" s="2" t="s">
@@ -5218,12 +5248,12 @@
         <f>AVERAGE(D327:J327)</f>
         <v>73.660714285714249</v>
       </c>
-      <c r="F329" s="3" t="s">
+      <c r="F329" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G329" s="4"/>
-      <c r="H329" s="4"/>
-      <c r="I329" s="4"/>
+      <c r="G329" s="13"/>
+      <c r="H329" s="13"/>
+      <c r="I329" s="13"/>
     </row>
     <row r="330" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C330" t="s">
@@ -5233,10 +5263,10 @@
         <f>(SUM((D327-D321)+(E327-E322)+(F327-F323)+(G327-G324)+(H327-H325)+(I327-I326)))/6</f>
         <v>-1.3888888888888999</v>
       </c>
-      <c r="F330" s="4"/>
-      <c r="G330" s="4"/>
-      <c r="H330" s="4"/>
-      <c r="I330" s="4"/>
+      <c r="F330" s="13"/>
+      <c r="G330" s="13"/>
+      <c r="H330" s="13"/>
+      <c r="I330" s="13"/>
     </row>
     <row r="331" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C331" t="s">
@@ -5246,23 +5276,23 @@
         <f>SUM((MAX(D321:D327)-D327)+(MAX(E322:E327)-E327)+(MAX(F323:F327)-F327)+(MAX(G324:G327)-G327)+(MAX(H325:H327)-H327)+(MAX(I326:I327)-I327))/6</f>
         <v>2.6041666666666665</v>
       </c>
-      <c r="F331" s="4"/>
-      <c r="G331" s="4"/>
-      <c r="H331" s="4"/>
-      <c r="I331" s="4"/>
+      <c r="F331" s="13"/>
+      <c r="G331" s="13"/>
+      <c r="H331" s="13"/>
+      <c r="I331" s="13"/>
     </row>
     <row r="333" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="334" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C334" s="5" t="s">
+      <c r="C334" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D334" s="6"/>
-      <c r="E334" s="6"/>
-      <c r="F334" s="6"/>
-      <c r="G334" s="6"/>
-      <c r="H334" s="6"/>
-      <c r="I334" s="6"/>
-      <c r="J334" s="7"/>
+      <c r="D334" s="4"/>
+      <c r="E334" s="4"/>
+      <c r="F334" s="4"/>
+      <c r="G334" s="4"/>
+      <c r="H334" s="4"/>
+      <c r="I334" s="4"/>
+      <c r="J334" s="5"/>
     </row>
     <row r="335" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C335" s="2" t="s">
@@ -5438,12 +5468,12 @@
         <f>AVERAGE(D342:J342)</f>
         <v>71.577380952380935</v>
       </c>
-      <c r="F344" s="3" t="s">
+      <c r="F344" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G344" s="4"/>
-      <c r="H344" s="4"/>
-      <c r="I344" s="4"/>
+      <c r="G344" s="13"/>
+      <c r="H344" s="13"/>
+      <c r="I344" s="13"/>
     </row>
     <row r="345" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C345" t="s">
@@ -5453,10 +5483,10 @@
         <f>(SUM((D342-D336)+(E342-E337)+(F342-F338)+(G342-G339)+(H342-H340)+(I342-I341)))/6</f>
         <v>-1.0416666666666667</v>
       </c>
-      <c r="F345" s="4"/>
-      <c r="G345" s="4"/>
-      <c r="H345" s="4"/>
-      <c r="I345" s="4"/>
+      <c r="F345" s="13"/>
+      <c r="G345" s="13"/>
+      <c r="H345" s="13"/>
+      <c r="I345" s="13"/>
     </row>
     <row r="346" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C346" t="s">
@@ -5466,23 +5496,23 @@
         <f>SUM((MAX(D336:D342)-D342)+(MAX(E337:E342)-E342)+(MAX(F338:F342)-F342)+(MAX(G339:G342)-G342)+(MAX(H340:H342)-H342)+(MAX(I341:I342)-I342))/6</f>
         <v>2.6041666666666665</v>
       </c>
-      <c r="F346" s="4"/>
-      <c r="G346" s="4"/>
-      <c r="H346" s="4"/>
-      <c r="I346" s="4"/>
+      <c r="F346" s="13"/>
+      <c r="G346" s="13"/>
+      <c r="H346" s="13"/>
+      <c r="I346" s="13"/>
     </row>
     <row r="349" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="350" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C350" s="5" t="s">
+      <c r="C350" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D350" s="6"/>
-      <c r="E350" s="6"/>
-      <c r="F350" s="6"/>
-      <c r="G350" s="6"/>
-      <c r="H350" s="6"/>
-      <c r="I350" s="6"/>
-      <c r="J350" s="7"/>
+      <c r="D350" s="4"/>
+      <c r="E350" s="4"/>
+      <c r="F350" s="4"/>
+      <c r="G350" s="4"/>
+      <c r="H350" s="4"/>
+      <c r="I350" s="4"/>
+      <c r="J350" s="5"/>
     </row>
     <row r="351" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C351" s="2" t="s">
@@ -5654,12 +5684,12 @@
         <f>AVERAGE(D358:J358)</f>
         <v>67.261904761904731</v>
       </c>
-      <c r="F360" s="3" t="s">
+      <c r="F360" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G360" s="4"/>
-      <c r="H360" s="4"/>
-      <c r="I360" s="4"/>
+      <c r="G360" s="13"/>
+      <c r="H360" s="13"/>
+      <c r="I360" s="13"/>
     </row>
     <row r="361" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C361" t="s">
@@ -5669,10 +5699,10 @@
         <f>(SUM((D358-D352)+(E358-E353)+(F358-F354)+(G358-G355)+(H358-H356)+(I358-I357)))/6</f>
         <v>-3.4722222222222334</v>
       </c>
-      <c r="F361" s="4"/>
-      <c r="G361" s="4"/>
-      <c r="H361" s="4"/>
-      <c r="I361" s="4"/>
+      <c r="F361" s="13"/>
+      <c r="G361" s="13"/>
+      <c r="H361" s="13"/>
+      <c r="I361" s="13"/>
     </row>
     <row r="362" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C362" t="s">
@@ -5682,34 +5712,13 @@
         <f>SUM((MAX(D352:D358)-D358)+(MAX(E353:E358)-E358)+(MAX(F355:F358)-F358)+(MAX(G355:G358)-G358)+(MAX(H356:H358)-H358)+(MAX(I357:I358)-I358))/6</f>
         <v>5.38194444444445</v>
       </c>
-      <c r="F362" s="4"/>
-      <c r="G362" s="4"/>
-      <c r="H362" s="4"/>
-      <c r="I362" s="4"/>
+      <c r="F362" s="13"/>
+      <c r="G362" s="13"/>
+      <c r="H362" s="13"/>
+      <c r="I362" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="C169:J169"/>
-    <mergeCell ref="C86:J86"/>
-    <mergeCell ref="C107:J107"/>
-    <mergeCell ref="C123:J123"/>
-    <mergeCell ref="C139:J139"/>
-    <mergeCell ref="C154:J154"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="C23:J23"/>
-    <mergeCell ref="C39:J39"/>
-    <mergeCell ref="C55:J55"/>
-    <mergeCell ref="C70:J70"/>
-    <mergeCell ref="C203:J204"/>
-    <mergeCell ref="C209:J209"/>
-    <mergeCell ref="C226:J226"/>
-    <mergeCell ref="C242:J242"/>
-    <mergeCell ref="C184:J184"/>
-    <mergeCell ref="M209:T209"/>
-    <mergeCell ref="M226:T226"/>
-    <mergeCell ref="M242:T242"/>
-    <mergeCell ref="C268:J268"/>
-    <mergeCell ref="C287:J287"/>
+  <mergeCells count="33">
     <mergeCell ref="F360:I362"/>
     <mergeCell ref="P252:T255"/>
     <mergeCell ref="F344:I346"/>
@@ -5721,6 +5730,28 @@
     <mergeCell ref="F297:I299"/>
     <mergeCell ref="F313:I315"/>
     <mergeCell ref="F329:I331"/>
+    <mergeCell ref="M209:T209"/>
+    <mergeCell ref="M226:T226"/>
+    <mergeCell ref="M242:T242"/>
+    <mergeCell ref="C268:J268"/>
+    <mergeCell ref="C287:J287"/>
+    <mergeCell ref="P219:T222"/>
+    <mergeCell ref="C203:J204"/>
+    <mergeCell ref="C209:J209"/>
+    <mergeCell ref="C226:J226"/>
+    <mergeCell ref="C242:J242"/>
+    <mergeCell ref="C184:J184"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="C39:J39"/>
+    <mergeCell ref="C55:J55"/>
+    <mergeCell ref="C70:J70"/>
+    <mergeCell ref="C169:J169"/>
+    <mergeCell ref="C86:J86"/>
+    <mergeCell ref="C107:J107"/>
+    <mergeCell ref="C123:J123"/>
+    <mergeCell ref="C139:J139"/>
+    <mergeCell ref="C154:J154"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
random_control_snippet & update: README update and random_control add in models\LEAR.py
</commit_message>
<xml_diff>
--- a/metrix_calculation.xlsx
+++ b/metrix_calculation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course\CS_764\project\NeurIPS2025-LEAR-main\csi764_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C115F016-8215-4692-85B9-20E2C4B7C120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F642EBF6-C0DC-430C-A927-4AD23980B035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="45">
   <si>
     <t>After Task</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -140,18 +140,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>t = 33 t_Agnostic Claude version</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>original Claude Version comparsion</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>t = 33 task aware Claude</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>t = 20 t_aware claude</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -203,9 +191,35 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>t = 33 t_Agnostic New version</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>original New Version comparsion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 33 task aware New</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>[DEBUG] Task 7 -&gt; Expert 2
-[DEBUG] Task-expert mapping: [1, 1, 1, 2, 1, 3, 2]
+[DEBUG] Task-expert mapping: [1, 1, 1, 2, 3, 2, 2]
 [DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 33 task aware random version</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[DEBUG] Task 7 -&gt; Expert 2
+[DEBUG] Task-expert mapping: [1, 1, 1, 2, 2, 3, 2]
+[DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 33 t_Agnostic random version</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -380,6 +394,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -405,12 +425,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -693,7 +707,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:T362"/>
+  <dimension ref="C3:AC362"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="18.625" customWidth="1"/>
@@ -706,16 +720,16 @@
   <sheetData>
     <row r="3" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="5"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="7"/>
     </row>
     <row r="5" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C5" s="2" t="s">
@@ -912,16 +926,16 @@
     </row>
     <row r="22" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="5"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="7"/>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C24" s="2" t="s">
@@ -1118,16 +1132,16 @@
     </row>
     <row r="38" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="5"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="7"/>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C40" s="2" t="s">
@@ -1324,16 +1338,16 @@
     </row>
     <row r="54" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="5"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="7"/>
     </row>
     <row r="56" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C56" s="2" t="s">
@@ -1530,16 +1544,16 @@
     </row>
     <row r="69" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="70" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
-      <c r="J70" s="5"/>
+      <c r="D70" s="6"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6"/>
+      <c r="H70" s="6"/>
+      <c r="I70" s="6"/>
+      <c r="J70" s="7"/>
     </row>
     <row r="71" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C71" s="2" t="s">
@@ -1736,16 +1750,16 @@
     </row>
     <row r="85" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="86" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="3" t="s">
+      <c r="C86" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D86" s="4"/>
-      <c r="E86" s="4"/>
-      <c r="F86" s="4"/>
-      <c r="G86" s="4"/>
-      <c r="H86" s="4"/>
-      <c r="I86" s="4"/>
-      <c r="J86" s="5"/>
+      <c r="D86" s="6"/>
+      <c r="E86" s="6"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="6"/>
+      <c r="H86" s="6"/>
+      <c r="I86" s="6"/>
+      <c r="J86" s="7"/>
     </row>
     <row r="87" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C87" s="2" t="s">
@@ -1942,16 +1956,16 @@
     </row>
     <row r="106" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="107" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C107" s="3" t="s">
+      <c r="C107" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D107" s="4"/>
-      <c r="E107" s="4"/>
-      <c r="F107" s="4"/>
-      <c r="G107" s="4"/>
-      <c r="H107" s="4"/>
-      <c r="I107" s="4"/>
-      <c r="J107" s="5"/>
+      <c r="D107" s="6"/>
+      <c r="E107" s="6"/>
+      <c r="F107" s="6"/>
+      <c r="G107" s="6"/>
+      <c r="H107" s="6"/>
+      <c r="I107" s="6"/>
+      <c r="J107" s="7"/>
     </row>
     <row r="108" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C108" s="2" t="s">
@@ -2148,16 +2162,16 @@
     </row>
     <row r="122" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="123" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C123" s="3" t="s">
+      <c r="C123" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D123" s="4"/>
-      <c r="E123" s="4"/>
-      <c r="F123" s="4"/>
-      <c r="G123" s="4"/>
-      <c r="H123" s="4"/>
-      <c r="I123" s="4"/>
-      <c r="J123" s="5"/>
+      <c r="D123" s="6"/>
+      <c r="E123" s="6"/>
+      <c r="F123" s="6"/>
+      <c r="G123" s="6"/>
+      <c r="H123" s="6"/>
+      <c r="I123" s="6"/>
+      <c r="J123" s="7"/>
     </row>
     <row r="124" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C124" s="2" t="s">
@@ -2354,16 +2368,16 @@
     </row>
     <row r="138" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="139" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C139" s="3" t="s">
+      <c r="C139" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D139" s="4"/>
-      <c r="E139" s="4"/>
-      <c r="F139" s="4"/>
-      <c r="G139" s="4"/>
-      <c r="H139" s="4"/>
-      <c r="I139" s="4"/>
-      <c r="J139" s="5"/>
+      <c r="D139" s="6"/>
+      <c r="E139" s="6"/>
+      <c r="F139" s="6"/>
+      <c r="G139" s="6"/>
+      <c r="H139" s="6"/>
+      <c r="I139" s="6"/>
+      <c r="J139" s="7"/>
     </row>
     <row r="140" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C140" s="2" t="s">
@@ -2560,16 +2574,16 @@
     </row>
     <row r="153" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="154" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C154" s="3" t="s">
+      <c r="C154" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D154" s="4"/>
-      <c r="E154" s="4"/>
-      <c r="F154" s="4"/>
-      <c r="G154" s="4"/>
-      <c r="H154" s="4"/>
-      <c r="I154" s="4"/>
-      <c r="J154" s="5"/>
+      <c r="D154" s="6"/>
+      <c r="E154" s="6"/>
+      <c r="F154" s="6"/>
+      <c r="G154" s="6"/>
+      <c r="H154" s="6"/>
+      <c r="I154" s="6"/>
+      <c r="J154" s="7"/>
     </row>
     <row r="155" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C155" s="2" t="s">
@@ -2766,16 +2780,16 @@
     </row>
     <row r="168" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="169" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C169" s="3" t="s">
+      <c r="C169" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D169" s="4"/>
-      <c r="E169" s="4"/>
-      <c r="F169" s="4"/>
-      <c r="G169" s="4"/>
-      <c r="H169" s="4"/>
-      <c r="I169" s="4"/>
-      <c r="J169" s="5"/>
+      <c r="D169" s="6"/>
+      <c r="E169" s="6"/>
+      <c r="F169" s="6"/>
+      <c r="G169" s="6"/>
+      <c r="H169" s="6"/>
+      <c r="I169" s="6"/>
+      <c r="J169" s="7"/>
     </row>
     <row r="170" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C170" s="2" t="s">
@@ -2972,16 +2986,16 @@
     </row>
     <row r="183" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="184" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C184" s="3" t="s">
+      <c r="C184" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D184" s="4"/>
-      <c r="E184" s="4"/>
-      <c r="F184" s="4"/>
-      <c r="G184" s="4"/>
-      <c r="H184" s="4"/>
-      <c r="I184" s="4"/>
-      <c r="J184" s="5"/>
+      <c r="D184" s="6"/>
+      <c r="E184" s="6"/>
+      <c r="F184" s="6"/>
+      <c r="G184" s="6"/>
+      <c r="H184" s="6"/>
+      <c r="I184" s="6"/>
+      <c r="J184" s="7"/>
     </row>
     <row r="185" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C185" s="2" t="s">
@@ -3177,51 +3191,61 @@
     </row>
     <row r="202" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="203" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C203" s="6" t="s">
+      <c r="C203" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D203" s="7"/>
-      <c r="E203" s="7"/>
-      <c r="F203" s="7"/>
-      <c r="G203" s="7"/>
-      <c r="H203" s="7"/>
-      <c r="I203" s="7"/>
-      <c r="J203" s="8"/>
+      <c r="D203" s="9"/>
+      <c r="E203" s="9"/>
+      <c r="F203" s="9"/>
+      <c r="G203" s="9"/>
+      <c r="H203" s="9"/>
+      <c r="I203" s="9"/>
+      <c r="J203" s="10"/>
     </row>
     <row r="204" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C204" s="9"/>
-      <c r="D204" s="10"/>
-      <c r="E204" s="10"/>
-      <c r="F204" s="10"/>
-      <c r="G204" s="10"/>
-      <c r="H204" s="10"/>
-      <c r="I204" s="10"/>
-      <c r="J204" s="11"/>
+      <c r="C204" s="11"/>
+      <c r="D204" s="12"/>
+      <c r="E204" s="12"/>
+      <c r="F204" s="12"/>
+      <c r="G204" s="12"/>
+      <c r="H204" s="12"/>
+      <c r="I204" s="12"/>
+      <c r="J204" s="13"/>
     </row>
     <row r="208" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C209" s="3" t="s">
+    <row r="209" spans="3:29" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C209" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D209" s="4"/>
-      <c r="E209" s="4"/>
-      <c r="F209" s="4"/>
-      <c r="G209" s="4"/>
-      <c r="H209" s="4"/>
-      <c r="I209" s="4"/>
-      <c r="J209" s="5"/>
-      <c r="M209" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="N209" s="4"/>
-      <c r="O209" s="4"/>
-      <c r="P209" s="4"/>
-      <c r="Q209" s="4"/>
-      <c r="R209" s="4"/>
-      <c r="S209" s="4"/>
-      <c r="T209" s="5"/>
-    </row>
-    <row r="210" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="D209" s="6"/>
+      <c r="E209" s="6"/>
+      <c r="F209" s="6"/>
+      <c r="G209" s="6"/>
+      <c r="H209" s="6"/>
+      <c r="I209" s="6"/>
+      <c r="J209" s="7"/>
+      <c r="M209" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="N209" s="6"/>
+      <c r="O209" s="6"/>
+      <c r="P209" s="6"/>
+      <c r="Q209" s="6"/>
+      <c r="R209" s="6"/>
+      <c r="S209" s="6"/>
+      <c r="T209" s="7"/>
+      <c r="V209" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="W209" s="6"/>
+      <c r="X209" s="6"/>
+      <c r="Y209" s="6"/>
+      <c r="Z209" s="6"/>
+      <c r="AA209" s="6"/>
+      <c r="AB209" s="6"/>
+      <c r="AC209" s="7"/>
+    </row>
+    <row r="210" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C210" s="2" t="s">
         <v>0</v>
       </c>
@@ -3270,8 +3294,32 @@
       <c r="T210" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="211" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V210" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W210" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X210" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y210" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z210" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA210" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AB210" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC210" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="211" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C211" s="1" t="s">
         <v>1</v>
       </c>
@@ -3288,7 +3336,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="1">
-        <v>96.794871794871796</v>
+        <v>96.624599358974294</v>
       </c>
       <c r="O211" s="1"/>
       <c r="P211" s="1"/>
@@ -3296,8 +3344,20 @@
       <c r="R211" s="1"/>
       <c r="S211" s="1"/>
       <c r="T211" s="1"/>
-    </row>
-    <row r="212" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V211" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="W211" s="1">
+        <v>96.694711538461505</v>
+      </c>
+      <c r="X211" s="1"/>
+      <c r="Y211" s="1"/>
+      <c r="Z211" s="1"/>
+      <c r="AA211" s="1"/>
+      <c r="AB211" s="1"/>
+      <c r="AC211" s="1"/>
+    </row>
+    <row r="212" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C212" s="1" t="s">
         <v>2</v>
       </c>
@@ -3316,18 +3376,32 @@
         <v>2</v>
       </c>
       <c r="N212" s="1">
-        <v>95.883413461538396</v>
+        <v>96.153846153846104</v>
       </c>
       <c r="O212" s="1">
-        <v>85.917467948717899</v>
+        <v>86.478365384615302</v>
       </c>
       <c r="P212" s="1"/>
       <c r="Q212" s="1"/>
       <c r="R212" s="1"/>
       <c r="S212" s="1"/>
       <c r="T212" s="1"/>
-    </row>
-    <row r="213" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V212" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="W212" s="1">
+        <v>96.043669871794805</v>
+      </c>
+      <c r="X212" s="1">
+        <v>86.668669871794805</v>
+      </c>
+      <c r="Y212" s="1"/>
+      <c r="Z212" s="1"/>
+      <c r="AA212" s="1"/>
+      <c r="AB212" s="1"/>
+      <c r="AC212" s="1"/>
+    </row>
+    <row r="213" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C213" s="1" t="s">
         <v>3</v>
       </c>
@@ -3347,19 +3421,34 @@
         <v>3</v>
       </c>
       <c r="N213" s="1">
-        <v>95.252403846153797</v>
+        <v>95.913461538461505</v>
       </c>
       <c r="O213" s="1">
-        <v>85.637019230769198</v>
+        <v>86.177884615384599</v>
       </c>
       <c r="P213" s="1">
-        <v>96.689723320158095</v>
+        <v>96.541501976284493</v>
       </c>
       <c r="R213" s="1"/>
       <c r="S213" s="1"/>
       <c r="T213" s="1"/>
-    </row>
-    <row r="214" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V213" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W213" s="1">
+        <v>95.773237179487097</v>
+      </c>
+      <c r="X213" s="1">
+        <v>85.777243589743506</v>
+      </c>
+      <c r="Y213" s="1">
+        <v>96.343873517786506</v>
+      </c>
+      <c r="AA213" s="1"/>
+      <c r="AB213" s="1"/>
+      <c r="AC213" s="1"/>
+    </row>
+    <row r="214" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C214" s="1" t="s">
         <v>4</v>
       </c>
@@ -3382,22 +3471,40 @@
         <v>4</v>
       </c>
       <c r="N214" s="1">
-        <v>94.340945512820497</v>
+        <v>94.901842948717899</v>
       </c>
       <c r="O214" s="1">
-        <v>83.954326923076906</v>
+        <v>83.974358974358907</v>
       </c>
       <c r="P214" s="1">
-        <v>95.615118577075094</v>
+        <v>95.973320158102695</v>
       </c>
       <c r="Q214" s="1">
-        <v>79.328208556149704</v>
+        <v>78.058155080213893</v>
       </c>
       <c r="R214" s="1"/>
       <c r="S214" s="1"/>
       <c r="T214" s="1"/>
-    </row>
-    <row r="215" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V214" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W214" s="1">
+        <v>94.170673076922995</v>
+      </c>
+      <c r="X214" s="1">
+        <v>83.693910256410206</v>
+      </c>
+      <c r="Y214" s="1">
+        <v>95.269268774703505</v>
+      </c>
+      <c r="Z214" s="1">
+        <v>78.893716577540104</v>
+      </c>
+      <c r="AA214" s="1"/>
+      <c r="AB214" s="1"/>
+      <c r="AC214" s="1"/>
+    </row>
+    <row r="215" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C215" s="1" t="s">
         <v>5</v>
       </c>
@@ -3422,24 +3529,44 @@
         <v>5</v>
       </c>
       <c r="N215" s="1">
-        <v>94.491185897435898</v>
+        <v>94.801682692307693</v>
       </c>
       <c r="O215" s="1">
-        <v>83.092948717948701</v>
+        <v>83.343349358974294</v>
       </c>
       <c r="P215">
-        <v>94.503458498023704</v>
+        <v>95.664525691699595</v>
       </c>
       <c r="Q215" s="1">
-        <v>76.353609625668398</v>
+        <v>75.167112299465202</v>
       </c>
       <c r="R215" s="1">
-        <v>85.226362179487097</v>
+        <v>85.056089743589695</v>
       </c>
       <c r="S215" s="1"/>
       <c r="T215" s="1"/>
-    </row>
-    <row r="216" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V215" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="W215" s="1">
+        <v>94.651442307692307</v>
+      </c>
+      <c r="X215" s="1">
+        <v>83.563701923076906</v>
+      </c>
+      <c r="Y215">
+        <v>93.947628458498002</v>
+      </c>
+      <c r="Z215" s="1">
+        <v>75.601604278074802</v>
+      </c>
+      <c r="AA215" s="1">
+        <v>85.016025641025607</v>
+      </c>
+      <c r="AB215" s="1"/>
+      <c r="AC215" s="1"/>
+    </row>
+    <row r="216" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C216" s="1" t="s">
         <v>6</v>
       </c>
@@ -3466,26 +3593,48 @@
         <v>6</v>
       </c>
       <c r="N216" s="1">
-        <v>93.459535256410206</v>
+        <v>94.220753205128204</v>
       </c>
       <c r="O216" s="1">
-        <v>81.951121794871796</v>
+        <v>82.171474358974294</v>
       </c>
       <c r="P216" s="1">
-        <v>92.243083003952506</v>
+        <v>94.7751976284585</v>
       </c>
       <c r="Q216" s="1">
-        <v>75.150401069518693</v>
+        <v>73.328877005347593</v>
       </c>
       <c r="R216" s="1">
-        <v>84.685496794871796</v>
+        <v>84.425080128205096</v>
       </c>
       <c r="S216" s="1">
-        <v>90.784438775510196</v>
+        <v>91.645408163265301</v>
       </c>
       <c r="T216" s="1"/>
-    </row>
-    <row r="217" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V216" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="W216" s="1">
+        <v>93.139022435897402</v>
+      </c>
+      <c r="X216" s="1">
+        <v>82.982772435897402</v>
+      </c>
+      <c r="Y216" s="1">
+        <v>93.070652173913004</v>
+      </c>
+      <c r="Z216" s="1">
+        <v>75.033422459893004</v>
+      </c>
+      <c r="AA216" s="1">
+        <v>84.785657051282001</v>
+      </c>
+      <c r="AB216" s="1">
+        <v>92.346938775510196</v>
+      </c>
+      <c r="AC216" s="1"/>
+    </row>
+    <row r="217" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C217" s="1" t="s">
         <v>7</v>
       </c>
@@ -3514,28 +3663,52 @@
         <v>7</v>
       </c>
       <c r="N217" s="1">
-        <v>94.080528846153797</v>
+        <v>94.501201923076906</v>
       </c>
       <c r="O217" s="1">
-        <v>82.171474358974294</v>
+        <v>82.341746794871796</v>
       </c>
       <c r="P217" s="1">
-        <v>91.983695652173907</v>
+        <v>95.1333992094861</v>
       </c>
       <c r="Q217" s="1">
-        <v>75.250668449197804</v>
+        <v>73.813502673796705</v>
       </c>
       <c r="R217" s="1">
-        <v>84.715544871794805</v>
+        <v>84.465144230769198</v>
       </c>
       <c r="S217" s="1">
-        <v>90.832270408163197</v>
+        <v>91.103316326530603</v>
       </c>
       <c r="T217" s="1">
-        <v>58.6805555555555</v>
-      </c>
-    </row>
-    <row r="219" spans="3:20" x14ac:dyDescent="0.2">
+        <v>55.0347222222222</v>
+      </c>
+      <c r="V217" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="W217" s="1">
+        <v>94.050480769230703</v>
+      </c>
+      <c r="X217" s="1">
+        <v>82.902644230769198</v>
+      </c>
+      <c r="Y217" s="1">
+        <v>93.169466403162005</v>
+      </c>
+      <c r="Z217" s="1">
+        <v>74.983288770053406</v>
+      </c>
+      <c r="AA217" s="1">
+        <v>84.835737179487097</v>
+      </c>
+      <c r="AB217" s="1">
+        <v>92.155612244897895</v>
+      </c>
+      <c r="AC217" s="1">
+        <v>59.5486111111111</v>
+      </c>
+    </row>
+    <row r="219" spans="3:29" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C219" t="s">
         <v>8</v>
       </c>
@@ -3548,17 +3721,31 @@
       </c>
       <c r="N219">
         <f>AVERAGE(N217:T217)</f>
-        <v>82.530676877430466</v>
-      </c>
-      <c r="P219" s="12" t="s">
+        <v>82.341861911536199</v>
+      </c>
+      <c r="P219" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="Q219" s="12"/>
-      <c r="R219" s="12"/>
-      <c r="S219" s="12"/>
-      <c r="T219" s="12"/>
-    </row>
-    <row r="220" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="Q219" s="3"/>
+      <c r="R219" s="3"/>
+      <c r="S219" s="3"/>
+      <c r="T219" s="3"/>
+      <c r="V219" t="s">
+        <v>8</v>
+      </c>
+      <c r="W219">
+        <f>AVERAGE(W217:AC217)</f>
+        <v>83.092262958387337</v>
+      </c>
+      <c r="Y219" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z219" s="3"/>
+      <c r="AA219" s="3"/>
+      <c r="AB219" s="3"/>
+      <c r="AC219" s="3"/>
+    </row>
+    <row r="220" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C220" t="s">
         <v>9</v>
       </c>
@@ -3571,15 +3758,27 @@
       </c>
       <c r="N220">
         <f>(SUM((N217-N211)+(O217-O212)+(P217-P213)+(Q217-Q214)+(R217-R215)+(S217-S216)))/6</f>
-        <v>-2.6178149980728307</v>
-      </c>
-      <c r="P220" s="12"/>
-      <c r="Q220" s="12"/>
-      <c r="R220" s="12"/>
-      <c r="S220" s="12"/>
-      <c r="T220" s="12"/>
-    </row>
-    <row r="221" spans="3:20" x14ac:dyDescent="0.2">
+        <v>-2.1743014247352783</v>
+      </c>
+      <c r="P220" s="3"/>
+      <c r="Q220" s="3"/>
+      <c r="R220" s="3"/>
+      <c r="S220" s="3"/>
+      <c r="T220" s="3"/>
+      <c r="V220" t="s">
+        <v>9</v>
+      </c>
+      <c r="W220">
+        <f>(SUM((W217-W211)+(X217-X212)+(Y217-Y213)+(Z217-Z214)+(AA217-AA215)+(AB217-AB216)))/6</f>
+        <v>-2.3111177207530695</v>
+      </c>
+      <c r="Y220" s="3"/>
+      <c r="Z220" s="3"/>
+      <c r="AA220" s="3"/>
+      <c r="AB220" s="3"/>
+      <c r="AC220" s="3"/>
+    </row>
+    <row r="221" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C221" t="s">
         <v>10</v>
       </c>
@@ -3592,43 +3791,60 @@
       </c>
       <c r="N221">
         <f>SUM((MAX(N211:N217)-N217)+(MAX(O212:O217)-O217)+(MAX(P213:P217)-P217)+(MAX(Q214:Q217)-Q217)+(MAX(R215:R217)-R217)+(MAX(S216:S217)-S217))/6</f>
-        <v>2.6257869368483306</v>
-      </c>
-      <c r="P221" s="12"/>
-      <c r="Q221" s="12"/>
-      <c r="R221" s="12"/>
-      <c r="S221" s="12"/>
-      <c r="T221" s="12"/>
-    </row>
-    <row r="222" spans="3:20" x14ac:dyDescent="0.2">
-      <c r="P222" s="12"/>
-      <c r="Q222" s="12"/>
-      <c r="R222" s="12"/>
-      <c r="S222" s="12"/>
-      <c r="T222" s="12"/>
+        <v>2.1743014247352783</v>
+      </c>
+      <c r="P221" s="3"/>
+      <c r="Q221" s="3"/>
+      <c r="R221" s="3"/>
+      <c r="S221" s="3"/>
+      <c r="T221" s="3"/>
+      <c r="V221" t="s">
+        <v>10</v>
+      </c>
+      <c r="W221">
+        <f>SUM((MAX(W211:W217)-W217)+(MAX(X212:X217)-X217)+(MAX(Y213:Y217)-Y217)+(MAX(Z214:Z217)-Z217)+(MAX(AA215:AA217)-AA217)+(MAX(AB216:AB217)-AB217))/6</f>
+        <v>2.3111177207530695</v>
+      </c>
+      <c r="Y221" s="3"/>
+      <c r="Z221" s="3"/>
+      <c r="AA221" s="3"/>
+      <c r="AB221" s="3"/>
+      <c r="AC221" s="3"/>
+    </row>
+    <row r="222" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="P222" s="3"/>
+      <c r="Q222" s="3"/>
+      <c r="R222" s="3"/>
+      <c r="S222" s="3"/>
+      <c r="T222" s="3"/>
+      <c r="Y222" s="3"/>
+      <c r="Z222" s="3"/>
+      <c r="AA222" s="3"/>
+      <c r="AB222" s="3"/>
+      <c r="AC222" s="3"/>
     </row>
     <row r="225" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="226" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C226" s="3" t="s">
+      <c r="C226" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D226" s="4"/>
-      <c r="E226" s="4"/>
-      <c r="F226" s="4"/>
-      <c r="G226" s="4"/>
-      <c r="H226" s="4"/>
-      <c r="I226" s="4"/>
-      <c r="J226" s="5"/>
-      <c r="M226" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="N226" s="4"/>
-      <c r="O226" s="4"/>
-      <c r="P226" s="4"/>
-      <c r="Q226" s="4"/>
-      <c r="R226" s="4"/>
-      <c r="S226" s="4"/>
-      <c r="T226" s="5"/>
+      <c r="D226" s="6"/>
+      <c r="E226" s="6"/>
+      <c r="F226" s="6"/>
+      <c r="G226" s="6"/>
+      <c r="H226" s="6"/>
+      <c r="I226" s="6"/>
+      <c r="J226" s="7"/>
+      <c r="M226" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N226" s="6"/>
+      <c r="O226" s="6"/>
+      <c r="P226" s="6"/>
+      <c r="Q226" s="6"/>
+      <c r="R226" s="6"/>
+      <c r="S226" s="6"/>
+      <c r="T226" s="7"/>
     </row>
     <row r="227" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C227" s="2" t="s">
@@ -3992,30 +4208,40 @@
         <v>2.0908121676384162</v>
       </c>
     </row>
-    <row r="241" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C242" s="3" t="s">
+    <row r="241" spans="3:29" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="3:29" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C242" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D242" s="4"/>
-      <c r="E242" s="4"/>
-      <c r="F242" s="4"/>
-      <c r="G242" s="4"/>
-      <c r="H242" s="4"/>
-      <c r="I242" s="4"/>
-      <c r="J242" s="5"/>
-      <c r="M242" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N242" s="4"/>
-      <c r="O242" s="4"/>
-      <c r="P242" s="4"/>
-      <c r="Q242" s="4"/>
-      <c r="R242" s="4"/>
-      <c r="S242" s="4"/>
-      <c r="T242" s="5"/>
-    </row>
-    <row r="243" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="D242" s="6"/>
+      <c r="E242" s="6"/>
+      <c r="F242" s="6"/>
+      <c r="G242" s="6"/>
+      <c r="H242" s="6"/>
+      <c r="I242" s="6"/>
+      <c r="J242" s="7"/>
+      <c r="M242" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="N242" s="6"/>
+      <c r="O242" s="6"/>
+      <c r="P242" s="6"/>
+      <c r="Q242" s="6"/>
+      <c r="R242" s="6"/>
+      <c r="S242" s="6"/>
+      <c r="T242" s="7"/>
+      <c r="V242" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="W242" s="6"/>
+      <c r="X242" s="6"/>
+      <c r="Y242" s="6"/>
+      <c r="Z242" s="6"/>
+      <c r="AA242" s="6"/>
+      <c r="AB242" s="6"/>
+      <c r="AC242" s="7"/>
+    </row>
+    <row r="243" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C243" s="2" t="s">
         <v>0</v>
       </c>
@@ -4064,8 +4290,32 @@
       <c r="T243" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="244" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V243" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W243" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X243" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y243" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z243" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA243" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AB243" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC243" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="244" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C244" s="1" t="s">
         <v>1</v>
       </c>
@@ -4090,8 +4340,20 @@
       <c r="R244" s="1"/>
       <c r="S244" s="1"/>
       <c r="T244" s="1"/>
-    </row>
-    <row r="245" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V244" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="W244" s="1">
+        <v>96.814903846153797</v>
+      </c>
+      <c r="X244" s="1"/>
+      <c r="Y244" s="1"/>
+      <c r="Z244" s="1"/>
+      <c r="AA244" s="1"/>
+      <c r="AB244" s="1"/>
+      <c r="AC244" s="1"/>
+    </row>
+    <row r="245" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C245" s="1" t="s">
         <v>2</v>
       </c>
@@ -4120,8 +4382,22 @@
       <c r="R245" s="1"/>
       <c r="S245" s="1"/>
       <c r="T245" s="1"/>
-    </row>
-    <row r="246" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V245" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="W245" s="1">
+        <v>96.564503205128204</v>
+      </c>
+      <c r="X245" s="1">
+        <v>86.488381410256395</v>
+      </c>
+      <c r="Y245" s="1"/>
+      <c r="Z245" s="1"/>
+      <c r="AA245" s="1"/>
+      <c r="AB245" s="1"/>
+      <c r="AC245" s="1"/>
+    </row>
+    <row r="246" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C246" s="1" t="s">
         <v>3</v>
       </c>
@@ -4152,8 +4428,23 @@
       <c r="R246" s="1"/>
       <c r="S246" s="1"/>
       <c r="T246" s="1"/>
-    </row>
-    <row r="247" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V246" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W246" s="1">
+        <v>96.113782051282001</v>
+      </c>
+      <c r="X246" s="1">
+        <v>85.456730769230703</v>
+      </c>
+      <c r="Y246" s="1">
+        <v>94.688735177865595</v>
+      </c>
+      <c r="AA246" s="1"/>
+      <c r="AB246" s="1"/>
+      <c r="AC246" s="1"/>
+    </row>
+    <row r="247" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C247" s="1" t="s">
         <v>4</v>
       </c>
@@ -4190,8 +4481,26 @@
       <c r="R247" s="1"/>
       <c r="S247" s="1"/>
       <c r="T247" s="1"/>
-    </row>
-    <row r="248" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V247" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W247" s="1">
+        <v>94.971955128205096</v>
+      </c>
+      <c r="X247">
+        <v>83.573717948717899</v>
+      </c>
+      <c r="Y247" s="1">
+        <v>94.849308300395194</v>
+      </c>
+      <c r="Z247" s="1">
+        <v>78.877005347593496</v>
+      </c>
+      <c r="AA247" s="1"/>
+      <c r="AB247" s="1"/>
+      <c r="AC247" s="1"/>
+    </row>
+    <row r="248" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C248" s="1" t="s">
         <v>5</v>
       </c>
@@ -4232,8 +4541,28 @@
       </c>
       <c r="S248" s="1"/>
       <c r="T248" s="1"/>
-    </row>
-    <row r="249" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V248" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="W248" s="1">
+        <v>95.252403846153797</v>
+      </c>
+      <c r="X248" s="1">
+        <v>83.573717948717899</v>
+      </c>
+      <c r="Y248">
+        <v>92.959486166007906</v>
+      </c>
+      <c r="Z248" s="1">
+        <v>75.451203208556095</v>
+      </c>
+      <c r="AA248" s="1">
+        <v>84.955929487179404</v>
+      </c>
+      <c r="AB248" s="1"/>
+      <c r="AC248" s="1"/>
+    </row>
+    <row r="249" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C249" s="1" t="s">
         <v>6</v>
       </c>
@@ -4278,8 +4607,30 @@
         <v>92.171556122448905</v>
       </c>
       <c r="T249" s="1"/>
-    </row>
-    <row r="250" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="V249" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="W249" s="1">
+        <v>94.100560897435898</v>
+      </c>
+      <c r="X249" s="1">
+        <v>82.702323717948701</v>
+      </c>
+      <c r="Y249" s="1">
+        <v>90.056818181818102</v>
+      </c>
+      <c r="Z249" s="1">
+        <v>74.699197860962499</v>
+      </c>
+      <c r="AA249" s="1">
+        <v>84.735576923076906</v>
+      </c>
+      <c r="AB249" s="1">
+        <v>92.857142857142804</v>
+      </c>
+      <c r="AC249" s="1"/>
+    </row>
+    <row r="250" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C250" s="1" t="s">
         <v>7</v>
       </c>
@@ -4328,8 +4679,32 @@
       <c r="T250" s="1">
         <v>60.9375</v>
       </c>
-    </row>
-    <row r="252" spans="3:20" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V250" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="W250" s="1">
+        <v>94.320913461538396</v>
+      </c>
+      <c r="X250" s="1">
+        <v>83.092948717948701</v>
+      </c>
+      <c r="Y250" s="1">
+        <v>90.180335968379396</v>
+      </c>
+      <c r="Z250" s="1">
+        <v>74.949866310160402</v>
+      </c>
+      <c r="AA250" s="1">
+        <v>84.5052083333333</v>
+      </c>
+      <c r="AB250" s="1">
+        <v>93.144132653061206</v>
+      </c>
+      <c r="AC250" s="1">
+        <v>57.8125</v>
+      </c>
+    </row>
+    <row r="252" spans="3:29" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C252" t="s">
         <v>8</v>
       </c>
@@ -4344,15 +4719,29 @@
         <f>AVERAGE(N250:T250)</f>
         <v>83.400848007784504</v>
       </c>
-      <c r="P252" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q252" s="12"/>
-      <c r="R252" s="12"/>
-      <c r="S252" s="12"/>
-      <c r="T252" s="12"/>
-    </row>
-    <row r="253" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="P252" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q252" s="3"/>
+      <c r="R252" s="3"/>
+      <c r="S252" s="3"/>
+      <c r="T252" s="3"/>
+      <c r="V252" t="s">
+        <v>8</v>
+      </c>
+      <c r="W252">
+        <f>AVERAGE(W250:AC250)</f>
+        <v>82.572272206345914</v>
+      </c>
+      <c r="Y252" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z252" s="3"/>
+      <c r="AA252" s="3"/>
+      <c r="AB252" s="3"/>
+      <c r="AC252" s="3"/>
+    </row>
+    <row r="253" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C253" t="s">
         <v>9</v>
       </c>
@@ -4367,13 +4756,25 @@
         <f>(SUM((N250-N244)+(O250-O245)+(P250-P246)+(Q250-Q247)+(R250-R248)+(S250-S249)))/6</f>
         <v>-2.0617011500049522</v>
       </c>
-      <c r="P253" s="12"/>
-      <c r="Q253" s="12"/>
-      <c r="R253" s="12"/>
-      <c r="S253" s="12"/>
-      <c r="T253" s="12"/>
-    </row>
-    <row r="254" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="P253" s="3"/>
+      <c r="Q253" s="3"/>
+      <c r="R253" s="3"/>
+      <c r="S253" s="3"/>
+      <c r="T253" s="3"/>
+      <c r="V253" t="s">
+        <v>9</v>
+      </c>
+      <c r="W253">
+        <f>(SUM((W250-W244)+(X250-X245)+(Y250-Y246)+(Z250-Z247)+(AA250-AA248)+(AB250-AB249)))/6</f>
+        <v>-2.4147821136283483</v>
+      </c>
+      <c r="Y253" s="3"/>
+      <c r="Z253" s="3"/>
+      <c r="AA253" s="3"/>
+      <c r="AB253" s="3"/>
+      <c r="AC253" s="3"/>
+    </row>
+    <row r="254" spans="3:29" x14ac:dyDescent="0.2">
       <c r="C254" t="s">
         <v>10</v>
       </c>
@@ -4388,31 +4789,48 @@
         <f>SUM((MAX(N244:N250)-N250)+(MAX(O245:O250)-O250)+(MAX(P246:P250)-P250)+(MAX(Q247:Q250)-Q250)+(MAX(R248:R250)-R250)+(MAX(S249:S250)-S250))/6</f>
         <v>2.0617011500049522</v>
       </c>
-      <c r="P254" s="12"/>
-      <c r="Q254" s="12"/>
-      <c r="R254" s="12"/>
-      <c r="S254" s="12"/>
-      <c r="T254" s="12"/>
-    </row>
-    <row r="255" spans="3:20" x14ac:dyDescent="0.2">
-      <c r="P255" s="12"/>
-      <c r="Q255" s="12"/>
-      <c r="R255" s="12"/>
-      <c r="S255" s="12"/>
-      <c r="T255" s="12"/>
+      <c r="P254" s="3"/>
+      <c r="Q254" s="3"/>
+      <c r="R254" s="3"/>
+      <c r="S254" s="3"/>
+      <c r="T254" s="3"/>
+      <c r="V254" t="s">
+        <v>10</v>
+      </c>
+      <c r="W254">
+        <f>SUM((MAX(W244:W250)-W250)+(MAX(X245:X250)-X250)+(MAX(Y246:Y250)-Y250)+(MAX(Z247:Z250)-Z250)+(MAX(AA248:AA250)-AA250)+(MAX(AB249:AB250)-AB250))/6</f>
+        <v>2.4893759333696814</v>
+      </c>
+      <c r="Y254" s="3"/>
+      <c r="Z254" s="3"/>
+      <c r="AA254" s="3"/>
+      <c r="AB254" s="3"/>
+      <c r="AC254" s="3"/>
+    </row>
+    <row r="255" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="P255" s="3"/>
+      <c r="Q255" s="3"/>
+      <c r="R255" s="3"/>
+      <c r="S255" s="3"/>
+      <c r="T255" s="3"/>
+      <c r="Y255" s="3"/>
+      <c r="Z255" s="3"/>
+      <c r="AA255" s="3"/>
+      <c r="AB255" s="3"/>
+      <c r="AC255" s="3"/>
     </row>
     <row r="267" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="268" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C268" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D268" s="4"/>
-      <c r="E268" s="4"/>
-      <c r="F268" s="4"/>
-      <c r="G268" s="4"/>
-      <c r="H268" s="4"/>
-      <c r="I268" s="4"/>
-      <c r="J268" s="5"/>
+      <c r="C268" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D268" s="6"/>
+      <c r="E268" s="6"/>
+      <c r="F268" s="6"/>
+      <c r="G268" s="6"/>
+      <c r="H268" s="6"/>
+      <c r="I268" s="6"/>
+      <c r="J268" s="7"/>
     </row>
     <row r="269" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C269" s="2" t="s">
@@ -4588,12 +5006,12 @@
         <f>AVERAGE(D276:J276)</f>
         <v>73.9583333333333</v>
       </c>
-      <c r="F278" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="G278" s="13"/>
-      <c r="H278" s="13"/>
-      <c r="I278" s="13"/>
+      <c r="F278" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G278" s="4"/>
+      <c r="H278" s="4"/>
+      <c r="I278" s="4"/>
     </row>
     <row r="279" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C279" t="s">
@@ -4603,10 +5021,10 @@
         <f>(SUM((D276-D270)+(E276-E271)+(F276-F272)+(G276-G273)+(H276-H274)+(I276-I275)))/6</f>
         <v>-0.17361111111111663</v>
       </c>
-      <c r="F279" s="13"/>
-      <c r="G279" s="13"/>
-      <c r="H279" s="13"/>
-      <c r="I279" s="13"/>
+      <c r="F279" s="4"/>
+      <c r="G279" s="4"/>
+      <c r="H279" s="4"/>
+      <c r="I279" s="4"/>
     </row>
     <row r="280" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C280" t="s">
@@ -4616,23 +5034,23 @@
         <f>SUM((MAX(D270:D276)-D276)+(MAX(E271:E276)-E276)+(MAX(F272:F276)-F276)+(MAX(G273:G276)-G276)+(MAX(H274:H276)-H276)+(MAX(I275:I276)-I276))/6</f>
         <v>1.9097222222222499</v>
       </c>
-      <c r="F280" s="13"/>
-      <c r="G280" s="13"/>
-      <c r="H280" s="13"/>
-      <c r="I280" s="13"/>
+      <c r="F280" s="4"/>
+      <c r="G280" s="4"/>
+      <c r="H280" s="4"/>
+      <c r="I280" s="4"/>
     </row>
     <row r="286" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="287" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C287" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D287" s="4"/>
-      <c r="E287" s="4"/>
-      <c r="F287" s="4"/>
-      <c r="G287" s="4"/>
-      <c r="H287" s="4"/>
-      <c r="I287" s="4"/>
-      <c r="J287" s="5"/>
+      <c r="C287" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D287" s="6"/>
+      <c r="E287" s="6"/>
+      <c r="F287" s="6"/>
+      <c r="G287" s="6"/>
+      <c r="H287" s="6"/>
+      <c r="I287" s="6"/>
+      <c r="J287" s="7"/>
     </row>
     <row r="288" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C288" s="2" t="s">
@@ -4808,12 +5226,12 @@
         <f>AVERAGE(D295:J295)</f>
         <v>64.5833333333333</v>
       </c>
-      <c r="F297" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="G297" s="13"/>
-      <c r="H297" s="13"/>
-      <c r="I297" s="13"/>
+      <c r="F297" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G297" s="4"/>
+      <c r="H297" s="4"/>
+      <c r="I297" s="4"/>
     </row>
     <row r="298" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C298" t="s">
@@ -4823,10 +5241,10 @@
         <f>(SUM((D295-D289)+(E295-E290)+(F295-F291)+(G295-G292)+(H295-H293)+(I295-I294)))/6</f>
         <v>-2.7777777777777835</v>
       </c>
-      <c r="F298" s="13"/>
-      <c r="G298" s="13"/>
-      <c r="H298" s="13"/>
-      <c r="I298" s="13"/>
+      <c r="F298" s="4"/>
+      <c r="G298" s="4"/>
+      <c r="H298" s="4"/>
+      <c r="I298" s="4"/>
     </row>
     <row r="299" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C299" t="s">
@@ -4836,23 +5254,23 @@
         <f>SUM((MAX(D289:D295)-D295)+(MAX(E290:E295)-E295)+(MAX(F291:F295)-F295)+(MAX(G292:G295)-G295)+(MAX(H293:H295)-H295)+(MAX(I294:I295)-I295))/6</f>
         <v>5.208333333333333</v>
       </c>
-      <c r="F299" s="13"/>
-      <c r="G299" s="13"/>
-      <c r="H299" s="13"/>
-      <c r="I299" s="13"/>
+      <c r="F299" s="4"/>
+      <c r="G299" s="4"/>
+      <c r="H299" s="4"/>
+      <c r="I299" s="4"/>
     </row>
     <row r="302" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="303" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C303" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D303" s="4"/>
-      <c r="E303" s="4"/>
-      <c r="F303" s="4"/>
-      <c r="G303" s="4"/>
-      <c r="H303" s="4"/>
-      <c r="I303" s="4"/>
-      <c r="J303" s="5"/>
+      <c r="C303" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D303" s="6"/>
+      <c r="E303" s="6"/>
+      <c r="F303" s="6"/>
+      <c r="G303" s="6"/>
+      <c r="H303" s="6"/>
+      <c r="I303" s="6"/>
+      <c r="J303" s="7"/>
     </row>
     <row r="304" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C304" s="2" t="s">
@@ -5017,7 +5435,7 @@
         <v>72.9166666666666</v>
       </c>
       <c r="J311" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="313" spans="3:10" x14ac:dyDescent="0.2">
@@ -5028,12 +5446,12 @@
         <f>AVERAGE(D311:J311)</f>
         <v>78.298611111111072</v>
       </c>
-      <c r="F313" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="G313" s="13"/>
-      <c r="H313" s="13"/>
-      <c r="I313" s="13"/>
+      <c r="F313" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G313" s="4"/>
+      <c r="H313" s="4"/>
+      <c r="I313" s="4"/>
     </row>
     <row r="314" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C314" t="s">
@@ -5043,10 +5461,10 @@
         <f>(SUM((D311-D305)+(E311-E306)+(F311-F307)+(G311-G308)+(H311-H309)+(I311-I310)))/6</f>
         <v>0.34722222222220012</v>
       </c>
-      <c r="F314" s="13"/>
-      <c r="G314" s="13"/>
-      <c r="H314" s="13"/>
-      <c r="I314" s="13"/>
+      <c r="F314" s="4"/>
+      <c r="G314" s="4"/>
+      <c r="H314" s="4"/>
+      <c r="I314" s="4"/>
     </row>
     <row r="315" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C315" t="s">
@@ -5056,23 +5474,23 @@
         <f>SUM((MAX(D305:D311)-D311)+(MAX(E306:E311)-E311)+(MAX(F307:F311)-F311)+(MAX(G308:G311)-G311)+(MAX(H309:H311)-H311)+(MAX(I310:I311)-I311))/6</f>
         <v>2.4305555555555665</v>
       </c>
-      <c r="F315" s="13"/>
-      <c r="G315" s="13"/>
-      <c r="H315" s="13"/>
-      <c r="I315" s="13"/>
+      <c r="F315" s="4"/>
+      <c r="G315" s="4"/>
+      <c r="H315" s="4"/>
+      <c r="I315" s="4"/>
     </row>
     <row r="318" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="319" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C319" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D319" s="4"/>
-      <c r="E319" s="4"/>
-      <c r="F319" s="4"/>
-      <c r="G319" s="4"/>
-      <c r="H319" s="4"/>
-      <c r="I319" s="4"/>
-      <c r="J319" s="5"/>
+      <c r="C319" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D319" s="6"/>
+      <c r="E319" s="6"/>
+      <c r="F319" s="6"/>
+      <c r="G319" s="6"/>
+      <c r="H319" s="6"/>
+      <c r="I319" s="6"/>
+      <c r="J319" s="7"/>
     </row>
     <row r="320" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C320" s="2" t="s">
@@ -5248,12 +5666,12 @@
         <f>AVERAGE(D327:J327)</f>
         <v>73.660714285714249</v>
       </c>
-      <c r="F329" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G329" s="13"/>
-      <c r="H329" s="13"/>
-      <c r="I329" s="13"/>
+      <c r="F329" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G329" s="4"/>
+      <c r="H329" s="4"/>
+      <c r="I329" s="4"/>
     </row>
     <row r="330" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C330" t="s">
@@ -5263,10 +5681,10 @@
         <f>(SUM((D327-D321)+(E327-E322)+(F327-F323)+(G327-G324)+(H327-H325)+(I327-I326)))/6</f>
         <v>-1.3888888888888999</v>
       </c>
-      <c r="F330" s="13"/>
-      <c r="G330" s="13"/>
-      <c r="H330" s="13"/>
-      <c r="I330" s="13"/>
+      <c r="F330" s="4"/>
+      <c r="G330" s="4"/>
+      <c r="H330" s="4"/>
+      <c r="I330" s="4"/>
     </row>
     <row r="331" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C331" t="s">
@@ -5276,23 +5694,23 @@
         <f>SUM((MAX(D321:D327)-D327)+(MAX(E322:E327)-E327)+(MAX(F323:F327)-F327)+(MAX(G324:G327)-G327)+(MAX(H325:H327)-H327)+(MAX(I326:I327)-I327))/6</f>
         <v>2.6041666666666665</v>
       </c>
-      <c r="F331" s="13"/>
-      <c r="G331" s="13"/>
-      <c r="H331" s="13"/>
-      <c r="I331" s="13"/>
+      <c r="F331" s="4"/>
+      <c r="G331" s="4"/>
+      <c r="H331" s="4"/>
+      <c r="I331" s="4"/>
     </row>
     <row r="333" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="334" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C334" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D334" s="4"/>
-      <c r="E334" s="4"/>
-      <c r="F334" s="4"/>
-      <c r="G334" s="4"/>
-      <c r="H334" s="4"/>
-      <c r="I334" s="4"/>
-      <c r="J334" s="5"/>
+      <c r="C334" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D334" s="6"/>
+      <c r="E334" s="6"/>
+      <c r="F334" s="6"/>
+      <c r="G334" s="6"/>
+      <c r="H334" s="6"/>
+      <c r="I334" s="6"/>
+      <c r="J334" s="7"/>
     </row>
     <row r="335" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C335" s="2" t="s">
@@ -5468,12 +5886,12 @@
         <f>AVERAGE(D342:J342)</f>
         <v>71.577380952380935</v>
       </c>
-      <c r="F344" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="G344" s="13"/>
-      <c r="H344" s="13"/>
-      <c r="I344" s="13"/>
+      <c r="F344" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G344" s="4"/>
+      <c r="H344" s="4"/>
+      <c r="I344" s="4"/>
     </row>
     <row r="345" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C345" t="s">
@@ -5483,10 +5901,10 @@
         <f>(SUM((D342-D336)+(E342-E337)+(F342-F338)+(G342-G339)+(H342-H340)+(I342-I341)))/6</f>
         <v>-1.0416666666666667</v>
       </c>
-      <c r="F345" s="13"/>
-      <c r="G345" s="13"/>
-      <c r="H345" s="13"/>
-      <c r="I345" s="13"/>
+      <c r="F345" s="4"/>
+      <c r="G345" s="4"/>
+      <c r="H345" s="4"/>
+      <c r="I345" s="4"/>
     </row>
     <row r="346" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C346" t="s">
@@ -5496,23 +5914,23 @@
         <f>SUM((MAX(D336:D342)-D342)+(MAX(E337:E342)-E342)+(MAX(F338:F342)-F342)+(MAX(G339:G342)-G342)+(MAX(H340:H342)-H342)+(MAX(I341:I342)-I342))/6</f>
         <v>2.6041666666666665</v>
       </c>
-      <c r="F346" s="13"/>
-      <c r="G346" s="13"/>
-      <c r="H346" s="13"/>
-      <c r="I346" s="13"/>
+      <c r="F346" s="4"/>
+      <c r="G346" s="4"/>
+      <c r="H346" s="4"/>
+      <c r="I346" s="4"/>
     </row>
     <row r="349" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="350" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C350" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D350" s="4"/>
-      <c r="E350" s="4"/>
-      <c r="F350" s="4"/>
-      <c r="G350" s="4"/>
-      <c r="H350" s="4"/>
-      <c r="I350" s="4"/>
-      <c r="J350" s="5"/>
+      <c r="C350" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D350" s="6"/>
+      <c r="E350" s="6"/>
+      <c r="F350" s="6"/>
+      <c r="G350" s="6"/>
+      <c r="H350" s="6"/>
+      <c r="I350" s="6"/>
+      <c r="J350" s="7"/>
     </row>
     <row r="351" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C351" s="2" t="s">
@@ -5684,12 +6102,12 @@
         <f>AVERAGE(D358:J358)</f>
         <v>67.261904761904731</v>
       </c>
-      <c r="F360" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="G360" s="13"/>
-      <c r="H360" s="13"/>
-      <c r="I360" s="13"/>
+      <c r="F360" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G360" s="4"/>
+      <c r="H360" s="4"/>
+      <c r="I360" s="4"/>
     </row>
     <row r="361" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C361" t="s">
@@ -5699,10 +6117,10 @@
         <f>(SUM((D358-D352)+(E358-E353)+(F358-F354)+(G358-G355)+(H358-H356)+(I358-I357)))/6</f>
         <v>-3.4722222222222334</v>
       </c>
-      <c r="F361" s="13"/>
-      <c r="G361" s="13"/>
-      <c r="H361" s="13"/>
-      <c r="I361" s="13"/>
+      <c r="F361" s="4"/>
+      <c r="G361" s="4"/>
+      <c r="H361" s="4"/>
+      <c r="I361" s="4"/>
     </row>
     <row r="362" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C362" t="s">
@@ -5712,13 +6130,39 @@
         <f>SUM((MAX(D352:D358)-D358)+(MAX(E353:E358)-E358)+(MAX(F355:F358)-F358)+(MAX(G355:G358)-G358)+(MAX(H356:H358)-H358)+(MAX(I357:I358)-I358))/6</f>
         <v>5.38194444444445</v>
       </c>
-      <c r="F362" s="13"/>
-      <c r="G362" s="13"/>
-      <c r="H362" s="13"/>
-      <c r="I362" s="13"/>
+      <c r="F362" s="4"/>
+      <c r="G362" s="4"/>
+      <c r="H362" s="4"/>
+      <c r="I362" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="37">
+    <mergeCell ref="V209:AC209"/>
+    <mergeCell ref="Y219:AC222"/>
+    <mergeCell ref="V242:AC242"/>
+    <mergeCell ref="Y252:AC255"/>
+    <mergeCell ref="C169:J169"/>
+    <mergeCell ref="C86:J86"/>
+    <mergeCell ref="C107:J107"/>
+    <mergeCell ref="C123:J123"/>
+    <mergeCell ref="C139:J139"/>
+    <mergeCell ref="C154:J154"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="C39:J39"/>
+    <mergeCell ref="C55:J55"/>
+    <mergeCell ref="C70:J70"/>
+    <mergeCell ref="C203:J204"/>
+    <mergeCell ref="C209:J209"/>
+    <mergeCell ref="C226:J226"/>
+    <mergeCell ref="C242:J242"/>
+    <mergeCell ref="C184:J184"/>
+    <mergeCell ref="M209:T209"/>
+    <mergeCell ref="M226:T226"/>
+    <mergeCell ref="M242:T242"/>
+    <mergeCell ref="C268:J268"/>
+    <mergeCell ref="C287:J287"/>
+    <mergeCell ref="P219:T222"/>
     <mergeCell ref="F360:I362"/>
     <mergeCell ref="P252:T255"/>
     <mergeCell ref="F344:I346"/>
@@ -5730,28 +6174,6 @@
     <mergeCell ref="F297:I299"/>
     <mergeCell ref="F313:I315"/>
     <mergeCell ref="F329:I331"/>
-    <mergeCell ref="M209:T209"/>
-    <mergeCell ref="M226:T226"/>
-    <mergeCell ref="M242:T242"/>
-    <mergeCell ref="C268:J268"/>
-    <mergeCell ref="C287:J287"/>
-    <mergeCell ref="P219:T222"/>
-    <mergeCell ref="C203:J204"/>
-    <mergeCell ref="C209:J209"/>
-    <mergeCell ref="C226:J226"/>
-    <mergeCell ref="C242:J242"/>
-    <mergeCell ref="C184:J184"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="C23:J23"/>
-    <mergeCell ref="C39:J39"/>
-    <mergeCell ref="C55:J55"/>
-    <mergeCell ref="C70:J70"/>
-    <mergeCell ref="C169:J169"/>
-    <mergeCell ref="C86:J86"/>
-    <mergeCell ref="C107:J107"/>
-    <mergeCell ref="C123:J123"/>
-    <mergeCell ref="C139:J139"/>
-    <mergeCell ref="C154:J154"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
finalise 1: finalise submission process (README and excel update)
</commit_message>
<xml_diff>
--- a/metrix_calculation.xlsx
+++ b/metrix_calculation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course\CS_764\project\NeurIPS2025-LEAR-main\csi764_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F642EBF6-C0DC-430C-A927-4AD23980B035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62AEFBEA-7190-478C-AAA8-8FD7EF2EF2ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -191,35 +191,35 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>t = 33 t_Agnostic New version</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>original New Version comparsion</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>t = 33 task aware New</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>[DEBUG] Task 7 -&gt; Expert 2
 [DEBUG] Task-expert mapping: [1, 1, 1, 2, 3, 2, 2]
 [DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>t = 33 task aware random version</t>
+    <t>t = 33 t_Agnostic Claude version 1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[DEBUG] Task 7 -&gt; Expert 2
-[DEBUG] Task-expert mapping: [1, 1, 1, 2, 2, 3, 2]
-[DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]</t>
+    <t>t = 33 t_Agnostic Claude version 2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>t = 33 t_Agnostic random version</t>
+    <t xml:space="preserve">[DEBUG] Task 7 -&gt; Expert 2
+[DEBUG] Task-expert mapping: [1, 1, 1, 2, 1, 3, 2]
+[DEBUG] Task-classifier mapping: [1, 2, 3, 4, 5, 6, 7]		</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>original Claude Version comparsion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 33 task aware Claude 1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t = 33 task aware Claude 2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -390,16 +390,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -408,6 +402,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -426,6 +423,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:AC362"/>
+  <dimension ref="C3:AD362"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="18.625" customWidth="1"/>
@@ -720,16 +723,16 @@
   <sheetData>
     <row r="3" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="7"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C5" s="2" t="s">
@@ -926,16 +929,16 @@
     </row>
     <row r="22" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="7"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="5"/>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C24" s="2" t="s">
@@ -1132,16 +1135,16 @@
     </row>
     <row r="38" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="7"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="5"/>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C40" s="2" t="s">
@@ -1338,16 +1341,16 @@
     </row>
     <row r="54" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6"/>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
-      <c r="I55" s="6"/>
-      <c r="J55" s="7"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+      <c r="H55" s="4"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="5"/>
     </row>
     <row r="56" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C56" s="2" t="s">
@@ -1544,16 +1547,16 @@
     </row>
     <row r="69" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="70" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="5" t="s">
+      <c r="C70" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D70" s="6"/>
-      <c r="E70" s="6"/>
-      <c r="F70" s="6"/>
-      <c r="G70" s="6"/>
-      <c r="H70" s="6"/>
-      <c r="I70" s="6"/>
-      <c r="J70" s="7"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+      <c r="H70" s="4"/>
+      <c r="I70" s="4"/>
+      <c r="J70" s="5"/>
     </row>
     <row r="71" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C71" s="2" t="s">
@@ -1750,16 +1753,16 @@
     </row>
     <row r="85" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="86" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="5" t="s">
+      <c r="C86" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D86" s="6"/>
-      <c r="E86" s="6"/>
-      <c r="F86" s="6"/>
-      <c r="G86" s="6"/>
-      <c r="H86" s="6"/>
-      <c r="I86" s="6"/>
-      <c r="J86" s="7"/>
+      <c r="D86" s="4"/>
+      <c r="E86" s="4"/>
+      <c r="F86" s="4"/>
+      <c r="G86" s="4"/>
+      <c r="H86" s="4"/>
+      <c r="I86" s="4"/>
+      <c r="J86" s="5"/>
     </row>
     <row r="87" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C87" s="2" t="s">
@@ -1956,16 +1959,16 @@
     </row>
     <row r="106" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="107" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C107" s="5" t="s">
+      <c r="C107" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D107" s="6"/>
-      <c r="E107" s="6"/>
-      <c r="F107" s="6"/>
-      <c r="G107" s="6"/>
-      <c r="H107" s="6"/>
-      <c r="I107" s="6"/>
-      <c r="J107" s="7"/>
+      <c r="D107" s="4"/>
+      <c r="E107" s="4"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="4"/>
+      <c r="H107" s="4"/>
+      <c r="I107" s="4"/>
+      <c r="J107" s="5"/>
     </row>
     <row r="108" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C108" s="2" t="s">
@@ -2162,16 +2165,16 @@
     </row>
     <row r="122" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="123" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C123" s="5" t="s">
+      <c r="C123" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D123" s="6"/>
-      <c r="E123" s="6"/>
-      <c r="F123" s="6"/>
-      <c r="G123" s="6"/>
-      <c r="H123" s="6"/>
-      <c r="I123" s="6"/>
-      <c r="J123" s="7"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
+      <c r="G123" s="4"/>
+      <c r="H123" s="4"/>
+      <c r="I123" s="4"/>
+      <c r="J123" s="5"/>
     </row>
     <row r="124" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C124" s="2" t="s">
@@ -2368,16 +2371,16 @@
     </row>
     <row r="138" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="139" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C139" s="5" t="s">
+      <c r="C139" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D139" s="6"/>
-      <c r="E139" s="6"/>
-      <c r="F139" s="6"/>
-      <c r="G139" s="6"/>
-      <c r="H139" s="6"/>
-      <c r="I139" s="6"/>
-      <c r="J139" s="7"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="4"/>
+      <c r="F139" s="4"/>
+      <c r="G139" s="4"/>
+      <c r="H139" s="4"/>
+      <c r="I139" s="4"/>
+      <c r="J139" s="5"/>
     </row>
     <row r="140" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C140" s="2" t="s">
@@ -2574,16 +2577,16 @@
     </row>
     <row r="153" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="154" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C154" s="5" t="s">
+      <c r="C154" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D154" s="6"/>
-      <c r="E154" s="6"/>
-      <c r="F154" s="6"/>
-      <c r="G154" s="6"/>
-      <c r="H154" s="6"/>
-      <c r="I154" s="6"/>
-      <c r="J154" s="7"/>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4"/>
+      <c r="F154" s="4"/>
+      <c r="G154" s="4"/>
+      <c r="H154" s="4"/>
+      <c r="I154" s="4"/>
+      <c r="J154" s="5"/>
     </row>
     <row r="155" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C155" s="2" t="s">
@@ -2780,16 +2783,16 @@
     </row>
     <row r="168" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="169" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C169" s="5" t="s">
+      <c r="C169" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D169" s="6"/>
-      <c r="E169" s="6"/>
-      <c r="F169" s="6"/>
-      <c r="G169" s="6"/>
-      <c r="H169" s="6"/>
-      <c r="I169" s="6"/>
-      <c r="J169" s="7"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="4"/>
+      <c r="H169" s="4"/>
+      <c r="I169" s="4"/>
+      <c r="J169" s="5"/>
     </row>
     <row r="170" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C170" s="2" t="s">
@@ -2986,16 +2989,16 @@
     </row>
     <row r="183" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="184" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C184" s="5" t="s">
+      <c r="C184" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D184" s="6"/>
-      <c r="E184" s="6"/>
-      <c r="F184" s="6"/>
-      <c r="G184" s="6"/>
-      <c r="H184" s="6"/>
-      <c r="I184" s="6"/>
-      <c r="J184" s="7"/>
+      <c r="D184" s="4"/>
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
+      <c r="G184" s="4"/>
+      <c r="H184" s="4"/>
+      <c r="I184" s="4"/>
+      <c r="J184" s="5"/>
     </row>
     <row r="185" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C185" s="2" t="s">
@@ -3191,61 +3194,61 @@
     </row>
     <row r="202" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="203" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C203" s="8" t="s">
+      <c r="C203" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D203" s="9"/>
-      <c r="E203" s="9"/>
-      <c r="F203" s="9"/>
-      <c r="G203" s="9"/>
-      <c r="H203" s="9"/>
-      <c r="I203" s="9"/>
-      <c r="J203" s="10"/>
+      <c r="D203" s="8"/>
+      <c r="E203" s="8"/>
+      <c r="F203" s="8"/>
+      <c r="G203" s="8"/>
+      <c r="H203" s="8"/>
+      <c r="I203" s="8"/>
+      <c r="J203" s="9"/>
     </row>
     <row r="204" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C204" s="11"/>
-      <c r="D204" s="12"/>
-      <c r="E204" s="12"/>
-      <c r="F204" s="12"/>
-      <c r="G204" s="12"/>
-      <c r="H204" s="12"/>
-      <c r="I204" s="12"/>
-      <c r="J204" s="13"/>
+      <c r="C204" s="10"/>
+      <c r="D204" s="11"/>
+      <c r="E204" s="11"/>
+      <c r="F204" s="11"/>
+      <c r="G204" s="11"/>
+      <c r="H204" s="11"/>
+      <c r="I204" s="11"/>
+      <c r="J204" s="12"/>
     </row>
     <row r="208" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="3:29" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C209" s="5" t="s">
+    <row r="209" spans="3:30" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C209" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D209" s="6"/>
-      <c r="E209" s="6"/>
-      <c r="F209" s="6"/>
-      <c r="G209" s="6"/>
-      <c r="H209" s="6"/>
-      <c r="I209" s="6"/>
-      <c r="J209" s="7"/>
-      <c r="M209" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="N209" s="6"/>
-      <c r="O209" s="6"/>
-      <c r="P209" s="6"/>
-      <c r="Q209" s="6"/>
-      <c r="R209" s="6"/>
-      <c r="S209" s="6"/>
-      <c r="T209" s="7"/>
-      <c r="V209" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="W209" s="6"/>
-      <c r="X209" s="6"/>
-      <c r="Y209" s="6"/>
-      <c r="Z209" s="6"/>
-      <c r="AA209" s="6"/>
-      <c r="AB209" s="6"/>
-      <c r="AC209" s="7"/>
-    </row>
-    <row r="210" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="D209" s="4"/>
+      <c r="E209" s="4"/>
+      <c r="F209" s="4"/>
+      <c r="G209" s="4"/>
+      <c r="H209" s="4"/>
+      <c r="I209" s="4"/>
+      <c r="J209" s="5"/>
+      <c r="M209" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="N209" s="4"/>
+      <c r="O209" s="4"/>
+      <c r="P209" s="4"/>
+      <c r="Q209" s="4"/>
+      <c r="R209" s="4"/>
+      <c r="S209" s="4"/>
+      <c r="T209" s="5"/>
+      <c r="W209" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="X209" s="4"/>
+      <c r="Y209" s="4"/>
+      <c r="Z209" s="4"/>
+      <c r="AA209" s="4"/>
+      <c r="AB209" s="4"/>
+      <c r="AC209" s="4"/>
+      <c r="AD209" s="5"/>
+    </row>
+    <row r="210" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C210" s="2" t="s">
         <v>0</v>
       </c>
@@ -3294,32 +3297,32 @@
       <c r="T210" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="V210" s="2" t="s">
+      <c r="W210" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="W210" s="2" t="s">
+      <c r="X210" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="X210" s="2" t="s">
+      <c r="Y210" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="Y210" s="2" t="s">
+      <c r="Z210" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="Z210" s="2" t="s">
+      <c r="AA210" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="AA210" s="2" t="s">
+      <c r="AB210" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="AB210" s="2" t="s">
+      <c r="AC210" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="AC210" s="2" t="s">
+      <c r="AD210" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="211" spans="3:29" x14ac:dyDescent="0.2">
+    <row r="211" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C211" s="1" t="s">
         <v>1</v>
       </c>
@@ -3336,7 +3339,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="1">
-        <v>96.624599358974294</v>
+        <v>96.794871794871796</v>
       </c>
       <c r="O211" s="1"/>
       <c r="P211" s="1"/>
@@ -3344,20 +3347,20 @@
       <c r="R211" s="1"/>
       <c r="S211" s="1"/>
       <c r="T211" s="1"/>
-      <c r="V211" s="1" t="s">
+      <c r="W211" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="W211" s="1">
-        <v>96.694711538461505</v>
-      </c>
-      <c r="X211" s="1"/>
+      <c r="X211" s="1">
+        <v>96.624599358974294</v>
+      </c>
       <c r="Y211" s="1"/>
       <c r="Z211" s="1"/>
       <c r="AA211" s="1"/>
       <c r="AB211" s="1"/>
       <c r="AC211" s="1"/>
-    </row>
-    <row r="212" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD211" s="1"/>
+    </row>
+    <row r="212" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C212" s="1" t="s">
         <v>2</v>
       </c>
@@ -3376,32 +3379,32 @@
         <v>2</v>
       </c>
       <c r="N212" s="1">
-        <v>96.153846153846104</v>
+        <v>95.883413461538396</v>
       </c>
       <c r="O212" s="1">
-        <v>86.478365384615302</v>
+        <v>85.917467948717899</v>
       </c>
       <c r="P212" s="1"/>
       <c r="Q212" s="1"/>
       <c r="R212" s="1"/>
       <c r="S212" s="1"/>
       <c r="T212" s="1"/>
-      <c r="V212" s="1" t="s">
+      <c r="W212" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="W212" s="1">
-        <v>96.043669871794805</v>
-      </c>
       <c r="X212" s="1">
-        <v>86.668669871794805</v>
-      </c>
-      <c r="Y212" s="1"/>
+        <v>96.153846153846104</v>
+      </c>
+      <c r="Y212" s="1">
+        <v>86.478365384615302</v>
+      </c>
       <c r="Z212" s="1"/>
       <c r="AA212" s="1"/>
       <c r="AB212" s="1"/>
       <c r="AC212" s="1"/>
-    </row>
-    <row r="213" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD212" s="1"/>
+    </row>
+    <row r="213" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C213" s="1" t="s">
         <v>3</v>
       </c>
@@ -3421,34 +3424,34 @@
         <v>3</v>
       </c>
       <c r="N213" s="1">
-        <v>95.913461538461505</v>
+        <v>95.252403846153797</v>
       </c>
       <c r="O213" s="1">
-        <v>86.177884615384599</v>
+        <v>85.637019230769198</v>
       </c>
       <c r="P213" s="1">
-        <v>96.541501976284493</v>
+        <v>96.689723320158095</v>
       </c>
       <c r="R213" s="1"/>
       <c r="S213" s="1"/>
       <c r="T213" s="1"/>
-      <c r="V213" s="1" t="s">
+      <c r="W213" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="W213" s="1">
-        <v>95.773237179487097</v>
-      </c>
       <c r="X213" s="1">
-        <v>85.777243589743506</v>
+        <v>95.913461538461505</v>
       </c>
       <c r="Y213" s="1">
-        <v>96.343873517786506</v>
-      </c>
-      <c r="AA213" s="1"/>
+        <v>86.177884615384599</v>
+      </c>
+      <c r="Z213" s="1">
+        <v>96.541501976284493</v>
+      </c>
       <c r="AB213" s="1"/>
       <c r="AC213" s="1"/>
-    </row>
-    <row r="214" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD213" s="1"/>
+    </row>
+    <row r="214" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C214" s="1" t="s">
         <v>4</v>
       </c>
@@ -3471,40 +3474,40 @@
         <v>4</v>
       </c>
       <c r="N214" s="1">
-        <v>94.901842948717899</v>
+        <v>94.340945512820497</v>
       </c>
       <c r="O214" s="1">
-        <v>83.974358974358907</v>
+        <v>83.954326923076906</v>
       </c>
       <c r="P214" s="1">
-        <v>95.973320158102695</v>
+        <v>95.615118577075094</v>
       </c>
       <c r="Q214" s="1">
-        <v>78.058155080213893</v>
+        <v>79.328208556149704</v>
       </c>
       <c r="R214" s="1"/>
       <c r="S214" s="1"/>
       <c r="T214" s="1"/>
-      <c r="V214" s="1" t="s">
+      <c r="W214" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="W214" s="1">
-        <v>94.170673076922995</v>
-      </c>
       <c r="X214" s="1">
-        <v>83.693910256410206</v>
+        <v>94.901842948717899</v>
       </c>
       <c r="Y214" s="1">
-        <v>95.269268774703505</v>
+        <v>83.974358974358907</v>
       </c>
       <c r="Z214" s="1">
-        <v>78.893716577540104</v>
-      </c>
-      <c r="AA214" s="1"/>
+        <v>95.973320158102695</v>
+      </c>
+      <c r="AA214" s="1">
+        <v>78.058155080213893</v>
+      </c>
       <c r="AB214" s="1"/>
       <c r="AC214" s="1"/>
-    </row>
-    <row r="215" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD214" s="1"/>
+    </row>
+    <row r="215" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C215" s="1" t="s">
         <v>5</v>
       </c>
@@ -3529,44 +3532,44 @@
         <v>5</v>
       </c>
       <c r="N215" s="1">
-        <v>94.801682692307693</v>
+        <v>94.491185897435898</v>
       </c>
       <c r="O215" s="1">
-        <v>83.343349358974294</v>
+        <v>83.092948717948701</v>
       </c>
       <c r="P215">
-        <v>95.664525691699595</v>
+        <v>94.503458498023704</v>
       </c>
       <c r="Q215" s="1">
-        <v>75.167112299465202</v>
+        <v>76.353609625668398</v>
       </c>
       <c r="R215" s="1">
-        <v>85.056089743589695</v>
+        <v>85.226362179487097</v>
       </c>
       <c r="S215" s="1"/>
       <c r="T215" s="1"/>
-      <c r="V215" s="1" t="s">
+      <c r="W215" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="W215" s="1">
-        <v>94.651442307692307</v>
-      </c>
       <c r="X215" s="1">
-        <v>83.563701923076906</v>
-      </c>
-      <c r="Y215">
-        <v>93.947628458498002</v>
-      </c>
-      <c r="Z215" s="1">
-        <v>75.601604278074802</v>
+        <v>94.801682692307693</v>
+      </c>
+      <c r="Y215" s="1">
+        <v>83.343349358974294</v>
+      </c>
+      <c r="Z215">
+        <v>95.664525691699595</v>
       </c>
       <c r="AA215" s="1">
-        <v>85.016025641025607</v>
-      </c>
-      <c r="AB215" s="1"/>
+        <v>75.167112299465202</v>
+      </c>
+      <c r="AB215" s="1">
+        <v>85.056089743589695</v>
+      </c>
       <c r="AC215" s="1"/>
-    </row>
-    <row r="216" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD215" s="1"/>
+    </row>
+    <row r="216" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C216" s="1" t="s">
         <v>6</v>
       </c>
@@ -3593,48 +3596,48 @@
         <v>6</v>
       </c>
       <c r="N216" s="1">
+        <v>93.459535256410206</v>
+      </c>
+      <c r="O216" s="1">
+        <v>81.951121794871796</v>
+      </c>
+      <c r="P216" s="1">
+        <v>92.243083003952506</v>
+      </c>
+      <c r="Q216" s="1">
+        <v>75.150401069518693</v>
+      </c>
+      <c r="R216" s="1">
+        <v>84.685496794871796</v>
+      </c>
+      <c r="S216" s="1">
+        <v>90.784438775510196</v>
+      </c>
+      <c r="T216" s="1"/>
+      <c r="W216" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="X216" s="1">
         <v>94.220753205128204</v>
       </c>
-      <c r="O216" s="1">
+      <c r="Y216" s="1">
         <v>82.171474358974294</v>
       </c>
-      <c r="P216" s="1">
+      <c r="Z216" s="1">
         <v>94.7751976284585</v>
       </c>
-      <c r="Q216" s="1">
+      <c r="AA216" s="1">
         <v>73.328877005347593</v>
       </c>
-      <c r="R216" s="1">
+      <c r="AB216" s="1">
         <v>84.425080128205096</v>
       </c>
-      <c r="S216" s="1">
+      <c r="AC216" s="1">
         <v>91.645408163265301</v>
       </c>
-      <c r="T216" s="1"/>
-      <c r="V216" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="W216" s="1">
-        <v>93.139022435897402</v>
-      </c>
-      <c r="X216" s="1">
-        <v>82.982772435897402</v>
-      </c>
-      <c r="Y216" s="1">
-        <v>93.070652173913004</v>
-      </c>
-      <c r="Z216" s="1">
-        <v>75.033422459893004</v>
-      </c>
-      <c r="AA216" s="1">
-        <v>84.785657051282001</v>
-      </c>
-      <c r="AB216" s="1">
-        <v>92.346938775510196</v>
-      </c>
-      <c r="AC216" s="1"/>
-    </row>
-    <row r="217" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD216" s="1"/>
+    </row>
+    <row r="217" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C217" s="1" t="s">
         <v>7</v>
       </c>
@@ -3663,52 +3666,52 @@
         <v>7</v>
       </c>
       <c r="N217" s="1">
+        <v>94.080528846153797</v>
+      </c>
+      <c r="O217" s="1">
+        <v>82.171474358974294</v>
+      </c>
+      <c r="P217" s="1">
+        <v>91.983695652173907</v>
+      </c>
+      <c r="Q217" s="1">
+        <v>75.250668449197804</v>
+      </c>
+      <c r="R217" s="1">
+        <v>84.715544871794805</v>
+      </c>
+      <c r="S217" s="1">
+        <v>90.832270408163197</v>
+      </c>
+      <c r="T217" s="1">
+        <v>58.6805555555555</v>
+      </c>
+      <c r="W217" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="X217" s="1">
         <v>94.501201923076906</v>
       </c>
-      <c r="O217" s="1">
+      <c r="Y217" s="1">
         <v>82.341746794871796</v>
       </c>
-      <c r="P217" s="1">
+      <c r="Z217" s="1">
         <v>95.1333992094861</v>
       </c>
-      <c r="Q217" s="1">
+      <c r="AA217" s="1">
         <v>73.813502673796705</v>
       </c>
-      <c r="R217" s="1">
+      <c r="AB217" s="1">
         <v>84.465144230769198</v>
       </c>
-      <c r="S217" s="1">
+      <c r="AC217" s="1">
         <v>91.103316326530603</v>
       </c>
-      <c r="T217" s="1">
+      <c r="AD217" s="1">
         <v>55.0347222222222</v>
       </c>
-      <c r="V217" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="W217" s="1">
-        <v>94.050480769230703</v>
-      </c>
-      <c r="X217" s="1">
-        <v>82.902644230769198</v>
-      </c>
-      <c r="Y217" s="1">
-        <v>93.169466403162005</v>
-      </c>
-      <c r="Z217" s="1">
-        <v>74.983288770053406</v>
-      </c>
-      <c r="AA217" s="1">
-        <v>84.835737179487097</v>
-      </c>
-      <c r="AB217" s="1">
-        <v>92.155612244897895</v>
-      </c>
-      <c r="AC217" s="1">
-        <v>59.5486111111111</v>
-      </c>
-    </row>
-    <row r="219" spans="3:29" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="219" spans="3:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C219" t="s">
         <v>8</v>
       </c>
@@ -3721,31 +3724,31 @@
       </c>
       <c r="N219">
         <f>AVERAGE(N217:T217)</f>
+        <v>82.530676877430466</v>
+      </c>
+      <c r="P219" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q219" s="6"/>
+      <c r="R219" s="6"/>
+      <c r="S219" s="6"/>
+      <c r="T219" s="6"/>
+      <c r="W219" t="s">
+        <v>8</v>
+      </c>
+      <c r="X219">
+        <f>AVERAGE(X217:AD217)</f>
         <v>82.341861911536199</v>
       </c>
-      <c r="P219" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q219" s="3"/>
-      <c r="R219" s="3"/>
-      <c r="S219" s="3"/>
-      <c r="T219" s="3"/>
-      <c r="V219" t="s">
-        <v>8</v>
-      </c>
-      <c r="W219">
-        <f>AVERAGE(W217:AC217)</f>
-        <v>83.092262958387337</v>
-      </c>
-      <c r="Y219" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Z219" s="3"/>
-      <c r="AA219" s="3"/>
-      <c r="AB219" s="3"/>
-      <c r="AC219" s="3"/>
-    </row>
-    <row r="220" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="Z219" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA219" s="6"/>
+      <c r="AB219" s="6"/>
+      <c r="AC219" s="6"/>
+      <c r="AD219" s="6"/>
+    </row>
+    <row r="220" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C220" t="s">
         <v>9</v>
       </c>
@@ -3758,27 +3761,27 @@
       </c>
       <c r="N220">
         <f>(SUM((N217-N211)+(O217-O212)+(P217-P213)+(Q217-Q214)+(R217-R215)+(S217-S216)))/6</f>
+        <v>-2.6178149980728307</v>
+      </c>
+      <c r="P220" s="6"/>
+      <c r="Q220" s="6"/>
+      <c r="R220" s="6"/>
+      <c r="S220" s="6"/>
+      <c r="T220" s="6"/>
+      <c r="W220" t="s">
+        <v>9</v>
+      </c>
+      <c r="X220">
+        <f>(SUM((X217-X211)+(Y217-Y212)+(Z217-Z213)+(AA217-AA214)+(AB217-AB215)+(AC217-AC216)))/6</f>
         <v>-2.1743014247352783</v>
       </c>
-      <c r="P220" s="3"/>
-      <c r="Q220" s="3"/>
-      <c r="R220" s="3"/>
-      <c r="S220" s="3"/>
-      <c r="T220" s="3"/>
-      <c r="V220" t="s">
-        <v>9</v>
-      </c>
-      <c r="W220">
-        <f>(SUM((W217-W211)+(X217-X212)+(Y217-Y213)+(Z217-Z214)+(AA217-AA215)+(AB217-AB216)))/6</f>
-        <v>-2.3111177207530695</v>
-      </c>
-      <c r="Y220" s="3"/>
-      <c r="Z220" s="3"/>
-      <c r="AA220" s="3"/>
-      <c r="AB220" s="3"/>
-      <c r="AC220" s="3"/>
-    </row>
-    <row r="221" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="Z220" s="6"/>
+      <c r="AA220" s="6"/>
+      <c r="AB220" s="6"/>
+      <c r="AC220" s="6"/>
+      <c r="AD220" s="6"/>
+    </row>
+    <row r="221" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C221" t="s">
         <v>10</v>
       </c>
@@ -3791,60 +3794,67 @@
       </c>
       <c r="N221">
         <f>SUM((MAX(N211:N217)-N217)+(MAX(O212:O217)-O217)+(MAX(P213:P217)-P217)+(MAX(Q214:Q217)-Q217)+(MAX(R215:R217)-R217)+(MAX(S216:S217)-S217))/6</f>
+        <v>2.6257869368483306</v>
+      </c>
+      <c r="P221" s="6"/>
+      <c r="Q221" s="6"/>
+      <c r="R221" s="6"/>
+      <c r="S221" s="6"/>
+      <c r="T221" s="6"/>
+      <c r="W221" t="s">
+        <v>10</v>
+      </c>
+      <c r="X221">
+        <f>SUM((MAX(X211:X217)-X217)+(MAX(Y212:Y217)-Y217)+(MAX(Z213:Z217)-Z217)+(MAX(AA214:AA217)-AA217)+(MAX(AB215:AB217)-AB217)+(MAX(AC216:AC217)-AC217))/6</f>
         <v>2.1743014247352783</v>
       </c>
-      <c r="P221" s="3"/>
-      <c r="Q221" s="3"/>
-      <c r="R221" s="3"/>
-      <c r="S221" s="3"/>
-      <c r="T221" s="3"/>
-      <c r="V221" t="s">
-        <v>10</v>
-      </c>
-      <c r="W221">
-        <f>SUM((MAX(W211:W217)-W217)+(MAX(X212:X217)-X217)+(MAX(Y213:Y217)-Y217)+(MAX(Z214:Z217)-Z217)+(MAX(AA215:AA217)-AA217)+(MAX(AB216:AB217)-AB217))/6</f>
-        <v>2.3111177207530695</v>
-      </c>
-      <c r="Y221" s="3"/>
-      <c r="Z221" s="3"/>
-      <c r="AA221" s="3"/>
-      <c r="AB221" s="3"/>
-      <c r="AC221" s="3"/>
-    </row>
-    <row r="222" spans="3:29" x14ac:dyDescent="0.2">
-      <c r="P222" s="3"/>
-      <c r="Q222" s="3"/>
-      <c r="R222" s="3"/>
-      <c r="S222" s="3"/>
-      <c r="T222" s="3"/>
-      <c r="Y222" s="3"/>
-      <c r="Z222" s="3"/>
-      <c r="AA222" s="3"/>
-      <c r="AB222" s="3"/>
-      <c r="AC222" s="3"/>
+      <c r="Z221" s="6"/>
+      <c r="AA221" s="6"/>
+      <c r="AB221" s="6"/>
+      <c r="AC221" s="6"/>
+      <c r="AD221" s="6"/>
+    </row>
+    <row r="222" spans="3:30" x14ac:dyDescent="0.2">
+      <c r="P222" s="6"/>
+      <c r="Q222" s="6"/>
+      <c r="R222" s="6"/>
+      <c r="S222" s="6"/>
+      <c r="T222" s="6"/>
+      <c r="Z222" s="6"/>
+      <c r="AA222" s="6"/>
+      <c r="AB222" s="6"/>
+      <c r="AC222" s="6"/>
+      <c r="AD222" s="6"/>
+    </row>
+    <row r="223" spans="3:30" x14ac:dyDescent="0.2">
+      <c r="P223" s="14"/>
+      <c r="Q223" s="14"/>
+      <c r="R223" s="14"/>
+      <c r="S223" s="14"/>
+      <c r="T223" s="14"/>
     </row>
     <row r="225" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="226" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C226" s="5" t="s">
+      <c r="C226" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D226" s="6"/>
-      <c r="E226" s="6"/>
-      <c r="F226" s="6"/>
-      <c r="G226" s="6"/>
-      <c r="H226" s="6"/>
-      <c r="I226" s="6"/>
-      <c r="J226" s="7"/>
-      <c r="M226" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="N226" s="6"/>
-      <c r="O226" s="6"/>
-      <c r="P226" s="6"/>
-      <c r="Q226" s="6"/>
-      <c r="R226" s="6"/>
-      <c r="S226" s="6"/>
-      <c r="T226" s="7"/>
+      <c r="D226" s="4"/>
+      <c r="E226" s="4"/>
+      <c r="F226" s="4"/>
+      <c r="G226" s="4"/>
+      <c r="H226" s="4"/>
+      <c r="I226" s="4"/>
+      <c r="J226" s="5"/>
+      <c r="M226" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="N226" s="4"/>
+      <c r="O226" s="4"/>
+      <c r="P226" s="4"/>
+      <c r="Q226" s="4"/>
+      <c r="R226" s="4"/>
+      <c r="S226" s="4"/>
+      <c r="T226" s="5"/>
     </row>
     <row r="227" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C227" s="2" t="s">
@@ -4208,40 +4218,40 @@
         <v>2.0908121676384162</v>
       </c>
     </row>
-    <row r="241" spans="3:29" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="3:29" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C242" s="5" t="s">
+    <row r="241" spans="3:30" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="3:30" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C242" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D242" s="6"/>
-      <c r="E242" s="6"/>
-      <c r="F242" s="6"/>
-      <c r="G242" s="6"/>
-      <c r="H242" s="6"/>
-      <c r="I242" s="6"/>
-      <c r="J242" s="7"/>
-      <c r="M242" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="N242" s="6"/>
-      <c r="O242" s="6"/>
-      <c r="P242" s="6"/>
-      <c r="Q242" s="6"/>
-      <c r="R242" s="6"/>
-      <c r="S242" s="6"/>
-      <c r="T242" s="7"/>
-      <c r="V242" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="W242" s="6"/>
-      <c r="X242" s="6"/>
-      <c r="Y242" s="6"/>
-      <c r="Z242" s="6"/>
-      <c r="AA242" s="6"/>
-      <c r="AB242" s="6"/>
-      <c r="AC242" s="7"/>
-    </row>
-    <row r="243" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="D242" s="4"/>
+      <c r="E242" s="4"/>
+      <c r="F242" s="4"/>
+      <c r="G242" s="4"/>
+      <c r="H242" s="4"/>
+      <c r="I242" s="4"/>
+      <c r="J242" s="5"/>
+      <c r="M242" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N242" s="4"/>
+      <c r="O242" s="4"/>
+      <c r="P242" s="4"/>
+      <c r="Q242" s="4"/>
+      <c r="R242" s="4"/>
+      <c r="S242" s="4"/>
+      <c r="T242" s="5"/>
+      <c r="W242" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="X242" s="4"/>
+      <c r="Y242" s="4"/>
+      <c r="Z242" s="4"/>
+      <c r="AA242" s="4"/>
+      <c r="AB242" s="4"/>
+      <c r="AC242" s="4"/>
+      <c r="AD242" s="5"/>
+    </row>
+    <row r="243" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C243" s="2" t="s">
         <v>0</v>
       </c>
@@ -4290,32 +4300,32 @@
       <c r="T243" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="V243" s="2" t="s">
+      <c r="W243" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="W243" s="2" t="s">
+      <c r="X243" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="X243" s="2" t="s">
+      <c r="Y243" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="Y243" s="2" t="s">
+      <c r="Z243" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="Z243" s="2" t="s">
+      <c r="AA243" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="AA243" s="2" t="s">
+      <c r="AB243" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="AB243" s="2" t="s">
+      <c r="AC243" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="AC243" s="2" t="s">
+      <c r="AD243" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="244" spans="3:29" x14ac:dyDescent="0.2">
+    <row r="244" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C244" s="1" t="s">
         <v>1</v>
       </c>
@@ -4340,20 +4350,20 @@
       <c r="R244" s="1"/>
       <c r="S244" s="1"/>
       <c r="T244" s="1"/>
-      <c r="V244" s="1" t="s">
+      <c r="W244" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="W244" s="1">
-        <v>96.814903846153797</v>
-      </c>
-      <c r="X244" s="1"/>
+      <c r="X244" s="1">
+        <v>96.885016025640994</v>
+      </c>
       <c r="Y244" s="1"/>
       <c r="Z244" s="1"/>
       <c r="AA244" s="1"/>
       <c r="AB244" s="1"/>
       <c r="AC244" s="1"/>
-    </row>
-    <row r="245" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD244" s="1"/>
+    </row>
+    <row r="245" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C245" s="1" t="s">
         <v>2</v>
       </c>
@@ -4382,22 +4392,22 @@
       <c r="R245" s="1"/>
       <c r="S245" s="1"/>
       <c r="T245" s="1"/>
-      <c r="V245" s="1" t="s">
+      <c r="W245" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="W245" s="1">
-        <v>96.564503205128204</v>
-      </c>
       <c r="X245" s="1">
-        <v>86.488381410256395</v>
-      </c>
-      <c r="Y245" s="1"/>
+        <v>96.684695512820497</v>
+      </c>
+      <c r="Y245" s="1">
+        <v>87.089342948717899</v>
+      </c>
       <c r="Z245" s="1"/>
       <c r="AA245" s="1"/>
       <c r="AB245" s="1"/>
       <c r="AC245" s="1"/>
-    </row>
-    <row r="246" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD245" s="1"/>
+    </row>
+    <row r="246" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C246" s="1" t="s">
         <v>3</v>
       </c>
@@ -4428,23 +4438,23 @@
       <c r="R246" s="1"/>
       <c r="S246" s="1"/>
       <c r="T246" s="1"/>
-      <c r="V246" s="1" t="s">
+      <c r="W246" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="W246" s="1">
-        <v>96.113782051282001</v>
-      </c>
       <c r="X246" s="1">
-        <v>85.456730769230703</v>
+        <v>95.983573717948701</v>
       </c>
       <c r="Y246" s="1">
-        <v>94.688735177865595</v>
-      </c>
-      <c r="AA246" s="1"/>
+        <v>86.5885416666666</v>
+      </c>
+      <c r="Z246" s="1">
+        <v>97.035573122529598</v>
+      </c>
       <c r="AB246" s="1"/>
       <c r="AC246" s="1"/>
-    </row>
-    <row r="247" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD246" s="1"/>
+    </row>
+    <row r="247" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C247" s="1" t="s">
         <v>4</v>
       </c>
@@ -4481,26 +4491,26 @@
       <c r="R247" s="1"/>
       <c r="S247" s="1"/>
       <c r="T247" s="1"/>
-      <c r="V247" s="1" t="s">
+      <c r="W247" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="W247" s="1">
-        <v>94.971955128205096</v>
-      </c>
-      <c r="X247">
-        <v>83.573717948717899</v>
-      </c>
-      <c r="Y247" s="1">
-        <v>94.849308300395194</v>
+      <c r="X247" s="1">
+        <v>93.970352564102498</v>
+      </c>
+      <c r="Y247">
+        <v>82.822516025640994</v>
       </c>
       <c r="Z247" s="1">
-        <v>78.877005347593496</v>
-      </c>
-      <c r="AA247" s="1"/>
+        <v>95.503952569169897</v>
+      </c>
+      <c r="AA247" s="1">
+        <v>78.659759358288696</v>
+      </c>
       <c r="AB247" s="1"/>
       <c r="AC247" s="1"/>
-    </row>
-    <row r="248" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD247" s="1"/>
+    </row>
+    <row r="248" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C248" s="1" t="s">
         <v>5</v>
       </c>
@@ -4541,28 +4551,28 @@
       </c>
       <c r="S248" s="1"/>
       <c r="T248" s="1"/>
-      <c r="V248" s="1" t="s">
+      <c r="W248" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="W248" s="1">
-        <v>95.252403846153797</v>
-      </c>
       <c r="X248" s="1">
-        <v>83.573717948717899</v>
-      </c>
-      <c r="Y248">
-        <v>92.959486166007906</v>
-      </c>
-      <c r="Z248" s="1">
-        <v>75.451203208556095</v>
+        <v>93.549679487179404</v>
+      </c>
+      <c r="Y248" s="1">
+        <v>83.173076923076906</v>
+      </c>
+      <c r="Z248">
+        <v>94.4169960474308</v>
       </c>
       <c r="AA248" s="1">
-        <v>84.955929487179404</v>
-      </c>
-      <c r="AB248" s="1"/>
+        <v>75.016711229946495</v>
+      </c>
+      <c r="AB248" s="1">
+        <v>85.346554487179404</v>
+      </c>
       <c r="AC248" s="1"/>
-    </row>
-    <row r="249" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="AD248" s="1"/>
+    </row>
+    <row r="249" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C249" s="1" t="s">
         <v>6</v>
       </c>
@@ -4607,30 +4617,30 @@
         <v>92.171556122448905</v>
       </c>
       <c r="T249" s="1"/>
-      <c r="V249" s="1" t="s">
+      <c r="W249" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="W249" s="1">
-        <v>94.100560897435898</v>
-      </c>
       <c r="X249" s="1">
-        <v>82.702323717948701</v>
+        <v>92.267628205128204</v>
       </c>
       <c r="Y249" s="1">
-        <v>90.056818181818102</v>
+        <v>81.891025641025607</v>
       </c>
       <c r="Z249" s="1">
-        <v>74.699197860962499</v>
+        <v>91.934288537549406</v>
       </c>
       <c r="AA249" s="1">
-        <v>84.735576923076906</v>
+        <v>74.247994652406405</v>
       </c>
       <c r="AB249" s="1">
-        <v>92.857142857142804</v>
-      </c>
-      <c r="AC249" s="1"/>
-    </row>
-    <row r="250" spans="3:29" x14ac:dyDescent="0.2">
+        <v>84.545272435897402</v>
+      </c>
+      <c r="AC249" s="1">
+        <v>92.570153061224403</v>
+      </c>
+      <c r="AD249" s="1"/>
+    </row>
+    <row r="250" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C250" s="1" t="s">
         <v>7</v>
       </c>
@@ -4679,32 +4689,32 @@
       <c r="T250" s="1">
         <v>60.9375</v>
       </c>
-      <c r="V250" s="1" t="s">
+      <c r="W250" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="W250" s="1">
-        <v>94.320913461538396</v>
-      </c>
       <c r="X250" s="1">
-        <v>83.092948717948701</v>
+        <v>92.397836538461505</v>
       </c>
       <c r="Y250" s="1">
-        <v>90.180335968379396</v>
+        <v>82.201522435897402</v>
       </c>
       <c r="Z250" s="1">
-        <v>74.949866310160402</v>
+        <v>92.255434782608603</v>
       </c>
       <c r="AA250" s="1">
-        <v>84.5052083333333</v>
+        <v>74.548796791443806</v>
       </c>
       <c r="AB250" s="1">
-        <v>93.144132653061206</v>
+        <v>84.8958333333333</v>
       </c>
       <c r="AC250" s="1">
-        <v>57.8125</v>
-      </c>
-    </row>
-    <row r="252" spans="3:29" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+        <v>92.522321428571402</v>
+      </c>
+      <c r="AD250" s="1">
+        <v>42.7083333333333</v>
+      </c>
+    </row>
+    <row r="252" spans="3:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C252" t="s">
         <v>8</v>
       </c>
@@ -4719,29 +4729,29 @@
         <f>AVERAGE(N250:T250)</f>
         <v>83.400848007784504</v>
       </c>
-      <c r="P252" s="3" t="s">
+      <c r="P252" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="Q252" s="3"/>
-      <c r="R252" s="3"/>
-      <c r="S252" s="3"/>
-      <c r="T252" s="3"/>
-      <c r="V252" t="s">
+      <c r="Q252" s="6"/>
+      <c r="R252" s="6"/>
+      <c r="S252" s="6"/>
+      <c r="T252" s="6"/>
+      <c r="W252" t="s">
         <v>8</v>
       </c>
-      <c r="W252">
-        <f>AVERAGE(W250:AC250)</f>
-        <v>82.572272206345914</v>
-      </c>
-      <c r="Y252" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="Z252" s="3"/>
-      <c r="AA252" s="3"/>
-      <c r="AB252" s="3"/>
-      <c r="AC252" s="3"/>
-    </row>
-    <row r="253" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="X252">
+        <f>AVERAGE(X250:AD250)</f>
+        <v>80.21858266337847</v>
+      </c>
+      <c r="Z252" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA252" s="6"/>
+      <c r="AB252" s="6"/>
+      <c r="AC252" s="6"/>
+      <c r="AD252" s="6"/>
+    </row>
+    <row r="253" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C253" t="s">
         <v>9</v>
       </c>
@@ -4756,25 +4766,25 @@
         <f>(SUM((N250-N244)+(O250-O245)+(P250-P246)+(Q250-Q247)+(R250-R248)+(S250-S249)))/6</f>
         <v>-2.0617011500049522</v>
       </c>
-      <c r="P253" s="3"/>
-      <c r="Q253" s="3"/>
-      <c r="R253" s="3"/>
-      <c r="S253" s="3"/>
-      <c r="T253" s="3"/>
-      <c r="V253" t="s">
+      <c r="P253" s="6"/>
+      <c r="Q253" s="6"/>
+      <c r="R253" s="6"/>
+      <c r="S253" s="6"/>
+      <c r="T253" s="6"/>
+      <c r="W253" t="s">
         <v>9</v>
       </c>
-      <c r="W253">
-        <f>(SUM((W250-W244)+(X250-X245)+(Y250-Y246)+(Z250-Z247)+(AA250-AA248)+(AB250-AB249)))/6</f>
-        <v>-2.4147821136283483</v>
-      </c>
-      <c r="Y253" s="3"/>
-      <c r="Z253" s="3"/>
-      <c r="AA253" s="3"/>
-      <c r="AB253" s="3"/>
-      <c r="AC253" s="3"/>
-    </row>
-    <row r="254" spans="3:29" x14ac:dyDescent="0.2">
+      <c r="X253">
+        <f>(SUM((X250-X244)+(Y250-Y245)+(Z250-Z246)+(AA250-AA247)+(AB250-AB248)+(AC250-AC249)))/6</f>
+        <v>-3.1274422822108292</v>
+      </c>
+      <c r="Z253" s="6"/>
+      <c r="AA253" s="6"/>
+      <c r="AB253" s="6"/>
+      <c r="AC253" s="6"/>
+      <c r="AD253" s="6"/>
+    </row>
+    <row r="254" spans="3:30" x14ac:dyDescent="0.2">
       <c r="C254" t="s">
         <v>10</v>
       </c>
@@ -4789,48 +4799,48 @@
         <f>SUM((MAX(N244:N250)-N250)+(MAX(O245:O250)-O250)+(MAX(P246:P250)-P250)+(MAX(Q247:Q250)-Q250)+(MAX(R248:R250)-R250)+(MAX(S249:S250)-S250))/6</f>
         <v>2.0617011500049522</v>
       </c>
-      <c r="P254" s="3"/>
-      <c r="Q254" s="3"/>
-      <c r="R254" s="3"/>
-      <c r="S254" s="3"/>
-      <c r="T254" s="3"/>
-      <c r="V254" t="s">
+      <c r="P254" s="6"/>
+      <c r="Q254" s="6"/>
+      <c r="R254" s="6"/>
+      <c r="S254" s="6"/>
+      <c r="T254" s="6"/>
+      <c r="W254" t="s">
         <v>10</v>
       </c>
-      <c r="W254">
-        <f>SUM((MAX(W244:W250)-W250)+(MAX(X245:X250)-X250)+(MAX(Y246:Y250)-Y250)+(MAX(Z247:Z250)-Z250)+(MAX(AA248:AA250)-AA250)+(MAX(AB249:AB250)-AB250))/6</f>
-        <v>2.4893759333696814</v>
-      </c>
-      <c r="Y254" s="3"/>
-      <c r="Z254" s="3"/>
-      <c r="AA254" s="3"/>
-      <c r="AB254" s="3"/>
-      <c r="AC254" s="3"/>
-    </row>
-    <row r="255" spans="3:29" x14ac:dyDescent="0.2">
-      <c r="P255" s="3"/>
-      <c r="Q255" s="3"/>
-      <c r="R255" s="3"/>
-      <c r="S255" s="3"/>
-      <c r="T255" s="3"/>
-      <c r="Y255" s="3"/>
-      <c r="Z255" s="3"/>
-      <c r="AA255" s="3"/>
-      <c r="AB255" s="3"/>
-      <c r="AC255" s="3"/>
+      <c r="X254">
+        <f>SUM((MAX(X244:X250)-X250)+(MAX(Y245:Y250)-Y250)+(MAX(Z246:Z250)-Z250)+(MAX(AA247:AA250)-AA250)+(MAX(AB248:AB250)-AB250)+(MAX(AC249:AC250)-AC250))/6</f>
+        <v>3.1274422822108292</v>
+      </c>
+      <c r="Z254" s="6"/>
+      <c r="AA254" s="6"/>
+      <c r="AB254" s="6"/>
+      <c r="AC254" s="6"/>
+      <c r="AD254" s="6"/>
+    </row>
+    <row r="255" spans="3:30" x14ac:dyDescent="0.2">
+      <c r="P255" s="6"/>
+      <c r="Q255" s="6"/>
+      <c r="R255" s="6"/>
+      <c r="S255" s="6"/>
+      <c r="T255" s="6"/>
+      <c r="Z255" s="6"/>
+      <c r="AA255" s="6"/>
+      <c r="AB255" s="6"/>
+      <c r="AC255" s="6"/>
+      <c r="AD255" s="6"/>
     </row>
     <row r="267" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="268" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C268" s="5" t="s">
+      <c r="C268" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D268" s="6"/>
-      <c r="E268" s="6"/>
-      <c r="F268" s="6"/>
-      <c r="G268" s="6"/>
-      <c r="H268" s="6"/>
-      <c r="I268" s="6"/>
-      <c r="J268" s="7"/>
+      <c r="D268" s="4"/>
+      <c r="E268" s="4"/>
+      <c r="F268" s="4"/>
+      <c r="G268" s="4"/>
+      <c r="H268" s="4"/>
+      <c r="I268" s="4"/>
+      <c r="J268" s="5"/>
     </row>
     <row r="269" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C269" s="2" t="s">
@@ -5006,12 +5016,12 @@
         <f>AVERAGE(D276:J276)</f>
         <v>73.9583333333333</v>
       </c>
-      <c r="F278" s="3" t="s">
+      <c r="F278" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G278" s="4"/>
-      <c r="H278" s="4"/>
-      <c r="I278" s="4"/>
+      <c r="G278" s="13"/>
+      <c r="H278" s="13"/>
+      <c r="I278" s="13"/>
     </row>
     <row r="279" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C279" t="s">
@@ -5021,10 +5031,10 @@
         <f>(SUM((D276-D270)+(E276-E271)+(F276-F272)+(G276-G273)+(H276-H274)+(I276-I275)))/6</f>
         <v>-0.17361111111111663</v>
       </c>
-      <c r="F279" s="4"/>
-      <c r="G279" s="4"/>
-      <c r="H279" s="4"/>
-      <c r="I279" s="4"/>
+      <c r="F279" s="13"/>
+      <c r="G279" s="13"/>
+      <c r="H279" s="13"/>
+      <c r="I279" s="13"/>
     </row>
     <row r="280" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C280" t="s">
@@ -5034,23 +5044,23 @@
         <f>SUM((MAX(D270:D276)-D276)+(MAX(E271:E276)-E276)+(MAX(F272:F276)-F276)+(MAX(G273:G276)-G276)+(MAX(H274:H276)-H276)+(MAX(I275:I276)-I276))/6</f>
         <v>1.9097222222222499</v>
       </c>
-      <c r="F280" s="4"/>
-      <c r="G280" s="4"/>
-      <c r="H280" s="4"/>
-      <c r="I280" s="4"/>
+      <c r="F280" s="13"/>
+      <c r="G280" s="13"/>
+      <c r="H280" s="13"/>
+      <c r="I280" s="13"/>
     </row>
     <row r="286" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="287" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C287" s="5" t="s">
+      <c r="C287" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D287" s="6"/>
-      <c r="E287" s="6"/>
-      <c r="F287" s="6"/>
-      <c r="G287" s="6"/>
-      <c r="H287" s="6"/>
-      <c r="I287" s="6"/>
-      <c r="J287" s="7"/>
+      <c r="D287" s="4"/>
+      <c r="E287" s="4"/>
+      <c r="F287" s="4"/>
+      <c r="G287" s="4"/>
+      <c r="H287" s="4"/>
+      <c r="I287" s="4"/>
+      <c r="J287" s="5"/>
     </row>
     <row r="288" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C288" s="2" t="s">
@@ -5226,12 +5236,12 @@
         <f>AVERAGE(D295:J295)</f>
         <v>64.5833333333333</v>
       </c>
-      <c r="F297" s="3" t="s">
+      <c r="F297" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G297" s="4"/>
-      <c r="H297" s="4"/>
-      <c r="I297" s="4"/>
+      <c r="G297" s="13"/>
+      <c r="H297" s="13"/>
+      <c r="I297" s="13"/>
     </row>
     <row r="298" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C298" t="s">
@@ -5241,10 +5251,10 @@
         <f>(SUM((D295-D289)+(E295-E290)+(F295-F291)+(G295-G292)+(H295-H293)+(I295-I294)))/6</f>
         <v>-2.7777777777777835</v>
       </c>
-      <c r="F298" s="4"/>
-      <c r="G298" s="4"/>
-      <c r="H298" s="4"/>
-      <c r="I298" s="4"/>
+      <c r="F298" s="13"/>
+      <c r="G298" s="13"/>
+      <c r="H298" s="13"/>
+      <c r="I298" s="13"/>
     </row>
     <row r="299" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C299" t="s">
@@ -5254,23 +5264,23 @@
         <f>SUM((MAX(D289:D295)-D295)+(MAX(E290:E295)-E295)+(MAX(F291:F295)-F295)+(MAX(G292:G295)-G295)+(MAX(H293:H295)-H295)+(MAX(I294:I295)-I295))/6</f>
         <v>5.208333333333333</v>
       </c>
-      <c r="F299" s="4"/>
-      <c r="G299" s="4"/>
-      <c r="H299" s="4"/>
-      <c r="I299" s="4"/>
+      <c r="F299" s="13"/>
+      <c r="G299" s="13"/>
+      <c r="H299" s="13"/>
+      <c r="I299" s="13"/>
     </row>
     <row r="302" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="303" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C303" s="5" t="s">
+      <c r="C303" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D303" s="6"/>
-      <c r="E303" s="6"/>
-      <c r="F303" s="6"/>
-      <c r="G303" s="6"/>
-      <c r="H303" s="6"/>
-      <c r="I303" s="6"/>
-      <c r="J303" s="7"/>
+      <c r="D303" s="4"/>
+      <c r="E303" s="4"/>
+      <c r="F303" s="4"/>
+      <c r="G303" s="4"/>
+      <c r="H303" s="4"/>
+      <c r="I303" s="4"/>
+      <c r="J303" s="5"/>
     </row>
     <row r="304" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C304" s="2" t="s">
@@ -5446,12 +5456,12 @@
         <f>AVERAGE(D311:J311)</f>
         <v>78.298611111111072</v>
       </c>
-      <c r="F313" s="3" t="s">
+      <c r="F313" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G313" s="4"/>
-      <c r="H313" s="4"/>
-      <c r="I313" s="4"/>
+      <c r="G313" s="13"/>
+      <c r="H313" s="13"/>
+      <c r="I313" s="13"/>
     </row>
     <row r="314" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C314" t="s">
@@ -5461,10 +5471,10 @@
         <f>(SUM((D311-D305)+(E311-E306)+(F311-F307)+(G311-G308)+(H311-H309)+(I311-I310)))/6</f>
         <v>0.34722222222220012</v>
       </c>
-      <c r="F314" s="4"/>
-      <c r="G314" s="4"/>
-      <c r="H314" s="4"/>
-      <c r="I314" s="4"/>
+      <c r="F314" s="13"/>
+      <c r="G314" s="13"/>
+      <c r="H314" s="13"/>
+      <c r="I314" s="13"/>
     </row>
     <row r="315" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C315" t="s">
@@ -5474,23 +5484,23 @@
         <f>SUM((MAX(D305:D311)-D311)+(MAX(E306:E311)-E311)+(MAX(F307:F311)-F311)+(MAX(G308:G311)-G311)+(MAX(H309:H311)-H311)+(MAX(I310:I311)-I311))/6</f>
         <v>2.4305555555555665</v>
       </c>
-      <c r="F315" s="4"/>
-      <c r="G315" s="4"/>
-      <c r="H315" s="4"/>
-      <c r="I315" s="4"/>
+      <c r="F315" s="13"/>
+      <c r="G315" s="13"/>
+      <c r="H315" s="13"/>
+      <c r="I315" s="13"/>
     </row>
     <row r="318" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="319" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C319" s="5" t="s">
+      <c r="C319" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D319" s="6"/>
-      <c r="E319" s="6"/>
-      <c r="F319" s="6"/>
-      <c r="G319" s="6"/>
-      <c r="H319" s="6"/>
-      <c r="I319" s="6"/>
-      <c r="J319" s="7"/>
+      <c r="D319" s="4"/>
+      <c r="E319" s="4"/>
+      <c r="F319" s="4"/>
+      <c r="G319" s="4"/>
+      <c r="H319" s="4"/>
+      <c r="I319" s="4"/>
+      <c r="J319" s="5"/>
     </row>
     <row r="320" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C320" s="2" t="s">
@@ -5666,12 +5676,12 @@
         <f>AVERAGE(D327:J327)</f>
         <v>73.660714285714249</v>
       </c>
-      <c r="F329" s="3" t="s">
+      <c r="F329" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G329" s="4"/>
-      <c r="H329" s="4"/>
-      <c r="I329" s="4"/>
+      <c r="G329" s="13"/>
+      <c r="H329" s="13"/>
+      <c r="I329" s="13"/>
     </row>
     <row r="330" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C330" t="s">
@@ -5681,10 +5691,10 @@
         <f>(SUM((D327-D321)+(E327-E322)+(F327-F323)+(G327-G324)+(H327-H325)+(I327-I326)))/6</f>
         <v>-1.3888888888888999</v>
       </c>
-      <c r="F330" s="4"/>
-      <c r="G330" s="4"/>
-      <c r="H330" s="4"/>
-      <c r="I330" s="4"/>
+      <c r="F330" s="13"/>
+      <c r="G330" s="13"/>
+      <c r="H330" s="13"/>
+      <c r="I330" s="13"/>
     </row>
     <row r="331" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C331" t="s">
@@ -5694,23 +5704,23 @@
         <f>SUM((MAX(D321:D327)-D327)+(MAX(E322:E327)-E327)+(MAX(F323:F327)-F327)+(MAX(G324:G327)-G327)+(MAX(H325:H327)-H327)+(MAX(I326:I327)-I327))/6</f>
         <v>2.6041666666666665</v>
       </c>
-      <c r="F331" s="4"/>
-      <c r="G331" s="4"/>
-      <c r="H331" s="4"/>
-      <c r="I331" s="4"/>
+      <c r="F331" s="13"/>
+      <c r="G331" s="13"/>
+      <c r="H331" s="13"/>
+      <c r="I331" s="13"/>
     </row>
     <row r="333" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="334" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C334" s="5" t="s">
+      <c r="C334" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D334" s="6"/>
-      <c r="E334" s="6"/>
-      <c r="F334" s="6"/>
-      <c r="G334" s="6"/>
-      <c r="H334" s="6"/>
-      <c r="I334" s="6"/>
-      <c r="J334" s="7"/>
+      <c r="D334" s="4"/>
+      <c r="E334" s="4"/>
+      <c r="F334" s="4"/>
+      <c r="G334" s="4"/>
+      <c r="H334" s="4"/>
+      <c r="I334" s="4"/>
+      <c r="J334" s="5"/>
     </row>
     <row r="335" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C335" s="2" t="s">
@@ -5886,12 +5896,12 @@
         <f>AVERAGE(D342:J342)</f>
         <v>71.577380952380935</v>
       </c>
-      <c r="F344" s="3" t="s">
+      <c r="F344" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G344" s="4"/>
-      <c r="H344" s="4"/>
-      <c r="I344" s="4"/>
+      <c r="G344" s="13"/>
+      <c r="H344" s="13"/>
+      <c r="I344" s="13"/>
     </row>
     <row r="345" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C345" t="s">
@@ -5901,10 +5911,10 @@
         <f>(SUM((D342-D336)+(E342-E337)+(F342-F338)+(G342-G339)+(H342-H340)+(I342-I341)))/6</f>
         <v>-1.0416666666666667</v>
       </c>
-      <c r="F345" s="4"/>
-      <c r="G345" s="4"/>
-      <c r="H345" s="4"/>
-      <c r="I345" s="4"/>
+      <c r="F345" s="13"/>
+      <c r="G345" s="13"/>
+      <c r="H345" s="13"/>
+      <c r="I345" s="13"/>
     </row>
     <row r="346" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C346" t="s">
@@ -5914,23 +5924,23 @@
         <f>SUM((MAX(D336:D342)-D342)+(MAX(E337:E342)-E342)+(MAX(F338:F342)-F342)+(MAX(G339:G342)-G342)+(MAX(H340:H342)-H342)+(MAX(I341:I342)-I342))/6</f>
         <v>2.6041666666666665</v>
       </c>
-      <c r="F346" s="4"/>
-      <c r="G346" s="4"/>
-      <c r="H346" s="4"/>
-      <c r="I346" s="4"/>
+      <c r="F346" s="13"/>
+      <c r="G346" s="13"/>
+      <c r="H346" s="13"/>
+      <c r="I346" s="13"/>
     </row>
     <row r="349" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="350" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C350" s="5" t="s">
+      <c r="C350" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D350" s="6"/>
-      <c r="E350" s="6"/>
-      <c r="F350" s="6"/>
-      <c r="G350" s="6"/>
-      <c r="H350" s="6"/>
-      <c r="I350" s="6"/>
-      <c r="J350" s="7"/>
+      <c r="D350" s="4"/>
+      <c r="E350" s="4"/>
+      <c r="F350" s="4"/>
+      <c r="G350" s="4"/>
+      <c r="H350" s="4"/>
+      <c r="I350" s="4"/>
+      <c r="J350" s="5"/>
     </row>
     <row r="351" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C351" s="2" t="s">
@@ -6102,12 +6112,12 @@
         <f>AVERAGE(D358:J358)</f>
         <v>67.261904761904731</v>
       </c>
-      <c r="F360" s="3" t="s">
+      <c r="F360" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G360" s="4"/>
-      <c r="H360" s="4"/>
-      <c r="I360" s="4"/>
+      <c r="G360" s="13"/>
+      <c r="H360" s="13"/>
+      <c r="I360" s="13"/>
     </row>
     <row r="361" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C361" t="s">
@@ -6117,10 +6127,10 @@
         <f>(SUM((D358-D352)+(E358-E353)+(F358-F354)+(G358-G355)+(H358-H356)+(I358-I357)))/6</f>
         <v>-3.4722222222222334</v>
       </c>
-      <c r="F361" s="4"/>
-      <c r="G361" s="4"/>
-      <c r="H361" s="4"/>
-      <c r="I361" s="4"/>
+      <c r="F361" s="13"/>
+      <c r="G361" s="13"/>
+      <c r="H361" s="13"/>
+      <c r="I361" s="13"/>
     </row>
     <row r="362" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C362" t="s">
@@ -6130,36 +6140,14 @@
         <f>SUM((MAX(D352:D358)-D358)+(MAX(E353:E358)-E358)+(MAX(F355:F358)-F358)+(MAX(G355:G358)-G358)+(MAX(H356:H358)-H358)+(MAX(I357:I358)-I358))/6</f>
         <v>5.38194444444445</v>
       </c>
-      <c r="F362" s="4"/>
-      <c r="G362" s="4"/>
-      <c r="H362" s="4"/>
-      <c r="I362" s="4"/>
+      <c r="F362" s="13"/>
+      <c r="G362" s="13"/>
+      <c r="H362" s="13"/>
+      <c r="I362" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="V209:AC209"/>
-    <mergeCell ref="Y219:AC222"/>
-    <mergeCell ref="V242:AC242"/>
-    <mergeCell ref="Y252:AC255"/>
-    <mergeCell ref="C169:J169"/>
-    <mergeCell ref="C86:J86"/>
-    <mergeCell ref="C107:J107"/>
-    <mergeCell ref="C123:J123"/>
-    <mergeCell ref="C139:J139"/>
-    <mergeCell ref="C154:J154"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="C23:J23"/>
-    <mergeCell ref="C39:J39"/>
-    <mergeCell ref="C55:J55"/>
-    <mergeCell ref="C70:J70"/>
-    <mergeCell ref="C203:J204"/>
-    <mergeCell ref="C209:J209"/>
-    <mergeCell ref="C226:J226"/>
-    <mergeCell ref="C242:J242"/>
-    <mergeCell ref="C184:J184"/>
-    <mergeCell ref="M209:T209"/>
-    <mergeCell ref="M226:T226"/>
-    <mergeCell ref="M242:T242"/>
+    <mergeCell ref="Z252:AD255"/>
     <mergeCell ref="C268:J268"/>
     <mergeCell ref="C287:J287"/>
     <mergeCell ref="P219:T222"/>
@@ -6174,6 +6162,28 @@
     <mergeCell ref="F297:I299"/>
     <mergeCell ref="F313:I315"/>
     <mergeCell ref="F329:I331"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="C39:J39"/>
+    <mergeCell ref="C55:J55"/>
+    <mergeCell ref="C70:J70"/>
+    <mergeCell ref="C86:J86"/>
+    <mergeCell ref="C107:J107"/>
+    <mergeCell ref="C123:J123"/>
+    <mergeCell ref="C139:J139"/>
+    <mergeCell ref="C154:J154"/>
+    <mergeCell ref="C169:J169"/>
+    <mergeCell ref="C203:J204"/>
+    <mergeCell ref="C209:J209"/>
+    <mergeCell ref="C226:J226"/>
+    <mergeCell ref="C242:J242"/>
+    <mergeCell ref="C184:J184"/>
+    <mergeCell ref="M209:T209"/>
+    <mergeCell ref="M226:T226"/>
+    <mergeCell ref="M242:T242"/>
+    <mergeCell ref="W209:AD209"/>
+    <mergeCell ref="Z219:AD222"/>
+    <mergeCell ref="W242:AD242"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>